<commit_message>
Shield topology (R207): C1 = CAN screen drain, loom screens never cross
- ECU-COMMS C1 = CAN_SCREEN: one trunk drain wire, a named splice per CAN branch (sp_can_sh_clu/_csb/_rd/_bh)
- FR wheel-speed spur screen ties at A7; the CAN drain to B17 is removed (no A-B shield bridge)
- audit_shields S1-S4; DECISIONS R207 (amends R27-R30), SHIELD-RULES, OPEN-ITEMS (N50 answered, N51, row 146)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-wirelist.xlsx
+++ b/docs/harness/wirelist/A-cabin-wirelist.xlsx
@@ -11158,11 +11158,7 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D86" s="39" t="inlineStr">
-        <is>
-          <t>B-cabin</t>
-        </is>
-      </c>
+      <c r="D86" s="39" t="inlineStr"/>
       <c r="E86" s="40" t="inlineStr">
         <is>
           <t>cable screen</t>
@@ -11192,12 +11188,12 @@
       </c>
       <c r="L86" s="44" t="inlineStr">
         <is>
-          <t>sp_shield_b</t>
+          <t>sp_shield_a</t>
         </is>
       </c>
       <c r="M86" s="45" t="inlineStr">
         <is>
-          <t>splice sp_shield_b on B-cabin</t>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
       <c r="N86" s="44" t="inlineStr"/>
@@ -11206,22 +11202,22 @@
           <t>FR wheel spd shield</t>
         </is>
       </c>
-      <c r="P86" s="45" t="inlineStr">
-        <is>
-          <t>at the ECU-B plug (B-cabin); to ECU-B B17</t>
-        </is>
-      </c>
+      <c r="P86" s="45" t="inlineStr"/>
       <c r="Q86" s="46" t="inlineStr">
         <is>
-          <t>ECU-B.B17</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R86" s="47" t="inlineStr">
         <is>
-          <t>Screen B (ECU B17, SHIELD_B)</t>
-        </is>
-      </c>
-      <c r="S86" s="48" t="inlineStr"/>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="S86" s="48" t="inlineStr">
+        <is>
+          <t>sp_shield_a</t>
+        </is>
+      </c>
       <c r="T86" s="48" t="inlineStr">
         <is>
           <t>cab_fspur_fr_ac</t>
@@ -11251,7 +11247,7 @@
       <c r="AD86" s="54" t="inlineStr"/>
       <c r="AE86" s="54" t="inlineStr">
         <is>
-          <t>splice sp_shield_b: node of the wire list (SoT)</t>
+          <t>splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF86" s="54" t="inlineStr">
@@ -11261,7 +11257,7 @@
       </c>
       <c r="AG86" s="54" t="inlineStr">
         <is>
-          <t>screen floats at the far end; owner TBD: a half has no length estimate (drawn today as cab_fspur_fr_sh_ac on A-cabin, ? mm; cab_fspur_fr_sh on B-cabin, ? mm)</t>
+          <t>tied at the A end only; the far (B) end floats, dressed back at the ECU-B plug (no A-B shield bridge)</t>
         </is>
       </c>
     </row>
@@ -12418,7 +12414,7 @@
         </is>
       </c>
       <c r="F5" s="32" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G5" s="32" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Shield topology (R207): C1 = CAN screen drain, loom screens never cross (#346)
- ECU-COMMS C1 = CAN_SCREEN: one trunk drain wire, a named splice per CAN branch (sp_can_sh_clu/_csb/_rd/_bh)
- FR wheel-speed spur screen ties at A7; the CAN drain to B17 is removed (no A-B shield bridge)
- audit_shields S1-S4; DECISIONS R207 (amends R27-R30), SHIELD-RULES, OPEN-ITEMS (N50 answered, N51, row 146)

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-wirelist.xlsx
+++ b/docs/harness/wirelist/A-cabin-wirelist.xlsx
@@ -11158,11 +11158,7 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D86" s="39" t="inlineStr">
-        <is>
-          <t>B-cabin</t>
-        </is>
-      </c>
+      <c r="D86" s="39" t="inlineStr"/>
       <c r="E86" s="40" t="inlineStr">
         <is>
           <t>cable screen</t>
@@ -11192,12 +11188,12 @@
       </c>
       <c r="L86" s="44" t="inlineStr">
         <is>
-          <t>sp_shield_b</t>
+          <t>sp_shield_a</t>
         </is>
       </c>
       <c r="M86" s="45" t="inlineStr">
         <is>
-          <t>splice sp_shield_b on B-cabin</t>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
       <c r="N86" s="44" t="inlineStr"/>
@@ -11206,22 +11202,22 @@
           <t>FR wheel spd shield</t>
         </is>
       </c>
-      <c r="P86" s="45" t="inlineStr">
-        <is>
-          <t>at the ECU-B plug (B-cabin); to ECU-B B17</t>
-        </is>
-      </c>
+      <c r="P86" s="45" t="inlineStr"/>
       <c r="Q86" s="46" t="inlineStr">
         <is>
-          <t>ECU-B.B17</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R86" s="47" t="inlineStr">
         <is>
-          <t>Screen B (ECU B17, SHIELD_B)</t>
-        </is>
-      </c>
-      <c r="S86" s="48" t="inlineStr"/>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="S86" s="48" t="inlineStr">
+        <is>
+          <t>sp_shield_a</t>
+        </is>
+      </c>
       <c r="T86" s="48" t="inlineStr">
         <is>
           <t>cab_fspur_fr_ac</t>
@@ -11251,7 +11247,7 @@
       <c r="AD86" s="54" t="inlineStr"/>
       <c r="AE86" s="54" t="inlineStr">
         <is>
-          <t>splice sp_shield_b: node of the wire list (SoT)</t>
+          <t>splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF86" s="54" t="inlineStr">
@@ -11261,7 +11257,7 @@
       </c>
       <c r="AG86" s="54" t="inlineStr">
         <is>
-          <t>screen floats at the far end; owner TBD: a half has no length estimate (drawn today as cab_fspur_fr_sh_ac on A-cabin, ? mm; cab_fspur_fr_sh on B-cabin, ? mm)</t>
+          <t>tied at the A end only; the far (B) end floats, dressed back at the ECU-B plug (no A-B shield bridge)</t>
         </is>
       </c>
     </row>
@@ -12418,7 +12414,7 @@
         </is>
       </c>
       <c r="F5" s="32" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G5" s="32" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Shield branch-point rule (R207 addendum): pedal and wheel-speed drains join at their own branch splice
sp_shield_a_aps, sp_shield_a_wsf, sp_shield_b_wsr; bulkhead devices keep own pins straight to the ECU splice; audit_shields S5.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-wirelist.xlsx
+++ b/docs/harness/wirelist/A-cabin-wirelist.xlsx
@@ -13,9 +13,9 @@
     <sheet name="Mates" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wire list'!$A$2:$AG$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wire list'!$A$2:$AG$100</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Wire list'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Splices'!$A$2:$L$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Splices'!$A$2:$L$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Splices'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Connectors'!$A$2:$G$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Connectors'!$1:$2</definedName>
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AG98"/>
+  <dimension ref="A1:AG100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -759,14 +759,14 @@
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="36" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="36" customWidth="1" min="16" max="16"/>
     <col width="45" customWidth="1" min="17" max="17"/>
     <col width="32" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
     <col width="18" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="9" customWidth="1" min="22" max="22"/>
@@ -8014,12 +8014,12 @@
     <row r="61">
       <c r="A61" s="23" t="inlineStr">
         <is>
-          <t>CRANKC</t>
+          <t>SHLD</t>
         </is>
       </c>
       <c r="B61" s="23" t="inlineStr">
         <is>
-          <t>w_shc_crank</t>
+          <t>w_shd_a_aps</t>
         </is>
       </c>
       <c r="C61" s="23" t="inlineStr">
@@ -8030,25 +8030,23 @@
       <c r="D61" s="23" t="inlineStr"/>
       <c r="E61" s="24" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="F61" s="25" t="inlineStr">
         <is>
-          <t>bh_a_fw</t>
+          <t>sp_shield_a_aps</t>
         </is>
       </c>
       <c r="G61" s="26" t="inlineStr">
         <is>
-          <t>BULKHEAD</t>
-        </is>
-      </c>
-      <c r="H61" s="25" t="n">
-        <v>11</v>
-      </c>
+          <t>splice sp_shield_a_aps (SP-SHIELD-A-APS)</t>
+        </is>
+      </c>
+      <c r="H61" s="25" t="inlineStr"/>
       <c r="I61" s="26" t="inlineStr">
         <is>
-          <t>Crank sensor shield</t>
+          <t>Shield drain</t>
         </is>
       </c>
       <c r="J61" s="26" t="inlineStr"/>
@@ -8064,13 +8062,13 @@
       </c>
       <c r="M61" s="29" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>splice sp_shield_a (SP-SHIELD-A)</t>
         </is>
       </c>
       <c r="N61" s="28" t="inlineStr"/>
       <c r="O61" s="29" t="inlineStr">
         <is>
-          <t>Crank sensor shield</t>
+          <t>Shield drain</t>
         </is>
       </c>
       <c r="P61" s="29" t="inlineStr"/>
@@ -8105,22 +8103,18 @@
       </c>
       <c r="X61" s="34" t="inlineStr">
         <is>
-          <t>White-Blue-White</t>
+          <t>White-Yellow-Blue</t>
         </is>
       </c>
       <c r="Y61" s="34" t="inlineStr"/>
-      <c r="Z61" s="35" t="inlineStr">
-        <is>
-          <t>trunk ECU-A to bulkhead (RH firewall)</t>
-        </is>
-      </c>
+      <c r="Z61" s="35" t="inlineStr"/>
       <c r="AA61" s="36" t="inlineStr"/>
       <c r="AB61" s="37" t="inlineStr"/>
       <c r="AC61" s="38" t="inlineStr"/>
       <c r="AD61" s="38" t="inlineStr"/>
       <c r="AE61" s="38" t="inlineStr">
         <is>
-          <t>DRB102 11 = section A c33 'Crank VR screen'; splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>splice sp_shield_a_aps: node of the wire list (SoT); splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF61" s="38" t="inlineStr">
@@ -8130,19 +8124,19 @@
       </c>
       <c r="AG61" s="38" t="inlineStr">
         <is>
-          <t>build (R30): this drain is the one crimped into A7</t>
+          <t>branch-point join (R207): the device drain meets the loom shield trunk where its signal wires join the main loom, then runs to the ECU splice</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="39" t="inlineStr">
         <is>
-          <t>CAM</t>
+          <t>SHLD</t>
         </is>
       </c>
       <c r="B62" s="39" t="inlineStr">
         <is>
-          <t>w_shc_cam</t>
+          <t>w_shd_a_wsf</t>
         </is>
       </c>
       <c r="C62" s="39" t="inlineStr">
@@ -8153,25 +8147,23 @@
       <c r="D62" s="39" t="inlineStr"/>
       <c r="E62" s="40" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="F62" s="41" t="inlineStr">
         <is>
-          <t>bh_a_fw</t>
+          <t>sp_shield_a_wsf</t>
         </is>
       </c>
       <c r="G62" s="42" t="inlineStr">
         <is>
-          <t>BULKHEAD</t>
-        </is>
-      </c>
-      <c r="H62" s="41" t="n">
-        <v>15</v>
-      </c>
+          <t>splice sp_shield_a_wsf (SP-SHIELD-A-WSF)</t>
+        </is>
+      </c>
+      <c r="H62" s="41" t="inlineStr"/>
       <c r="I62" s="42" t="inlineStr">
         <is>
-          <t>Cam sensor shield</t>
+          <t>Shield drain</t>
         </is>
       </c>
       <c r="J62" s="42" t="inlineStr"/>
@@ -8187,13 +8179,13 @@
       </c>
       <c r="M62" s="45" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>splice sp_shield_a (SP-SHIELD-A)</t>
         </is>
       </c>
       <c r="N62" s="44" t="inlineStr"/>
       <c r="O62" s="45" t="inlineStr">
         <is>
-          <t>Cam sensor shield</t>
+          <t>Shield drain</t>
         </is>
       </c>
       <c r="P62" s="45" t="inlineStr"/>
@@ -8228,22 +8220,18 @@
       </c>
       <c r="X62" s="50" t="inlineStr">
         <is>
-          <t>Yellow-Yellow</t>
+          <t>White-Yellow-Blue</t>
         </is>
       </c>
       <c r="Y62" s="50" t="inlineStr"/>
-      <c r="Z62" s="51" t="inlineStr">
-        <is>
-          <t>trunk ECU-A to bulkhead (RH firewall)</t>
-        </is>
-      </c>
+      <c r="Z62" s="51" t="inlineStr"/>
       <c r="AA62" s="52" t="inlineStr"/>
       <c r="AB62" s="53" t="inlineStr"/>
       <c r="AC62" s="54" t="inlineStr"/>
       <c r="AD62" s="54" t="inlineStr"/>
       <c r="AE62" s="54" t="inlineStr">
         <is>
-          <t>DRB102 15 = section A c34 'Cam Hall screen'; splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>splice sp_shield_a_wsf: node of the wire list (SoT); splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF62" s="54" t="inlineStr">
@@ -8251,17 +8239,21 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG62" s="54" t="inlineStr"/>
+      <c r="AG62" s="54" t="inlineStr">
+        <is>
+          <t>branch-point join (R207): the device drain meets the loom shield trunk where its signal wires join the main loom, then runs to the ECU splice</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="23" t="inlineStr">
         <is>
-          <t>TURBO</t>
+          <t>CRANKC</t>
         </is>
       </c>
       <c r="B63" s="23" t="inlineStr">
         <is>
-          <t>w_shc_turbo</t>
+          <t>w_shc_crank</t>
         </is>
       </c>
       <c r="C63" s="23" t="inlineStr">
@@ -8286,11 +8278,11 @@
         </is>
       </c>
       <c r="H63" s="25" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="I63" s="26" t="inlineStr">
         <is>
-          <t>Turbo speed shield</t>
+          <t>Crank sensor shield</t>
         </is>
       </c>
       <c r="J63" s="26" t="inlineStr"/>
@@ -8312,7 +8304,7 @@
       <c r="N63" s="28" t="inlineStr"/>
       <c r="O63" s="29" t="inlineStr">
         <is>
-          <t>Turbo speed shield</t>
+          <t>Crank sensor shield</t>
         </is>
       </c>
       <c r="P63" s="29" t="inlineStr"/>
@@ -8347,7 +8339,7 @@
       </c>
       <c r="X63" s="34" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>White-Blue-White</t>
         </is>
       </c>
       <c r="Y63" s="34" t="inlineStr"/>
@@ -8362,7 +8354,7 @@
       <c r="AD63" s="38" t="inlineStr"/>
       <c r="AE63" s="38" t="inlineStr">
         <is>
-          <t>DRB102 19 = section A c6 'Turbo speed screen (to A7)'; splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>DRB102 11 = section A c33 'Crank VR screen'; splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF63" s="38" t="inlineStr">
@@ -8370,17 +8362,21 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG63" s="38" t="inlineStr"/>
+      <c r="AG63" s="38" t="inlineStr">
+        <is>
+          <t>build (R30): this drain is the one crimped into A7</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="39" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>CAM</t>
         </is>
       </c>
       <c r="B64" s="39" t="inlineStr">
         <is>
-          <t>w_shc_flex</t>
+          <t>w_shc_cam</t>
         </is>
       </c>
       <c r="C64" s="39" t="inlineStr">
@@ -8405,11 +8401,11 @@
         </is>
       </c>
       <c r="H64" s="41" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="I64" s="42" t="inlineStr">
         <is>
-          <t>Flex fuel shield</t>
+          <t>Cam sensor shield</t>
         </is>
       </c>
       <c r="J64" s="42" t="inlineStr"/>
@@ -8431,7 +8427,7 @@
       <c r="N64" s="44" t="inlineStr"/>
       <c r="O64" s="45" t="inlineStr">
         <is>
-          <t>Flex fuel shield</t>
+          <t>Cam sensor shield</t>
         </is>
       </c>
       <c r="P64" s="45" t="inlineStr"/>
@@ -8466,7 +8462,7 @@
       </c>
       <c r="X64" s="50" t="inlineStr">
         <is>
-          <t>White-Blue</t>
+          <t>Yellow-Yellow</t>
         </is>
       </c>
       <c r="Y64" s="50" t="inlineStr"/>
@@ -8481,7 +8477,7 @@
       <c r="AD64" s="54" t="inlineStr"/>
       <c r="AE64" s="54" t="inlineStr">
         <is>
-          <t>DRB102 22 = section A c10 'Flex fuel screen (to A7)'; splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>DRB102 15 = section A c34 'Cam Hall screen'; splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF64" s="54" t="inlineStr">
@@ -8494,12 +8490,12 @@
     <row r="65">
       <c r="A65" s="23" t="inlineStr">
         <is>
-          <t>ETBS</t>
+          <t>TURBO</t>
         </is>
       </c>
       <c r="B65" s="23" t="inlineStr">
         <is>
-          <t>w_shc_etbs</t>
+          <t>w_shc_turbo</t>
         </is>
       </c>
       <c r="C65" s="23" t="inlineStr">
@@ -8524,11 +8520,11 @@
         </is>
       </c>
       <c r="H65" s="25" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="I65" s="26" t="inlineStr">
         <is>
-          <t>Throttle shield</t>
+          <t>Turbo speed shield</t>
         </is>
       </c>
       <c r="J65" s="26" t="inlineStr"/>
@@ -8550,7 +8546,7 @@
       <c r="N65" s="28" t="inlineStr"/>
       <c r="O65" s="29" t="inlineStr">
         <is>
-          <t>Throttle shield</t>
+          <t>Turbo speed shield</t>
         </is>
       </c>
       <c r="P65" s="29" t="inlineStr"/>
@@ -8585,7 +8581,7 @@
       </c>
       <c r="X65" s="34" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>White</t>
         </is>
       </c>
       <c r="Y65" s="34" t="inlineStr"/>
@@ -8600,7 +8596,7 @@
       <c r="AD65" s="38" t="inlineStr"/>
       <c r="AE65" s="38" t="inlineStr">
         <is>
-          <t>DRB102 27 = section A c11 'ETB sensor group screen (to A7)'; splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>DRB102 19 = section A c6 'Turbo speed screen (to A7)'; splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF65" s="38" t="inlineStr">
@@ -8613,12 +8609,12 @@
     <row r="66">
       <c r="A66" s="39" t="inlineStr">
         <is>
-          <t>FP</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B66" s="39" t="inlineStr">
         <is>
-          <t>w_fp85</t>
+          <t>w_shc_flex</t>
         </is>
       </c>
       <c r="C66" s="39" t="inlineStr">
@@ -8626,11 +8622,7 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D66" s="39" t="inlineStr">
-        <is>
-          <t>HeavyDC</t>
-        </is>
-      </c>
+      <c r="D66" s="39" t="inlineStr"/>
       <c r="E66" s="40" t="inlineStr">
         <is>
           <t>connector</t>
@@ -8638,85 +8630,83 @@
       </c>
       <c r="F66" s="41" t="inlineStr">
         <is>
-          <t>k_fp</t>
+          <t>bh_a_fw</t>
         </is>
       </c>
       <c r="G66" s="42" t="inlineStr">
         <is>
-          <t>FP RELAY K1</t>
+          <t>BULKHEAD</t>
         </is>
       </c>
       <c r="H66" s="41" t="n">
-        <v>85</v>
+        <v>22</v>
       </c>
       <c r="I66" s="42" t="inlineStr">
         <is>
-          <t>Fuel pump relay (-)</t>
-        </is>
-      </c>
-      <c r="J66" s="42" t="inlineStr">
-        <is>
-          <t>Battery relay block (trunk) relay K1 fuel pump, pin 85</t>
-        </is>
-      </c>
+          <t>Flex fuel shield</t>
+        </is>
+      </c>
+      <c r="J66" s="42" t="inlineStr"/>
       <c r="K66" s="43" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="L66" s="44" t="inlineStr">
         <is>
-          <t>ecu_a</t>
+          <t>sp_shield_a</t>
         </is>
       </c>
       <c r="M66" s="45" t="inlineStr">
         <is>
-          <t>ECU-A</t>
-        </is>
-      </c>
-      <c r="N66" s="44" t="inlineStr">
-        <is>
-          <t>A19</t>
-        </is>
-      </c>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+        </is>
+      </c>
+      <c r="N66" s="44" t="inlineStr"/>
       <c r="O66" s="45" t="inlineStr">
         <is>
-          <t>Fuel pump relay (-)</t>
+          <t>Flex fuel shield</t>
         </is>
       </c>
       <c r="P66" s="45" t="inlineStr"/>
       <c r="Q66" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A19</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R66" s="47" t="inlineStr">
         <is>
-          <t>Fuel pump relay (-) (ECU-A A19)</t>
-        </is>
-      </c>
-      <c r="S66" s="48" t="inlineStr"/>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="S66" s="48" t="inlineStr">
+        <is>
+          <t>sp_shield_a</t>
+        </is>
+      </c>
       <c r="T66" s="48" t="inlineStr"/>
       <c r="U66" s="49" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="V66" s="50" t="inlineStr">
         <is>
-          <t>White</t>
-        </is>
-      </c>
-      <c r="W66" s="50" t="inlineStr"/>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="W66" s="50" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
       <c r="X66" s="50" t="inlineStr">
         <is>
-          <t>White-White-Blue</t>
-        </is>
-      </c>
-      <c r="Y66" s="50" t="n">
-        <v>390</v>
-      </c>
+          <t>White-Blue</t>
+        </is>
+      </c>
+      <c r="Y66" s="50" t="inlineStr"/>
       <c r="Z66" s="51" t="inlineStr">
         <is>
-          <t>glove-box branch (POWER / LOGIC boxes)</t>
+          <t>trunk ECU-A to bulkhead (RH firewall)</t>
         </is>
       </c>
       <c r="AA66" s="52" t="inlineStr"/>
@@ -8725,7 +8715,7 @@
       <c r="AD66" s="54" t="inlineStr"/>
       <c r="AE66" s="54" t="inlineStr">
         <is>
-          <t>fuse-box plan k_fp 85 (18 AWG); channels.csv ecu_a A19 Aux 3 (AUX3_FP_RLY)</t>
+          <t>DRB102 22 = section A c10 'Flex fuel screen (to A7)'; splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF66" s="54" t="inlineStr">
@@ -8733,21 +8723,17 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG66" s="54" t="inlineStr">
-        <is>
-          <t>owner proposed: longer half (drawn today as w_fp85 on A-cabin, 390 mm; w_fp85_h on HeavyDC, 150 mm)</t>
-        </is>
-      </c>
+      <c r="AG66" s="54" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="23" t="inlineStr">
         <is>
-          <t>STR</t>
+          <t>ETBS</t>
         </is>
       </c>
       <c r="B67" s="23" t="inlineStr">
         <is>
-          <t>w_str85</t>
+          <t>w_shc_etbs</t>
         </is>
       </c>
       <c r="C67" s="23" t="inlineStr">
@@ -8755,11 +8741,7 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D67" s="23" t="inlineStr">
-        <is>
-          <t>CabinPower</t>
-        </is>
-      </c>
+      <c r="D67" s="23" t="inlineStr"/>
       <c r="E67" s="24" t="inlineStr">
         <is>
           <t>connector</t>
@@ -8767,85 +8749,83 @@
       </c>
       <c r="F67" s="25" t="inlineStr">
         <is>
-          <t>k_str</t>
+          <t>bh_a_fw</t>
         </is>
       </c>
       <c r="G67" s="26" t="inlineStr">
         <is>
-          <t>POWER R3</t>
+          <t>BULKHEAD</t>
         </is>
       </c>
       <c r="H67" s="25" t="n">
-        <v>85</v>
+        <v>27</v>
       </c>
       <c r="I67" s="26" t="inlineStr">
         <is>
-          <t>Start relay coil (-)</t>
-        </is>
-      </c>
-      <c r="J67" s="26" t="inlineStr">
-        <is>
-          <t>POWER box (glove box) relay R3 start, pin 85</t>
-        </is>
-      </c>
+          <t>Throttle shield</t>
+        </is>
+      </c>
+      <c r="J67" s="26" t="inlineStr"/>
       <c r="K67" s="27" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="L67" s="28" t="inlineStr">
         <is>
-          <t>ecu_a</t>
+          <t>sp_shield_a</t>
         </is>
       </c>
       <c r="M67" s="29" t="inlineStr">
         <is>
-          <t>ECU-A</t>
-        </is>
-      </c>
-      <c r="N67" s="28" t="inlineStr">
-        <is>
-          <t>A26</t>
-        </is>
-      </c>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+        </is>
+      </c>
+      <c r="N67" s="28" t="inlineStr"/>
       <c r="O67" s="29" t="inlineStr">
         <is>
-          <t>Start relay coil (-)</t>
+          <t>Throttle shield</t>
         </is>
       </c>
       <c r="P67" s="29" t="inlineStr"/>
       <c r="Q67" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A26</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R67" s="31" t="inlineStr">
         <is>
-          <t>Start relay coil (-) (ECU-A A26)</t>
-        </is>
-      </c>
-      <c r="S67" s="32" t="inlineStr"/>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="S67" s="32" t="inlineStr">
+        <is>
+          <t>sp_shield_a</t>
+        </is>
+      </c>
       <c r="T67" s="32" t="inlineStr"/>
       <c r="U67" s="33" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="V67" s="34" t="inlineStr">
         <is>
-          <t>White</t>
-        </is>
-      </c>
-      <c r="W67" s="34" t="inlineStr"/>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="W67" s="34" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
       <c r="X67" s="34" t="inlineStr">
         <is>
-          <t>White-Yellow</t>
-        </is>
-      </c>
-      <c r="Y67" s="34" t="n">
-        <v>400</v>
-      </c>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="Y67" s="34" t="inlineStr"/>
       <c r="Z67" s="35" t="inlineStr">
         <is>
-          <t>glove-box branch (POWER / LOGIC boxes)</t>
+          <t>trunk ECU-A to bulkhead (RH firewall)</t>
         </is>
       </c>
       <c r="AA67" s="36" t="inlineStr"/>
@@ -8854,7 +8834,7 @@
       <c r="AD67" s="38" t="inlineStr"/>
       <c r="AE67" s="38" t="inlineStr">
         <is>
-          <t>fuse-box plan k_str 85 (18 AWG); channels.csv ecu_a A26 Aux 8 (AUX8_START_RLY)</t>
+          <t>DRB102 27 = section A c11 'ETB sensor group screen (to A7)'; splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF67" s="38" t="inlineStr">
@@ -8862,21 +8842,17 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG67" s="38" t="inlineStr">
-        <is>
-          <t>owner proposed: longer half (drawn today as w_str85 on A-cabin, 400 mm; w_str85_cp on CabinPower, 400 mm)</t>
-        </is>
-      </c>
+      <c r="AG67" s="38" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="39" t="inlineStr">
         <is>
-          <t>FAN</t>
+          <t>FP</t>
         </is>
       </c>
       <c r="B68" s="39" t="inlineStr">
         <is>
-          <t>w_fan85</t>
+          <t>w_fp85</t>
         </is>
       </c>
       <c r="C68" s="39" t="inlineStr">
@@ -8886,7 +8862,7 @@
       </c>
       <c r="D68" s="39" t="inlineStr">
         <is>
-          <t>CabinPower</t>
+          <t>HeavyDC</t>
         </is>
       </c>
       <c r="E68" s="40" t="inlineStr">
@@ -8896,12 +8872,12 @@
       </c>
       <c r="F68" s="41" t="inlineStr">
         <is>
-          <t>k_fan</t>
+          <t>k_fp</t>
         </is>
       </c>
       <c r="G68" s="42" t="inlineStr">
         <is>
-          <t>POWER R4</t>
+          <t>FP RELAY K1</t>
         </is>
       </c>
       <c r="H68" s="41" t="n">
@@ -8909,12 +8885,12 @@
       </c>
       <c r="I68" s="42" t="inlineStr">
         <is>
-          <t>Rad fan relay (-)</t>
+          <t>Fuel pump relay (-)</t>
         </is>
       </c>
       <c r="J68" s="42" t="inlineStr">
         <is>
-          <t>POWER box (glove box) relay R4 radiator fan, pin 85</t>
+          <t>Battery relay block (trunk) relay K1 fuel pump, pin 85</t>
         </is>
       </c>
       <c r="K68" s="43" t="inlineStr">
@@ -8934,23 +8910,23 @@
       </c>
       <c r="N68" s="44" t="inlineStr">
         <is>
-          <t>A29</t>
+          <t>A19</t>
         </is>
       </c>
       <c r="O68" s="45" t="inlineStr">
         <is>
-          <t>Rad fan relay (-)</t>
+          <t>Fuel pump relay (-)</t>
         </is>
       </c>
       <c r="P68" s="45" t="inlineStr"/>
       <c r="Q68" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A29</t>
+          <t>ECU-A.A19</t>
         </is>
       </c>
       <c r="R68" s="47" t="inlineStr">
         <is>
-          <t>Rad fan relay (-) (ECU-A A29)</t>
+          <t>Fuel pump relay (-) (ECU-A A19)</t>
         </is>
       </c>
       <c r="S68" s="48" t="inlineStr"/>
@@ -8966,11 +8942,11 @@
       <c r="W68" s="50" t="inlineStr"/>
       <c r="X68" s="50" t="inlineStr">
         <is>
-          <t>Yellow-White</t>
+          <t>White-White-Blue</t>
         </is>
       </c>
       <c r="Y68" s="50" t="n">
-        <v>410</v>
+        <v>390</v>
       </c>
       <c r="Z68" s="51" t="inlineStr">
         <is>
@@ -8983,7 +8959,7 @@
       <c r="AD68" s="54" t="inlineStr"/>
       <c r="AE68" s="54" t="inlineStr">
         <is>
-          <t>fuse-box plan k_fan 85 (18 AWG); channels.csv ecu_a A29 Aux 5 (AUX5_RAD_FAN)</t>
+          <t>fuse-box plan k_fp 85 (18 AWG); channels.csv ecu_a A19 Aux 3 (AUX3_FP_RLY)</t>
         </is>
       </c>
       <c r="AF68" s="54" t="inlineStr">
@@ -8993,19 +8969,19 @@
       </c>
       <c r="AG68" s="54" t="inlineStr">
         <is>
-          <t>owner proposed: longer half (drawn today as w_fan85 on A-cabin, 410 mm; w_fan85_cp on CabinPower, 400 mm)</t>
+          <t>owner proposed: longer half (drawn today as w_fp85 on A-cabin, 390 mm; w_fp85_h on HeavyDC, 150 mm)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="23" t="inlineStr">
         <is>
-          <t>EPS</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="B69" s="23" t="inlineStr">
         <is>
-          <t>w_eps_rly</t>
+          <t>w_str85</t>
         </is>
       </c>
       <c r="C69" s="23" t="inlineStr">
@@ -9025,12 +9001,12 @@
       </c>
       <c r="F69" s="25" t="inlineStr">
         <is>
-          <t>k_eps</t>
+          <t>k_str</t>
         </is>
       </c>
       <c r="G69" s="26" t="inlineStr">
         <is>
-          <t>EHPS RELAY</t>
+          <t>POWER R3</t>
         </is>
       </c>
       <c r="H69" s="25" t="n">
@@ -9038,12 +9014,12 @@
       </c>
       <c r="I69" s="26" t="inlineStr">
         <is>
-          <t>EHPS relay coil (-)</t>
+          <t>Start relay coil (-)</t>
         </is>
       </c>
       <c r="J69" s="26" t="inlineStr">
         <is>
-          <t>EHPS pump relay (glove box), pin 85</t>
+          <t>POWER box (glove box) relay R3 start, pin 85</t>
         </is>
       </c>
       <c r="K69" s="27" t="inlineStr">
@@ -9053,31 +9029,33 @@
       </c>
       <c r="L69" s="28" t="inlineStr">
         <is>
-          <t>bh_a_fw</t>
+          <t>ecu_a</t>
         </is>
       </c>
       <c r="M69" s="29" t="inlineStr">
         <is>
-          <t>BULKHEAD</t>
-        </is>
-      </c>
-      <c r="N69" s="28" t="n">
-        <v>56</v>
+          <t>ECU-A</t>
+        </is>
+      </c>
+      <c r="N69" s="28" t="inlineStr">
+        <is>
+          <t>A26</t>
+        </is>
       </c>
       <c r="O69" s="29" t="inlineStr">
         <is>
-          <t>EHPS relay coil (-)</t>
+          <t>Start relay coil (-)</t>
         </is>
       </c>
       <c r="P69" s="29" t="inlineStr"/>
       <c r="Q69" s="30" t="inlineStr">
         <is>
-          <t>DRB102.56</t>
+          <t>ECU-A.A26</t>
         </is>
       </c>
       <c r="R69" s="31" t="inlineStr">
         <is>
-          <t>EHPS relay coil (-) (DRB102 56)</t>
+          <t>Start relay coil (-) (ECU-A A26)</t>
         </is>
       </c>
       <c r="S69" s="32" t="inlineStr"/>
@@ -9087,21 +9065,21 @@
       </c>
       <c r="V69" s="34" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W69" s="34" t="inlineStr"/>
       <c r="X69" s="34" t="inlineStr">
         <is>
-          <t>Blue-Blue-Blue</t>
+          <t>White-Yellow</t>
         </is>
       </c>
       <c r="Y69" s="34" t="n">
-        <v>530</v>
+        <v>400</v>
       </c>
       <c r="Z69" s="35" t="inlineStr">
         <is>
-          <t>glove-box branch (POWER / LOGIC boxes) / trunk ECU-A to bulkhead (RH firewall)</t>
+          <t>glove-box branch (POWER / LOGIC boxes)</t>
         </is>
       </c>
       <c r="AA69" s="36" t="inlineStr"/>
@@ -9110,7 +9088,7 @@
       <c r="AD69" s="38" t="inlineStr"/>
       <c r="AE69" s="38" t="inlineStr">
         <is>
-          <t>channels.csv k_eps c2 Coil 85 (MRS_RLY); DRB102 56 = section A c27 'EPS relay coil 85 (R22) - from the MR-S pump B5'</t>
+          <t>fuse-box plan k_str 85 (18 AWG); channels.csv ecu_a A26 Aux 8 (AUX8_START_RLY)</t>
         </is>
       </c>
       <c r="AF69" s="38" t="inlineStr">
@@ -9120,19 +9098,19 @@
       </c>
       <c r="AG69" s="38" t="inlineStr">
         <is>
-          <t>owner proposed: longer half (drawn today as w_eps_rly on A-cabin, 530 mm; w_eps_rly_cp on CabinPower, 400 mm)</t>
+          <t>owner proposed: longer half (drawn today as w_str85 on A-cabin, 400 mm; w_str85_cp on CabinPower, 400 mm)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="39" t="inlineStr">
         <is>
-          <t>ACKILL</t>
+          <t>FAN</t>
         </is>
       </c>
       <c r="B70" s="39" t="inlineStr">
         <is>
-          <t>w_ac_kill</t>
+          <t>w_fan85</t>
         </is>
       </c>
       <c r="C70" s="39" t="inlineStr">
@@ -9140,7 +9118,11 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D70" s="39" t="inlineStr"/>
+      <c r="D70" s="39" t="inlineStr">
+        <is>
+          <t>CabinPower</t>
+        </is>
+      </c>
       <c r="E70" s="40" t="inlineStr">
         <is>
           <t>connector</t>
@@ -9148,110 +9130,94 @@
       </c>
       <c r="F70" s="41" t="inlineStr">
         <is>
+          <t>k_fan</t>
+        </is>
+      </c>
+      <c r="G70" s="42" t="inlineStr">
+        <is>
+          <t>POWER R4</t>
+        </is>
+      </c>
+      <c r="H70" s="41" t="n">
+        <v>85</v>
+      </c>
+      <c r="I70" s="42" t="inlineStr">
+        <is>
+          <t>Rad fan relay (-)</t>
+        </is>
+      </c>
+      <c r="J70" s="42" t="inlineStr">
+        <is>
+          <t>POWER box (glove box) relay R4 radiator fan, pin 85</t>
+        </is>
+      </c>
+      <c r="K70" s="43" t="inlineStr">
+        <is>
+          <t>connector</t>
+        </is>
+      </c>
+      <c r="L70" s="44" t="inlineStr">
+        <is>
           <t>ecu_a</t>
         </is>
       </c>
-      <c r="G70" s="42" t="inlineStr">
+      <c r="M70" s="45" t="inlineStr">
         <is>
           <t>ECU-A</t>
         </is>
       </c>
-      <c r="H70" s="41" t="inlineStr">
-        <is>
-          <t>A18</t>
-        </is>
-      </c>
-      <c r="I70" s="42" t="inlineStr">
-        <is>
-          <t>A/C cancel (ACT)</t>
-        </is>
-      </c>
-      <c r="J70" s="42" t="inlineStr"/>
-      <c r="K70" s="43" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="L70" s="44" t="inlineStr">
-        <is>
-          <t>A18 (factory)</t>
-        </is>
-      </c>
-      <c r="M70" s="45" t="inlineStr">
-        <is>
-          <t>OEM A/C amplifier</t>
-        </is>
-      </c>
-      <c r="N70" s="44" t="n">
-        <v>11</v>
+      <c r="N70" s="44" t="inlineStr">
+        <is>
+          <t>A29</t>
+        </is>
       </c>
       <c r="O70" s="45" t="inlineStr">
         <is>
-          <t>A/C cancel (ACT)</t>
-        </is>
-      </c>
-      <c r="P70" s="45" t="inlineStr">
-        <is>
-          <t>A/C amp A18 pin 11 (1993: A15), behind the glove box. Solder splice onto the factory G-Y lead. EWD 1992 p.93 / p.218; locator 1990 p.17.</t>
-        </is>
-      </c>
+          <t>Rad fan relay (-)</t>
+        </is>
+      </c>
+      <c r="P70" s="45" t="inlineStr"/>
       <c r="Q70" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A18</t>
+          <t>ECU-A.A29</t>
         </is>
       </c>
       <c r="R70" s="47" t="inlineStr">
         <is>
-          <t>A/C cancel (ACT) (ECU-A A18)</t>
+          <t>Rad fan relay (-) (ECU-A A29)</t>
         </is>
       </c>
       <c r="S70" s="48" t="inlineStr"/>
       <c r="T70" s="48" t="inlineStr"/>
       <c r="U70" s="49" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="V70" s="50" t="inlineStr">
         <is>
-          <t>Gray</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W70" s="50" t="inlineStr"/>
       <c r="X70" s="50" t="inlineStr">
         <is>
-          <t>White-Yellow-Yellow</t>
+          <t>Yellow-White</t>
         </is>
       </c>
       <c r="Y70" s="50" t="n">
-        <v>600</v>
+        <v>410</v>
       </c>
       <c r="Z70" s="51" t="inlineStr">
         <is>
-          <t>A/C amp branch (behind dash)</t>
-        </is>
-      </c>
-      <c r="AA70" s="52" t="inlineStr">
-        <is>
-          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD</t>
-        </is>
-      </c>
-      <c r="AB70" s="53" t="inlineStr">
-        <is>
-          <t>G-Y</t>
-        </is>
-      </c>
-      <c r="AC70" s="54" t="inlineStr">
-        <is>
-          <t>1992 Celica EWD132U p.93 and p.218 (docs/electrical/ewd-snips/1992-celica-ewd132u-a17-act-p093.png, 1992-celica-ewd132u-a17-clutch-p218.png); 1990 ST185 book locator A18; 1992 EWD132U p.93 and p.218 (A17-11 = A18-11); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html)</t>
-        </is>
-      </c>
-      <c r="AD70" s="54" t="inlineStr">
-        <is>
-          <t>solder splice onto the factory G-Y ACT lead at the A/C amplifier</t>
-        </is>
-      </c>
+          <t>glove-box branch (POWER / LOGIC boxes)</t>
+        </is>
+      </c>
+      <c r="AA70" s="52" t="inlineStr"/>
+      <c r="AB70" s="53" t="inlineStr"/>
+      <c r="AC70" s="54" t="inlineStr"/>
+      <c r="AD70" s="54" t="inlineStr"/>
       <c r="AE70" s="54" t="inlineStr">
         <is>
-          <t>channels.csv ecu_a A18 Aux 4 (AUX4_AC_KILL); flying lead FL_ACAMP_ACT: EWD A18 pin 11 G-Y</t>
+          <t>fuse-box plan k_fan 85 (18 AWG); channels.csv ecu_a A29 Aux 5 (AUX5_RAD_FAN)</t>
         </is>
       </c>
       <c r="AF70" s="54" t="inlineStr">
@@ -9259,17 +9225,21 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG70" s="54" t="inlineStr"/>
+      <c r="AG70" s="54" t="inlineStr">
+        <is>
+          <t>owner proposed: longer half (drawn today as w_fan85 on A-cabin, 410 mm; w_fan85_cp on CabinPower, 400 mm)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="23" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>EPS</t>
         </is>
       </c>
       <c r="B71" s="23" t="inlineStr">
         <is>
-          <t>w_ac_psw_in</t>
+          <t>w_eps_rly</t>
         </is>
       </c>
       <c r="C71" s="23" t="inlineStr">
@@ -9279,122 +9249,102 @@
       </c>
       <c r="D71" s="23" t="inlineStr">
         <is>
-          <t>EngineRoom-C</t>
+          <t>CabinPower</t>
         </is>
       </c>
       <c r="E71" s="24" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="F71" s="25" t="inlineStr">
         <is>
-          <t>A5 (factory)</t>
+          <t>k_eps</t>
         </is>
       </c>
       <c r="G71" s="26" t="inlineStr">
         <is>
-          <t>OEM A5, factory Y-R lead</t>
+          <t>EHPS RELAY</t>
         </is>
       </c>
       <c r="H71" s="25" t="n">
-        <v>4</v>
+        <v>85</v>
       </c>
       <c r="I71" s="26" t="inlineStr">
         <is>
-          <t>A/C pressure sw out</t>
+          <t>EHPS relay coil (-)</t>
         </is>
       </c>
       <c r="J71" s="26" t="inlineStr">
         <is>
-          <t>Runs on in ST185-EngineRoom-C to A/C pressure switch A5 pin 4 (engine bay): new wire to the switch's own mating plug, plug part TBD. EWD 1990 p.152.</t>
+          <t>EHPS pump relay (glove box), pin 85</t>
         </is>
       </c>
       <c r="K71" s="27" t="inlineStr">
         <is>
-          <t>splice</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="L71" s="28" t="inlineStr">
         <is>
-          <t>sp_ac_psw</t>
+          <t>bh_a_fw</t>
         </is>
       </c>
       <c r="M71" s="29" t="inlineStr">
         <is>
-          <t>splice sp_ac_psw (SP-AC-PSW: A/C pressure switch output)</t>
-        </is>
-      </c>
-      <c r="N71" s="28" t="inlineStr"/>
+          <t>BULKHEAD</t>
+        </is>
+      </c>
+      <c r="N71" s="28" t="n">
+        <v>56</v>
+      </c>
       <c r="O71" s="29" t="inlineStr">
         <is>
-          <t>A/C pressure sw out</t>
+          <t>EHPS relay coil (-)</t>
         </is>
       </c>
       <c r="P71" s="29" t="inlineStr"/>
       <c r="Q71" s="30" t="inlineStr">
         <is>
-          <t>A5.4</t>
+          <t>DRB102.56</t>
         </is>
       </c>
       <c r="R71" s="31" t="inlineStr">
         <is>
-          <t>A/C pressure-switched relay coil +</t>
-        </is>
-      </c>
-      <c r="S71" s="32" t="inlineStr">
-        <is>
-          <t>sp_ac_psw</t>
-        </is>
-      </c>
+          <t>EHPS relay coil (-) (DRB102 56)</t>
+        </is>
+      </c>
+      <c r="S71" s="32" t="inlineStr"/>
       <c r="T71" s="32" t="inlineStr"/>
       <c r="U71" s="33" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="V71" s="34" t="inlineStr">
         <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="W71" s="34" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
+          <t>Violet</t>
+        </is>
+      </c>
+      <c r="W71" s="34" t="inlineStr"/>
       <c r="X71" s="34" t="inlineStr">
         <is>
-          <t>Yellow-Blue</t>
-        </is>
-      </c>
-      <c r="Y71" s="34" t="inlineStr"/>
+          <t>Blue-Blue-Blue</t>
+        </is>
+      </c>
+      <c r="Y71" s="34" t="n">
+        <v>530</v>
+      </c>
       <c r="Z71" s="35" t="inlineStr">
         <is>
-          <t>A/C amp branch (behind dash)</t>
-        </is>
-      </c>
-      <c r="AA71" s="36" t="inlineStr">
-        <is>
-          <t>A/C pressure switch A5, engine bay; exact spot TBD (no locator figure in the repo)</t>
-        </is>
-      </c>
-      <c r="AB71" s="37" t="inlineStr">
-        <is>
-          <t>Y-R (factory wiring; new wire here)</t>
-        </is>
-      </c>
-      <c r="AC71" s="38" t="inlineStr">
-        <is>
-          <t>1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1990 ST185 EWD p.152 (A5 pin 4 Y-R)</t>
-        </is>
-      </c>
-      <c r="AD71" s="38" t="inlineStr">
-        <is>
-          <t>new-wire run terminated at the switch's own mating plug (no factory engine-bay wire reused, Section 39, 2026-10-04); plug part number not yet chosen</t>
-        </is>
-      </c>
+          <t>glove-box branch (POWER / LOGIC boxes) / trunk ECU-A to bulkhead (RH firewall)</t>
+        </is>
+      </c>
+      <c r="AA71" s="36" t="inlineStr"/>
+      <c r="AB71" s="37" t="inlineStr"/>
+      <c r="AC71" s="38" t="inlineStr"/>
+      <c r="AD71" s="38" t="inlineStr"/>
       <c r="AE71" s="38" t="inlineStr">
         <is>
-          <t>flying lead FL_A5_4: EWD A5 pin 4 Y-R (factory wiring; new wire here); splice sp_ac_psw: node of the wire list (SoT)</t>
+          <t>channels.csv k_eps c2 Coil 85 (MRS_RLY); DRB102 56 = section A c27 'EPS relay coil 85 (R22) - from the MR-S pump B5'</t>
         </is>
       </c>
       <c r="AF71" s="38" t="inlineStr">
@@ -9404,19 +9354,19 @@
       </c>
       <c r="AG71" s="38" t="inlineStr">
         <is>
-          <t>owner TBD: a half has no length estimate (drawn today as w_ac_psw_in on A-cabin, ? mm; w_ac_psw on EngineRoom-C, 100 mm)</t>
+          <t>owner proposed: longer half (drawn today as w_eps_rly on A-cabin, 530 mm; w_eps_rly_cp on CabinPower, 400 mm)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="39" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>ACKILL</t>
         </is>
       </c>
       <c r="B72" s="39" t="inlineStr">
         <is>
-          <t>w_ac_psw_sw</t>
+          <t>w_ac_kill</t>
         </is>
       </c>
       <c r="C72" s="39" t="inlineStr">
@@ -9427,89 +9377,87 @@
       <c r="D72" s="39" t="inlineStr"/>
       <c r="E72" s="40" t="inlineStr">
         <is>
+          <t>connector</t>
+        </is>
+      </c>
+      <c r="F72" s="41" t="inlineStr">
+        <is>
+          <t>ecu_a</t>
+        </is>
+      </c>
+      <c r="G72" s="42" t="inlineStr">
+        <is>
+          <t>ECU-A</t>
+        </is>
+      </c>
+      <c r="H72" s="41" t="inlineStr">
+        <is>
+          <t>A18</t>
+        </is>
+      </c>
+      <c r="I72" s="42" t="inlineStr">
+        <is>
+          <t>A/C cancel (ACT)</t>
+        </is>
+      </c>
+      <c r="J72" s="42" t="inlineStr"/>
+      <c r="K72" s="43" t="inlineStr">
+        <is>
           <t>OEM</t>
         </is>
       </c>
-      <c r="F72" s="41" t="inlineStr">
+      <c r="L72" s="44" t="inlineStr">
         <is>
           <t>A18 (factory)</t>
         </is>
       </c>
-      <c r="G72" s="42" t="inlineStr">
+      <c r="M72" s="45" t="inlineStr">
         <is>
           <t>OEM A/C amplifier</t>
         </is>
       </c>
-      <c r="H72" s="41" t="n">
-        <v>13</v>
-      </c>
-      <c r="I72" s="42" t="inlineStr">
-        <is>
-          <t>A/C pressure sw out</t>
-        </is>
-      </c>
-      <c r="J72" s="42" t="inlineStr">
-        <is>
-          <t>A/C amp A18 pin 13 (1993: A15), behind the glove box. Solder splice onto the factory Y-R lead. EWD 1990 p.152; locator 1990 p.17.</t>
-        </is>
-      </c>
-      <c r="K72" s="43" t="inlineStr">
-        <is>
-          <t>splice</t>
-        </is>
-      </c>
-      <c r="L72" s="44" t="inlineStr">
-        <is>
-          <t>sp_ac_psw</t>
-        </is>
-      </c>
-      <c r="M72" s="45" t="inlineStr">
-        <is>
-          <t>splice sp_ac_psw (SP-AC-PSW: A/C pressure switch output)</t>
-        </is>
-      </c>
-      <c r="N72" s="44" t="inlineStr"/>
+      <c r="N72" s="44" t="n">
+        <v>11</v>
+      </c>
       <c r="O72" s="45" t="inlineStr">
         <is>
-          <t>A/C pressure sw out</t>
-        </is>
-      </c>
-      <c r="P72" s="45" t="inlineStr"/>
+          <t>A/C cancel (ACT)</t>
+        </is>
+      </c>
+      <c r="P72" s="45" t="inlineStr">
+        <is>
+          <t>A/C amp A18 pin 11 (1993: A15), behind the glove box. Solder splice onto the factory G-Y lead. EWD 1992 p.93 / p.218; locator 1990 p.17.</t>
+        </is>
+      </c>
       <c r="Q72" s="46" t="inlineStr">
         <is>
-          <t>A5.4</t>
+          <t>ECU-A.A18</t>
         </is>
       </c>
       <c r="R72" s="47" t="inlineStr">
         <is>
-          <t>A/C pressure-switched relay coil +</t>
-        </is>
-      </c>
-      <c r="S72" s="48" t="inlineStr">
-        <is>
-          <t>sp_ac_psw</t>
-        </is>
-      </c>
+          <t>A/C cancel (ACT) (ECU-A A18)</t>
+        </is>
+      </c>
+      <c r="S72" s="48" t="inlineStr"/>
       <c r="T72" s="48" t="inlineStr"/>
       <c r="U72" s="49" t="n">
         <v>20</v>
       </c>
       <c r="V72" s="50" t="inlineStr">
         <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="W72" s="50" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
+          <t>Gray</t>
+        </is>
+      </c>
+      <c r="W72" s="50" t="inlineStr"/>
       <c r="X72" s="50" t="inlineStr">
         <is>
-          <t>Yellow-Blue</t>
-        </is>
-      </c>
-      <c r="Y72" s="50" t="inlineStr"/>
+          <t>White-Yellow-Yellow</t>
+        </is>
+      </c>
+      <c r="Y72" s="50" t="n">
+        <v>600</v>
+      </c>
       <c r="Z72" s="51" t="inlineStr">
         <is>
           <t>A/C amp branch (behind dash)</t>
@@ -9522,22 +9470,22 @@
       </c>
       <c r="AB72" s="53" t="inlineStr">
         <is>
-          <t>Y-R</t>
+          <t>G-Y</t>
         </is>
       </c>
       <c r="AC72" s="54" t="inlineStr">
         <is>
-          <t>1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1992 EWD132U p.219 A17-13 (ewd-snips/1992-celica-ewd132u-a17-pressure-p219.png); 1990 ST185 EWD p.152; 1992 EWD132U p.219 (A17-13); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html)</t>
+          <t>1992 Celica EWD132U p.93 and p.218 (docs/electrical/ewd-snips/1992-celica-ewd132u-a17-act-p093.png, 1992-celica-ewd132u-a17-clutch-p218.png); 1990 ST185 book locator A18; 1992 EWD132U p.93 and p.218 (A17-11 = A18-11); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html)</t>
         </is>
       </c>
       <c r="AD72" s="54" t="inlineStr">
         <is>
-          <t>solder splice onto the factory Y-R lead at the A/C amplifier</t>
+          <t>solder splice onto the factory G-Y ACT lead at the A/C amplifier</t>
         </is>
       </c>
       <c r="AE72" s="54" t="inlineStr">
         <is>
-          <t>flying lead FL_ACAMP_PSW: EWD A18 pin 13 Y-R; splice sp_ac_psw: node of the wire list (SoT)</t>
+          <t>channels.csv ecu_a A18 Aux 4 (AUX4_AC_KILL); flying lead FL_ACAMP_ACT: EWD A18 pin 11 G-Y</t>
         </is>
       </c>
       <c r="AF72" s="54" t="inlineStr">
@@ -9555,7 +9503,7 @@
       </c>
       <c r="B73" s="23" t="inlineStr">
         <is>
-          <t>w_acc86</t>
+          <t>w_ac_psw_in</t>
         </is>
       </c>
       <c r="C73" s="23" t="inlineStr">
@@ -9565,59 +9513,59 @@
       </c>
       <c r="D73" s="23" t="inlineStr">
         <is>
-          <t>CabinPower</t>
+          <t>EngineRoom-C</t>
         </is>
       </c>
       <c r="E73" s="24" t="inlineStr">
         <is>
+          <t>OEM</t>
+        </is>
+      </c>
+      <c r="F73" s="25" t="inlineStr">
+        <is>
+          <t>A5 (factory)</t>
+        </is>
+      </c>
+      <c r="G73" s="26" t="inlineStr">
+        <is>
+          <t>OEM A5, factory Y-R lead</t>
+        </is>
+      </c>
+      <c r="H73" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="I73" s="26" t="inlineStr">
+        <is>
+          <t>A/C pressure sw out</t>
+        </is>
+      </c>
+      <c r="J73" s="26" t="inlineStr">
+        <is>
+          <t>Runs on in ST185-EngineRoom-C to A/C pressure switch A5 pin 4 (engine bay): new wire to the switch's own mating plug, plug part TBD. EWD 1990 p.152.</t>
+        </is>
+      </c>
+      <c r="K73" s="27" t="inlineStr">
+        <is>
           <t>splice</t>
         </is>
       </c>
-      <c r="F73" s="25" t="inlineStr">
+      <c r="L73" s="28" t="inlineStr">
         <is>
           <t>sp_ac_psw</t>
         </is>
       </c>
-      <c r="G73" s="26" t="inlineStr">
+      <c r="M73" s="29" t="inlineStr">
         <is>
           <t>splice sp_ac_psw (SP-AC-PSW: A/C pressure switch output)</t>
         </is>
       </c>
-      <c r="H73" s="25" t="inlineStr"/>
-      <c r="I73" s="26" t="inlineStr">
-        <is>
-          <t>A/C clutch relay (+)</t>
-        </is>
-      </c>
-      <c r="J73" s="26" t="inlineStr"/>
-      <c r="K73" s="27" t="inlineStr">
-        <is>
-          <t>connector</t>
-        </is>
-      </c>
-      <c r="L73" s="28" t="inlineStr">
-        <is>
-          <t>k_acc</t>
-        </is>
-      </c>
-      <c r="M73" s="29" t="inlineStr">
-        <is>
-          <t>LOGIC M5</t>
-        </is>
-      </c>
-      <c r="N73" s="28" t="n">
-        <v>86</v>
-      </c>
+      <c r="N73" s="28" t="inlineStr"/>
       <c r="O73" s="29" t="inlineStr">
         <is>
-          <t>A/C clutch relay (+)</t>
-        </is>
-      </c>
-      <c r="P73" s="29" t="inlineStr">
-        <is>
-          <t>LOGIC box (glove box) relay M15 A/C clutch, pin 86</t>
-        </is>
-      </c>
+          <t>A/C pressure sw out</t>
+        </is>
+      </c>
+      <c r="P73" s="29" t="inlineStr"/>
       <c r="Q73" s="30" t="inlineStr">
         <is>
           <t>A5.4</t>
@@ -9635,7 +9583,7 @@
       </c>
       <c r="T73" s="32" t="inlineStr"/>
       <c r="U73" s="33" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="V73" s="34" t="inlineStr">
         <is>
@@ -9658,13 +9606,29 @@
           <t>A/C amp branch (behind dash)</t>
         </is>
       </c>
-      <c r="AA73" s="36" t="inlineStr"/>
-      <c r="AB73" s="37" t="inlineStr"/>
-      <c r="AC73" s="38" t="inlineStr"/>
-      <c r="AD73" s="38" t="inlineStr"/>
+      <c r="AA73" s="36" t="inlineStr">
+        <is>
+          <t>A/C pressure switch A5, engine bay; exact spot TBD (no locator figure in the repo)</t>
+        </is>
+      </c>
+      <c r="AB73" s="37" t="inlineStr">
+        <is>
+          <t>Y-R (factory wiring; new wire here)</t>
+        </is>
+      </c>
+      <c r="AC73" s="38" t="inlineStr">
+        <is>
+          <t>1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1990 ST185 EWD p.152 (A5 pin 4 Y-R)</t>
+        </is>
+      </c>
+      <c r="AD73" s="38" t="inlineStr">
+        <is>
+          <t>new-wire run terminated at the switch's own mating plug (no factory engine-bay wire reused, Section 39, 2026-10-04); plug part number not yet chosen</t>
+        </is>
+      </c>
       <c r="AE73" s="38" t="inlineStr">
         <is>
-          <t>splice sp_ac_psw: node of the wire list (SoT); fuse-box plan k_acc 86 (18 AWG)</t>
+          <t>flying lead FL_A5_4: EWD A5 pin 4 Y-R (factory wiring; new wire here); splice sp_ac_psw: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF73" s="38" t="inlineStr">
@@ -9674,19 +9638,19 @@
       </c>
       <c r="AG73" s="38" t="inlineStr">
         <is>
-          <t>owner TBD: a half has no length estimate (drawn today as w_acc86 on A-cabin, ? mm; w_acc86_cp on CabinPower, 400 mm)</t>
+          <t>owner TBD: a half has no length estimate (drawn today as w_ac_psw_in on A-cabin, ? mm; w_ac_psw on EngineRoom-C, 100 mm)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="39" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="B74" s="39" t="inlineStr">
         <is>
-          <t>w_aps_vc1</t>
+          <t>w_ac_psw_sw</t>
         </is>
       </c>
       <c r="C74" s="39" t="inlineStr">
@@ -9697,28 +9661,32 @@
       <c r="D74" s="39" t="inlineStr"/>
       <c r="E74" s="40" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F74" s="41" t="inlineStr">
         <is>
-          <t>aps</t>
+          <t>A18 (factory)</t>
         </is>
       </c>
       <c r="G74" s="42" t="inlineStr">
         <is>
-          <t>PEDAL</t>
+          <t>OEM A/C amplifier</t>
         </is>
       </c>
       <c r="H74" s="41" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="I74" s="42" t="inlineStr">
         <is>
-          <t>+5 V pedal sensor 1</t>
-        </is>
-      </c>
-      <c r="J74" s="42" t="inlineStr"/>
+          <t>A/C pressure sw out</t>
+        </is>
+      </c>
+      <c r="J74" s="42" t="inlineStr">
+        <is>
+          <t>A/C amp A18 pin 13 (1993: A15), behind the glove box. Solder splice onto the factory Y-R lead. EWD 1990 p.152; locator 1990 p.17.</t>
+        </is>
+      </c>
       <c r="K74" s="43" t="inlineStr">
         <is>
           <t>splice</t>
@@ -9726,68 +9694,84 @@
       </c>
       <c r="L74" s="44" t="inlineStr">
         <is>
-          <t>sp_5v_2</t>
+          <t>sp_ac_psw</t>
         </is>
       </c>
       <c r="M74" s="45" t="inlineStr">
         <is>
-          <t>splice sp_5v_2 (SP-5V-PEDAL: +5 V to pedal + cruise)</t>
+          <t>splice sp_ac_psw (SP-AC-PSW: A/C pressure switch output)</t>
         </is>
       </c>
       <c r="N74" s="44" t="inlineStr"/>
       <c r="O74" s="45" t="inlineStr">
         <is>
-          <t>+5 V pedal sensor 1</t>
+          <t>A/C pressure sw out</t>
         </is>
       </c>
       <c r="P74" s="45" t="inlineStr"/>
       <c r="Q74" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A32</t>
+          <t>A5.4</t>
         </is>
       </c>
       <c r="R74" s="47" t="inlineStr">
         <is>
-          <t>+5V sensor (ECU-A A32)</t>
+          <t>A/C pressure-switched relay coil +</t>
         </is>
       </c>
       <c r="S74" s="48" t="inlineStr">
         <is>
-          <t>sp_5v_2</t>
-        </is>
-      </c>
-      <c r="T74" s="48" t="inlineStr">
-        <is>
-          <t>cab_aps1</t>
-        </is>
-      </c>
+          <t>sp_ac_psw</t>
+        </is>
+      </c>
+      <c r="T74" s="48" t="inlineStr"/>
       <c r="U74" s="49" t="n">
         <v>20</v>
       </c>
       <c r="V74" s="50" t="inlineStr">
         <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="W74" s="50" t="inlineStr">
+        <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="W74" s="50" t="inlineStr"/>
       <c r="X74" s="50" t="inlineStr">
         <is>
-          <t>Blue-Blue</t>
+          <t>Yellow-Blue</t>
         </is>
       </c>
       <c r="Y74" s="50" t="inlineStr"/>
       <c r="Z74" s="51" t="inlineStr">
         <is>
-          <t>pedal branch (driver footwell)</t>
-        </is>
-      </c>
-      <c r="AA74" s="52" t="inlineStr"/>
-      <c r="AB74" s="53" t="inlineStr"/>
-      <c r="AC74" s="54" t="inlineStr"/>
-      <c r="AD74" s="54" t="inlineStr"/>
+          <t>A/C amp branch (behind dash)</t>
+        </is>
+      </c>
+      <c r="AA74" s="52" t="inlineStr">
+        <is>
+          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD</t>
+        </is>
+      </c>
+      <c r="AB74" s="53" t="inlineStr">
+        <is>
+          <t>Y-R</t>
+        </is>
+      </c>
+      <c r="AC74" s="54" t="inlineStr">
+        <is>
+          <t>1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1992 EWD132U p.219 A17-13 (ewd-snips/1992-celica-ewd132u-a17-pressure-p219.png); 1990 ST185 EWD p.152; 1992 EWD132U p.219 (A17-13); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html)</t>
+        </is>
+      </c>
+      <c r="AD74" s="54" t="inlineStr">
+        <is>
+          <t>solder splice onto the factory Y-R lead at the A/C amplifier</t>
+        </is>
+      </c>
       <c r="AE74" s="54" t="inlineStr">
         <is>
-          <t>splice sp_5v_2: node of the wire list (SoT)</t>
+          <t>flying lead FL_ACAMP_PSW: EWD A18 pin 13 Y-R; splice sp_ac_psw: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF74" s="54" t="inlineStr">
@@ -9795,21 +9779,17 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG74" s="54" t="inlineStr">
-        <is>
-          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
-        </is>
-      </c>
+      <c r="AG74" s="54" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="23" t="inlineStr">
         <is>
-          <t>SGND</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="B75" s="23" t="inlineStr">
         <is>
-          <t>w40</t>
+          <t>w_acc86</t>
         </is>
       </c>
       <c r="C75" s="23" t="inlineStr">
@@ -9817,91 +9797,99 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D75" s="23" t="inlineStr"/>
+      <c r="D75" s="23" t="inlineStr">
+        <is>
+          <t>CabinPower</t>
+        </is>
+      </c>
       <c r="E75" s="24" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="F75" s="25" t="inlineStr">
         <is>
-          <t>aps</t>
+          <t>sp_ac_psw</t>
         </is>
       </c>
       <c r="G75" s="26" t="inlineStr">
         <is>
-          <t>PEDAL</t>
-        </is>
-      </c>
-      <c r="H75" s="25" t="n">
-        <v>5</v>
-      </c>
+          <t>splice sp_ac_psw (SP-AC-PSW: A/C pressure switch output)</t>
+        </is>
+      </c>
+      <c r="H75" s="25" t="inlineStr"/>
       <c r="I75" s="26" t="inlineStr">
         <is>
-          <t>Pedal 1 ground</t>
+          <t>A/C clutch relay (+)</t>
         </is>
       </c>
       <c r="J75" s="26" t="inlineStr"/>
       <c r="K75" s="27" t="inlineStr">
         <is>
-          <t>splice</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="L75" s="28" t="inlineStr">
         <is>
-          <t>sp_gndout</t>
+          <t>k_acc</t>
         </is>
       </c>
       <c r="M75" s="29" t="inlineStr">
         <is>
-          <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
-        </is>
-      </c>
-      <c r="N75" s="28" t="inlineStr"/>
+          <t>LOGIC M5</t>
+        </is>
+      </c>
+      <c r="N75" s="28" t="n">
+        <v>86</v>
+      </c>
       <c r="O75" s="29" t="inlineStr">
         <is>
-          <t>Pedal 1 ground</t>
-        </is>
-      </c>
-      <c r="P75" s="29" t="inlineStr"/>
+          <t>A/C clutch relay (+)</t>
+        </is>
+      </c>
+      <c r="P75" s="29" t="inlineStr">
+        <is>
+          <t>LOGIC box (glove box) relay M15 A/C clutch, pin 86</t>
+        </is>
+      </c>
       <c r="Q75" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A24</t>
+          <t>A5.4</t>
         </is>
       </c>
       <c r="R75" s="31" t="inlineStr">
         <is>
-          <t>Sensor GND (ECU-A A24)</t>
+          <t>A/C pressure-switched relay coil +</t>
         </is>
       </c>
       <c r="S75" s="32" t="inlineStr">
         <is>
-          <t>sp_gndout</t>
-        </is>
-      </c>
-      <c r="T75" s="32" t="inlineStr">
-        <is>
-          <t>cab_aps1</t>
-        </is>
-      </c>
+          <t>sp_ac_psw</t>
+        </is>
+      </c>
+      <c r="T75" s="32" t="inlineStr"/>
       <c r="U75" s="33" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="V75" s="34" t="inlineStr">
         <is>
           <t>Yellow</t>
         </is>
       </c>
-      <c r="W75" s="34" t="inlineStr"/>
+      <c r="W75" s="34" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
       <c r="X75" s="34" t="inlineStr">
         <is>
-          <t>Yellow-Yellow-Blue</t>
+          <t>Yellow-Blue</t>
         </is>
       </c>
       <c r="Y75" s="34" t="inlineStr"/>
       <c r="Z75" s="35" t="inlineStr">
         <is>
-          <t>pedal branch (driver footwell)</t>
+          <t>A/C amp branch (behind dash)</t>
         </is>
       </c>
       <c r="AA75" s="36" t="inlineStr"/>
@@ -9910,7 +9898,7 @@
       <c r="AD75" s="38" t="inlineStr"/>
       <c r="AE75" s="38" t="inlineStr">
         <is>
-          <t>splice sp_gndout: node of the wire list (SoT)</t>
+          <t>splice sp_ac_psw: node of the wire list (SoT); fuse-box plan k_acc 86 (18 AWG)</t>
         </is>
       </c>
       <c r="AF75" s="38" t="inlineStr">
@@ -9920,19 +9908,19 @@
       </c>
       <c r="AG75" s="38" t="inlineStr">
         <is>
-          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
+          <t>owner TBD: a half has no length estimate (drawn today as w_acc86 on A-cabin, ? mm; w_acc86_cp on CabinPower, 400 mm)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="39" t="inlineStr">
         <is>
-          <t>APS</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="B76" s="39" t="inlineStr">
         <is>
-          <t>w38</t>
+          <t>w_aps_vc1</t>
         </is>
       </c>
       <c r="C76" s="39" t="inlineStr">
@@ -9957,51 +9945,51 @@
         </is>
       </c>
       <c r="H76" s="41" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I76" s="42" t="inlineStr">
         <is>
-          <t>Pedal 1 signal main</t>
+          <t>+5 V pedal sensor 1</t>
         </is>
       </c>
       <c r="J76" s="42" t="inlineStr"/>
       <c r="K76" s="43" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="L76" s="44" t="inlineStr">
         <is>
-          <t>ecu_a</t>
+          <t>sp_5v_2</t>
         </is>
       </c>
       <c r="M76" s="45" t="inlineStr">
         <is>
-          <t>ECU-A</t>
-        </is>
-      </c>
-      <c r="N76" s="44" t="inlineStr">
-        <is>
-          <t>A14</t>
-        </is>
-      </c>
+          <t>splice sp_5v_2 (SP-5V-PEDAL: +5 V to pedal + cruise)</t>
+        </is>
+      </c>
+      <c r="N76" s="44" t="inlineStr"/>
       <c r="O76" s="45" t="inlineStr">
         <is>
-          <t>Pedal 1 signal main</t>
+          <t>+5 V pedal sensor 1</t>
         </is>
       </c>
       <c r="P76" s="45" t="inlineStr"/>
       <c r="Q76" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A14</t>
+          <t>ECU-A.A32</t>
         </is>
       </c>
       <c r="R76" s="47" t="inlineStr">
         <is>
-          <t>Pedal 1 signal main (ECU-A A14)</t>
-        </is>
-      </c>
-      <c r="S76" s="48" t="inlineStr"/>
+          <t>+5V sensor (ECU-A A32)</t>
+        </is>
+      </c>
+      <c r="S76" s="48" t="inlineStr">
+        <is>
+          <t>sp_5v_2</t>
+        </is>
+      </c>
       <c r="T76" s="48" t="inlineStr">
         <is>
           <t>cab_aps1</t>
@@ -10012,18 +10000,16 @@
       </c>
       <c r="V76" s="50" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="W76" s="50" t="inlineStr"/>
       <c r="X76" s="50" t="inlineStr">
         <is>
-          <t>White-Blue-Yellow</t>
-        </is>
-      </c>
-      <c r="Y76" s="50" t="n">
-        <v>1050</v>
-      </c>
+          <t>Blue-Blue</t>
+        </is>
+      </c>
+      <c r="Y76" s="50" t="inlineStr"/>
       <c r="Z76" s="51" t="inlineStr">
         <is>
           <t>pedal branch (driver footwell)</t>
@@ -10035,7 +10021,7 @@
       <c r="AD76" s="54" t="inlineStr"/>
       <c r="AE76" s="54" t="inlineStr">
         <is>
-          <t>channels.csv ecu_a A14 An Volt 4 (AV4_APS_MAIN)</t>
+          <t>splice sp_5v_2: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF76" s="54" t="inlineStr">
@@ -10052,12 +10038,12 @@
     <row r="77">
       <c r="A77" s="23" t="inlineStr">
         <is>
-          <t>APS</t>
+          <t>SGND</t>
         </is>
       </c>
       <c r="B77" s="23" t="inlineStr">
         <is>
-          <t>cab_aps1_sh</t>
+          <t>w40</t>
         </is>
       </c>
       <c r="C77" s="23" t="inlineStr">
@@ -10068,23 +10054,25 @@
       <c r="D77" s="23" t="inlineStr"/>
       <c r="E77" s="24" t="inlineStr">
         <is>
-          <t>cable screen</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="F77" s="25" t="inlineStr">
         <is>
-          <t>cab_aps1</t>
+          <t>aps</t>
         </is>
       </c>
       <c r="G77" s="26" t="inlineStr">
         <is>
-          <t>cable screen (one end only)</t>
-        </is>
-      </c>
-      <c r="H77" s="25" t="inlineStr"/>
+          <t>PEDAL</t>
+        </is>
+      </c>
+      <c r="H77" s="25" t="n">
+        <v>5</v>
+      </c>
       <c r="I77" s="26" t="inlineStr">
         <is>
-          <t>Pedal 1 cable shield</t>
+          <t>Pedal 1 ground</t>
         </is>
       </c>
       <c r="J77" s="26" t="inlineStr"/>
@@ -10095,34 +10083,34 @@
       </c>
       <c r="L77" s="28" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>sp_gndout</t>
         </is>
       </c>
       <c r="M77" s="29" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
       <c r="N77" s="28" t="inlineStr"/>
       <c r="O77" s="29" t="inlineStr">
         <is>
-          <t>Pedal 1 cable shield</t>
+          <t>Pedal 1 ground</t>
         </is>
       </c>
       <c r="P77" s="29" t="inlineStr"/>
       <c r="Q77" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A7</t>
+          <t>ECU-A.A24</t>
         </is>
       </c>
       <c r="R77" s="31" t="inlineStr">
         <is>
-          <t>Screen A (ECU A7, SHIELD_A)</t>
+          <t>Sensor GND (ECU-A A24)</t>
         </is>
       </c>
       <c r="S77" s="32" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>sp_gndout</t>
         </is>
       </c>
       <c r="T77" s="32" t="inlineStr">
@@ -10130,22 +10118,24 @@
           <t>cab_aps1</t>
         </is>
       </c>
-      <c r="U77" s="33" t="inlineStr"/>
+      <c r="U77" s="33" t="n">
+        <v>20</v>
+      </c>
       <c r="V77" s="34" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="W77" s="34" t="inlineStr"/>
       <c r="X77" s="34" t="inlineStr">
         <is>
-          <t>White-Blue-Yellow</t>
+          <t>Yellow-Yellow-Blue</t>
         </is>
       </c>
       <c r="Y77" s="34" t="inlineStr"/>
       <c r="Z77" s="35" t="inlineStr">
         <is>
-          <t>at ECU-A plug</t>
+          <t>pedal branch (driver footwell)</t>
         </is>
       </c>
       <c r="AA77" s="36" t="inlineStr"/>
@@ -10154,7 +10144,7 @@
       <c r="AD77" s="38" t="inlineStr"/>
       <c r="AE77" s="38" t="inlineStr">
         <is>
-          <t>splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>splice sp_gndout: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF77" s="38" t="inlineStr">
@@ -10164,19 +10154,19 @@
       </c>
       <c r="AG77" s="38" t="inlineStr">
         <is>
-          <t>screen floats at the far end; pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
+          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="39" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>APS</t>
         </is>
       </c>
       <c r="B78" s="39" t="inlineStr">
         <is>
-          <t>w210</t>
+          <t>w38</t>
         </is>
       </c>
       <c r="C78" s="39" t="inlineStr">
@@ -10201,54 +10191,54 @@
         </is>
       </c>
       <c r="H78" s="41" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I78" s="42" t="inlineStr">
         <is>
-          <t>+5 V pedal sensor 2</t>
+          <t>Pedal 1 signal main</t>
         </is>
       </c>
       <c r="J78" s="42" t="inlineStr"/>
       <c r="K78" s="43" t="inlineStr">
         <is>
-          <t>splice</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="L78" s="44" t="inlineStr">
         <is>
-          <t>sp_5v_2</t>
+          <t>ecu_a</t>
         </is>
       </c>
       <c r="M78" s="45" t="inlineStr">
         <is>
-          <t>splice sp_5v_2 (SP-5V-PEDAL: +5 V to pedal + cruise)</t>
-        </is>
-      </c>
-      <c r="N78" s="44" t="inlineStr"/>
+          <t>ECU-A</t>
+        </is>
+      </c>
+      <c r="N78" s="44" t="inlineStr">
+        <is>
+          <t>A14</t>
+        </is>
+      </c>
       <c r="O78" s="45" t="inlineStr">
         <is>
-          <t>+5 V pedal sensor 2</t>
+          <t>Pedal 1 signal main</t>
         </is>
       </c>
       <c r="P78" s="45" t="inlineStr"/>
       <c r="Q78" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A32</t>
+          <t>ECU-A.A14</t>
         </is>
       </c>
       <c r="R78" s="47" t="inlineStr">
         <is>
-          <t>+5V sensor (ECU-A A32)</t>
-        </is>
-      </c>
-      <c r="S78" s="48" t="inlineStr">
-        <is>
-          <t>sp_5v_2</t>
-        </is>
-      </c>
+          <t>Pedal 1 signal main (ECU-A A14)</t>
+        </is>
+      </c>
+      <c r="S78" s="48" t="inlineStr"/>
       <c r="T78" s="48" t="inlineStr">
         <is>
-          <t>cab_aps2</t>
+          <t>cab_aps1</t>
         </is>
       </c>
       <c r="U78" s="49" t="n">
@@ -10256,16 +10246,18 @@
       </c>
       <c r="V78" s="50" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="W78" s="50" t="inlineStr"/>
       <c r="X78" s="50" t="inlineStr">
         <is>
-          <t>Blue-Blue</t>
-        </is>
-      </c>
-      <c r="Y78" s="50" t="inlineStr"/>
+          <t>White-Blue-Yellow</t>
+        </is>
+      </c>
+      <c r="Y78" s="50" t="n">
+        <v>1050</v>
+      </c>
       <c r="Z78" s="51" t="inlineStr">
         <is>
           <t>pedal branch (driver footwell)</t>
@@ -10277,7 +10269,7 @@
       <c r="AD78" s="54" t="inlineStr"/>
       <c r="AE78" s="54" t="inlineStr">
         <is>
-          <t>splice sp_5v_2: node of the wire list (SoT)</t>
+          <t>channels.csv ecu_a A14 An Volt 4 (AV4_APS_MAIN)</t>
         </is>
       </c>
       <c r="AF78" s="54" t="inlineStr">
@@ -10294,12 +10286,12 @@
     <row r="79">
       <c r="A79" s="23" t="inlineStr">
         <is>
-          <t>SGND</t>
+          <t>APS</t>
         </is>
       </c>
       <c r="B79" s="23" t="inlineStr">
         <is>
-          <t>w_aps_gnd2</t>
+          <t>cab_aps1_sh</t>
         </is>
       </c>
       <c r="C79" s="23" t="inlineStr">
@@ -10310,25 +10302,23 @@
       <c r="D79" s="23" t="inlineStr"/>
       <c r="E79" s="24" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>cable screen</t>
         </is>
       </c>
       <c r="F79" s="25" t="inlineStr">
         <is>
-          <t>aps</t>
+          <t>cab_aps1</t>
         </is>
       </c>
       <c r="G79" s="26" t="inlineStr">
         <is>
-          <t>PEDAL</t>
-        </is>
-      </c>
-      <c r="H79" s="25" t="n">
-        <v>2</v>
-      </c>
+          <t>cable screen (one end only)</t>
+        </is>
+      </c>
+      <c r="H79" s="25" t="inlineStr"/>
       <c r="I79" s="26" t="inlineStr">
         <is>
-          <t>Pedal 2 ground</t>
+          <t>Pedal 1 cable shield</t>
         </is>
       </c>
       <c r="J79" s="26" t="inlineStr"/>
@@ -10339,59 +10329,57 @@
       </c>
       <c r="L79" s="28" t="inlineStr">
         <is>
-          <t>sp_gndout</t>
+          <t>sp_shield_a_aps</t>
         </is>
       </c>
       <c r="M79" s="29" t="inlineStr">
         <is>
-          <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
+          <t>splice sp_shield_a_aps (SP-SHIELD-A-APS)</t>
         </is>
       </c>
       <c r="N79" s="28" t="inlineStr"/>
       <c r="O79" s="29" t="inlineStr">
         <is>
-          <t>Pedal 2 ground</t>
+          <t>Pedal 1 cable shield</t>
         </is>
       </c>
       <c r="P79" s="29" t="inlineStr"/>
       <c r="Q79" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A24</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R79" s="31" t="inlineStr">
         <is>
-          <t>Sensor GND (ECU-A A24)</t>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
         </is>
       </c>
       <c r="S79" s="32" t="inlineStr">
         <is>
-          <t>sp_gndout</t>
+          <t>sp_shield_a_aps</t>
         </is>
       </c>
       <c r="T79" s="32" t="inlineStr">
         <is>
-          <t>cab_aps2</t>
-        </is>
-      </c>
-      <c r="U79" s="33" t="n">
-        <v>20</v>
-      </c>
+          <t>cab_aps1</t>
+        </is>
+      </c>
+      <c r="U79" s="33" t="inlineStr"/>
       <c r="V79" s="34" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="W79" s="34" t="inlineStr"/>
       <c r="X79" s="34" t="inlineStr">
         <is>
-          <t>Yellow-Yellow-Blue</t>
+          <t>White-Blue-Yellow</t>
         </is>
       </c>
       <c r="Y79" s="34" t="inlineStr"/>
       <c r="Z79" s="35" t="inlineStr">
         <is>
-          <t>pedal branch (driver footwell)</t>
+          <t>at ECU-A plug</t>
         </is>
       </c>
       <c r="AA79" s="36" t="inlineStr"/>
@@ -10400,7 +10388,7 @@
       <c r="AD79" s="38" t="inlineStr"/>
       <c r="AE79" s="38" t="inlineStr">
         <is>
-          <t>splice sp_gndout: node of the wire list (SoT)</t>
+          <t>splice sp_shield_a_aps: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF79" s="38" t="inlineStr">
@@ -10410,19 +10398,19 @@
       </c>
       <c r="AG79" s="38" t="inlineStr">
         <is>
-          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
+          <t>screen floats at the far end; pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="39" t="inlineStr">
         <is>
-          <t>APS</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="B80" s="39" t="inlineStr">
         <is>
-          <t>w_aps_vpa2</t>
+          <t>w210</t>
         </is>
       </c>
       <c r="C80" s="39" t="inlineStr">
@@ -10430,11 +10418,7 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D80" s="39" t="inlineStr">
-        <is>
-          <t>B-cabin</t>
-        </is>
-      </c>
+      <c r="D80" s="39" t="inlineStr"/>
       <c r="E80" s="40" t="inlineStr">
         <is>
           <t>connector</t>
@@ -10451,55 +10435,51 @@
         </is>
       </c>
       <c r="H80" s="41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I80" s="42" t="inlineStr">
         <is>
-          <t>Pedal 2 signal sub</t>
+          <t>+5 V pedal sensor 2</t>
         </is>
       </c>
       <c r="J80" s="42" t="inlineStr"/>
       <c r="K80" s="43" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="L80" s="44" t="inlineStr">
         <is>
-          <t>ecu_b</t>
+          <t>sp_5v_2</t>
         </is>
       </c>
       <c r="M80" s="45" t="inlineStr">
         <is>
-          <t>ECU-B (Link G4X plug B, centre dash)</t>
-        </is>
-      </c>
-      <c r="N80" s="44" t="inlineStr">
-        <is>
-          <t>B33</t>
-        </is>
-      </c>
+          <t>splice sp_5v_2 (SP-5V-PEDAL: +5 V to pedal + cruise)</t>
+        </is>
+      </c>
+      <c r="N80" s="44" t="inlineStr"/>
       <c r="O80" s="45" t="inlineStr">
         <is>
-          <t>Pedal 2 signal sub</t>
-        </is>
-      </c>
-      <c r="P80" s="45" t="inlineStr">
-        <is>
-          <t>ECU-B plug pin B33 (Link G4X, centre dash); VPA2</t>
-        </is>
-      </c>
+          <t>+5 V pedal sensor 2</t>
+        </is>
+      </c>
+      <c r="P80" s="45" t="inlineStr"/>
       <c r="Q80" s="46" t="inlineStr">
         <is>
-          <t>ECU-B.B33</t>
+          <t>ECU-A.A32</t>
         </is>
       </c>
       <c r="R80" s="47" t="inlineStr">
         <is>
-          <t>Pedal 2 signal sub (ECU-B B33)</t>
-        </is>
-      </c>
-      <c r="S80" s="48" t="inlineStr"/>
+          <t>+5V sensor (ECU-A A32)</t>
+        </is>
+      </c>
+      <c r="S80" s="48" t="inlineStr">
+        <is>
+          <t>sp_5v_2</t>
+        </is>
+      </c>
       <c r="T80" s="48" t="inlineStr">
         <is>
           <t>cab_aps2</t>
@@ -10510,21 +10490,19 @@
       </c>
       <c r="V80" s="50" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="W80" s="50" t="inlineStr"/>
       <c r="X80" s="50" t="inlineStr">
         <is>
-          <t>White-Blue-Yellow</t>
-        </is>
-      </c>
-      <c r="Y80" s="50" t="n">
-        <v>1720</v>
-      </c>
+          <t>Blue-Blue</t>
+        </is>
+      </c>
+      <c r="Y80" s="50" t="inlineStr"/>
       <c r="Z80" s="51" t="inlineStr">
         <is>
-          <t>pedal branch (driver footwell) / to ECU-B plug (beside ECU-A)</t>
+          <t>pedal branch (driver footwell)</t>
         </is>
       </c>
       <c r="AA80" s="52" t="inlineStr"/>
@@ -10533,7 +10511,7 @@
       <c r="AD80" s="54" t="inlineStr"/>
       <c r="AE80" s="54" t="inlineStr">
         <is>
-          <t>channels.csv ecu_b B33 An Volt 5 (AV5_APS_SUB)</t>
+          <t>splice sp_5v_2: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF80" s="54" t="inlineStr">
@@ -10543,19 +10521,19 @@
       </c>
       <c r="AG80" s="54" t="inlineStr">
         <is>
-          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143); owner proposed: longer half (drawn today as w_aps_vpa2 on A-cabin, 1720 mm; w39 on B-cabin, 1250 mm)</t>
+          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="23" t="inlineStr">
         <is>
-          <t>APS</t>
+          <t>SGND</t>
         </is>
       </c>
       <c r="B81" s="23" t="inlineStr">
         <is>
-          <t>cab_aps_sh</t>
+          <t>w_aps_gnd2</t>
         </is>
       </c>
       <c r="C81" s="23" t="inlineStr">
@@ -10566,23 +10544,25 @@
       <c r="D81" s="23" t="inlineStr"/>
       <c r="E81" s="24" t="inlineStr">
         <is>
-          <t>cable screen</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="F81" s="25" t="inlineStr">
         <is>
-          <t>cab_aps2</t>
+          <t>aps</t>
         </is>
       </c>
       <c r="G81" s="26" t="inlineStr">
         <is>
-          <t>cable screen (one end only)</t>
-        </is>
-      </c>
-      <c r="H81" s="25" t="inlineStr"/>
+          <t>PEDAL</t>
+        </is>
+      </c>
+      <c r="H81" s="25" t="n">
+        <v>2</v>
+      </c>
       <c r="I81" s="26" t="inlineStr">
         <is>
-          <t>Pedal 2 cable shield</t>
+          <t>Pedal 2 ground</t>
         </is>
       </c>
       <c r="J81" s="26" t="inlineStr"/>
@@ -10593,34 +10573,34 @@
       </c>
       <c r="L81" s="28" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>sp_gndout</t>
         </is>
       </c>
       <c r="M81" s="29" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
       <c r="N81" s="28" t="inlineStr"/>
       <c r="O81" s="29" t="inlineStr">
         <is>
-          <t>Pedal 2 cable shield</t>
+          <t>Pedal 2 ground</t>
         </is>
       </c>
       <c r="P81" s="29" t="inlineStr"/>
       <c r="Q81" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A7</t>
+          <t>ECU-A.A24</t>
         </is>
       </c>
       <c r="R81" s="31" t="inlineStr">
         <is>
-          <t>Screen A (ECU A7, SHIELD_A)</t>
+          <t>Sensor GND (ECU-A A24)</t>
         </is>
       </c>
       <c r="S81" s="32" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>sp_gndout</t>
         </is>
       </c>
       <c r="T81" s="32" t="inlineStr">
@@ -10628,22 +10608,24 @@
           <t>cab_aps2</t>
         </is>
       </c>
-      <c r="U81" s="33" t="inlineStr"/>
+      <c r="U81" s="33" t="n">
+        <v>20</v>
+      </c>
       <c r="V81" s="34" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="W81" s="34" t="inlineStr"/>
       <c r="X81" s="34" t="inlineStr">
         <is>
-          <t>White-Blue-Yellow</t>
+          <t>Yellow-Yellow-Blue</t>
         </is>
       </c>
       <c r="Y81" s="34" t="inlineStr"/>
       <c r="Z81" s="35" t="inlineStr">
         <is>
-          <t>at ECU-A plug</t>
+          <t>pedal branch (driver footwell)</t>
         </is>
       </c>
       <c r="AA81" s="36" t="inlineStr"/>
@@ -10652,7 +10634,7 @@
       <c r="AD81" s="38" t="inlineStr"/>
       <c r="AE81" s="38" t="inlineStr">
         <is>
-          <t>splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>splice sp_gndout: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF81" s="38" t="inlineStr">
@@ -10662,19 +10644,19 @@
       </c>
       <c r="AG81" s="38" t="inlineStr">
         <is>
-          <t>screen floats at the far end; pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
+          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="39" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>APS</t>
         </is>
       </c>
       <c r="B82" s="39" t="inlineStr">
         <is>
-          <t>cab_fspur_5v</t>
+          <t>w_aps_vpa2</t>
         </is>
       </c>
       <c r="C82" s="39" t="inlineStr">
@@ -10682,7 +10664,11 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D82" s="39" t="inlineStr"/>
+      <c r="D82" s="39" t="inlineStr">
+        <is>
+          <t>B-cabin</t>
+        </is>
+      </c>
       <c r="E82" s="40" t="inlineStr">
         <is>
           <t>connector</t>
@@ -10690,63 +10676,67 @@
       </c>
       <c r="F82" s="41" t="inlineStr">
         <is>
-          <t>ix_ws_front_p</t>
+          <t>aps</t>
         </is>
       </c>
       <c r="G82" s="42" t="inlineStr">
         <is>
-          <t>FRONT WS INLINE</t>
+          <t>PEDAL</t>
         </is>
       </c>
       <c r="H82" s="41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I82" s="42" t="inlineStr">
         <is>
-          <t>VRC-F +5V</t>
+          <t>Pedal 2 signal sub</t>
         </is>
       </c>
       <c r="J82" s="42" t="inlineStr"/>
       <c r="K82" s="43" t="inlineStr">
         <is>
-          <t>splice</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="L82" s="44" t="inlineStr">
         <is>
-          <t>sp_5v</t>
+          <t>ecu_b</t>
         </is>
       </c>
       <c r="M82" s="45" t="inlineStr">
         <is>
-          <t>splice sp_5v (SP-5V-A: +5 V sensor supply)</t>
-        </is>
-      </c>
-      <c r="N82" s="44" t="inlineStr"/>
+          <t>ECU-B (Link G4X plug B, centre dash)</t>
+        </is>
+      </c>
+      <c r="N82" s="44" t="inlineStr">
+        <is>
+          <t>B33</t>
+        </is>
+      </c>
       <c r="O82" s="45" t="inlineStr">
         <is>
-          <t>VRC-F +5V</t>
-        </is>
-      </c>
-      <c r="P82" s="45" t="inlineStr"/>
+          <t>Pedal 2 signal sub</t>
+        </is>
+      </c>
+      <c r="P82" s="45" t="inlineStr">
+        <is>
+          <t>ECU-B plug pin B33 (Link G4X, centre dash); VPA2</t>
+        </is>
+      </c>
       <c r="Q82" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A32</t>
+          <t>ECU-B.B33</t>
         </is>
       </c>
       <c r="R82" s="47" t="inlineStr">
         <is>
-          <t>+5V sensor (ECU-A A32)</t>
-        </is>
-      </c>
-      <c r="S82" s="48" t="inlineStr">
-        <is>
-          <t>sp_5v</t>
-        </is>
-      </c>
+          <t>Pedal 2 signal sub (ECU-B B33)</t>
+        </is>
+      </c>
+      <c r="S82" s="48" t="inlineStr"/>
       <c r="T82" s="48" t="inlineStr">
         <is>
-          <t>cab_fspur</t>
+          <t>cab_aps2</t>
         </is>
       </c>
       <c r="U82" s="49" t="n">
@@ -10754,19 +10744,21 @@
       </c>
       <c r="V82" s="50" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="W82" s="50" t="inlineStr"/>
       <c r="X82" s="50" t="inlineStr">
         <is>
-          <t>Blue-Blue</t>
-        </is>
-      </c>
-      <c r="Y82" s="50" t="inlineStr"/>
+          <t>White-Blue-Yellow</t>
+        </is>
+      </c>
+      <c r="Y82" s="50" t="n">
+        <v>1720</v>
+      </c>
       <c r="Z82" s="51" t="inlineStr">
         <is>
-          <t>dash branch (front WS inline)</t>
+          <t>pedal branch (driver footwell) / to ECU-B plug (beside ECU-A)</t>
         </is>
       </c>
       <c r="AA82" s="52" t="inlineStr"/>
@@ -10775,7 +10767,7 @@
       <c r="AD82" s="54" t="inlineStr"/>
       <c r="AE82" s="54" t="inlineStr">
         <is>
-          <t>splice sp_5v: node of the wire list (SoT)</t>
+          <t>channels.csv ecu_b B33 An Volt 5 (AV5_APS_SUB)</t>
         </is>
       </c>
       <c r="AF82" s="54" t="inlineStr">
@@ -10783,17 +10775,21 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG82" s="54" t="inlineStr"/>
+      <c r="AG82" s="54" t="inlineStr">
+        <is>
+          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143); owner proposed: longer half (drawn today as w_aps_vpa2 on A-cabin, 1720 mm; w39 on B-cabin, 1250 mm)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="23" t="inlineStr">
         <is>
-          <t>SGND</t>
+          <t>APS</t>
         </is>
       </c>
       <c r="B83" s="23" t="inlineStr">
         <is>
-          <t>cab_fspur_gnd</t>
+          <t>cab_aps_sh</t>
         </is>
       </c>
       <c r="C83" s="23" t="inlineStr">
@@ -10804,25 +10800,23 @@
       <c r="D83" s="23" t="inlineStr"/>
       <c r="E83" s="24" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>cable screen</t>
         </is>
       </c>
       <c r="F83" s="25" t="inlineStr">
         <is>
-          <t>ix_ws_front_p</t>
+          <t>cab_aps2</t>
         </is>
       </c>
       <c r="G83" s="26" t="inlineStr">
         <is>
-          <t>FRONT WS INLINE</t>
-        </is>
-      </c>
-      <c r="H83" s="25" t="n">
-        <v>2</v>
-      </c>
+          <t>cable screen (one end only)</t>
+        </is>
+      </c>
+      <c r="H83" s="25" t="inlineStr"/>
       <c r="I83" s="26" t="inlineStr">
         <is>
-          <t>VRC-F GND</t>
+          <t>Pedal 2 cable shield</t>
         </is>
       </c>
       <c r="J83" s="26" t="inlineStr"/>
@@ -10833,59 +10827,57 @@
       </c>
       <c r="L83" s="28" t="inlineStr">
         <is>
-          <t>sp_gndout</t>
+          <t>sp_shield_a_aps</t>
         </is>
       </c>
       <c r="M83" s="29" t="inlineStr">
         <is>
-          <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
+          <t>splice sp_shield_a_aps (SP-SHIELD-A-APS)</t>
         </is>
       </c>
       <c r="N83" s="28" t="inlineStr"/>
       <c r="O83" s="29" t="inlineStr">
         <is>
-          <t>VRC-F GND</t>
+          <t>Pedal 2 cable shield</t>
         </is>
       </c>
       <c r="P83" s="29" t="inlineStr"/>
       <c r="Q83" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A24</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R83" s="31" t="inlineStr">
         <is>
-          <t>Sensor GND (ECU-A A24)</t>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
         </is>
       </c>
       <c r="S83" s="32" t="inlineStr">
         <is>
-          <t>sp_gndout</t>
+          <t>sp_shield_a_aps</t>
         </is>
       </c>
       <c r="T83" s="32" t="inlineStr">
         <is>
-          <t>cab_fspur</t>
-        </is>
-      </c>
-      <c r="U83" s="33" t="n">
-        <v>20</v>
-      </c>
+          <t>cab_aps2</t>
+        </is>
+      </c>
+      <c r="U83" s="33" t="inlineStr"/>
       <c r="V83" s="34" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="W83" s="34" t="inlineStr"/>
       <c r="X83" s="34" t="inlineStr">
         <is>
-          <t>Yellow-Yellow-Blue</t>
+          <t>White-Blue-Yellow</t>
         </is>
       </c>
       <c r="Y83" s="34" t="inlineStr"/>
       <c r="Z83" s="35" t="inlineStr">
         <is>
-          <t>dash branch (front WS inline)</t>
+          <t>at ECU-A plug</t>
         </is>
       </c>
       <c r="AA83" s="36" t="inlineStr"/>
@@ -10894,7 +10886,7 @@
       <c r="AD83" s="38" t="inlineStr"/>
       <c r="AE83" s="38" t="inlineStr">
         <is>
-          <t>splice sp_gndout: node of the wire list (SoT)</t>
+          <t>splice sp_shield_a_aps: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF83" s="38" t="inlineStr">
@@ -10902,17 +10894,21 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG83" s="38" t="inlineStr"/>
+      <c r="AG83" s="38" t="inlineStr">
+        <is>
+          <t>screen floats at the far end; pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="39" t="inlineStr">
         <is>
-          <t>WSSF</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="B84" s="39" t="inlineStr">
         <is>
-          <t>cab_fspur_l</t>
+          <t>cab_fspur_5v</t>
         </is>
       </c>
       <c r="C84" s="39" t="inlineStr">
@@ -10937,51 +10933,51 @@
         </is>
       </c>
       <c r="H84" s="41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I84" s="42" t="inlineStr">
         <is>
-          <t>FL conditioned out</t>
+          <t>VRC-F +5V</t>
         </is>
       </c>
       <c r="J84" s="42" t="inlineStr"/>
       <c r="K84" s="43" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="L84" s="44" t="inlineStr">
         <is>
-          <t>ecu_a</t>
+          <t>sp_5v</t>
         </is>
       </c>
       <c r="M84" s="45" t="inlineStr">
         <is>
-          <t>ECU-A</t>
-        </is>
-      </c>
-      <c r="N84" s="44" t="inlineStr">
-        <is>
-          <t>A23</t>
-        </is>
-      </c>
+          <t>splice sp_5v (SP-5V-A: +5 V sensor supply)</t>
+        </is>
+      </c>
+      <c r="N84" s="44" t="inlineStr"/>
       <c r="O84" s="45" t="inlineStr">
         <is>
-          <t>FL conditioned out</t>
+          <t>VRC-F +5V</t>
         </is>
       </c>
       <c r="P84" s="45" t="inlineStr"/>
       <c r="Q84" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A23</t>
+          <t>ECU-A.A32</t>
         </is>
       </c>
       <c r="R84" s="47" t="inlineStr">
         <is>
-          <t>FL conditioned out (ECU-A A23)</t>
-        </is>
-      </c>
-      <c r="S84" s="48" t="inlineStr"/>
+          <t>+5V sensor (ECU-A A32)</t>
+        </is>
+      </c>
+      <c r="S84" s="48" t="inlineStr">
+        <is>
+          <t>sp_5v</t>
+        </is>
+      </c>
       <c r="T84" s="48" t="inlineStr">
         <is>
           <t>cab_fspur</t>
@@ -10992,18 +10988,16 @@
       </c>
       <c r="V84" s="50" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="W84" s="50" t="inlineStr"/>
       <c r="X84" s="50" t="inlineStr">
         <is>
-          <t>White-Blue-Blue</t>
-        </is>
-      </c>
-      <c r="Y84" s="50" t="n">
-        <v>330</v>
-      </c>
+          <t>Blue-Blue</t>
+        </is>
+      </c>
+      <c r="Y84" s="50" t="inlineStr"/>
       <c r="Z84" s="51" t="inlineStr">
         <is>
           <t>dash branch (front WS inline)</t>
@@ -11015,7 +11009,7 @@
       <c r="AD84" s="54" t="inlineStr"/>
       <c r="AE84" s="54" t="inlineStr">
         <is>
-          <t>channels.csv ecu_a A23 DI 3 (DI3_WSS_FL)</t>
+          <t>splice sp_5v: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF84" s="54" t="inlineStr">
@@ -11028,12 +11022,12 @@
     <row r="85">
       <c r="A85" s="23" t="inlineStr">
         <is>
-          <t>WSSF</t>
+          <t>SGND</t>
         </is>
       </c>
       <c r="B85" s="23" t="inlineStr">
         <is>
-          <t>cab_fspur_sh</t>
+          <t>cab_fspur_gnd</t>
         </is>
       </c>
       <c r="C85" s="23" t="inlineStr">
@@ -11058,11 +11052,11 @@
         </is>
       </c>
       <c r="H85" s="25" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I85" s="26" t="inlineStr">
         <is>
-          <t>WS-F screen drain</t>
+          <t>VRC-F GND</t>
         </is>
       </c>
       <c r="J85" s="26" t="inlineStr"/>
@@ -11073,34 +11067,34 @@
       </c>
       <c r="L85" s="28" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>sp_gndout</t>
         </is>
       </c>
       <c r="M85" s="29" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
       <c r="N85" s="28" t="inlineStr"/>
       <c r="O85" s="29" t="inlineStr">
         <is>
-          <t>WS-F screen drain</t>
+          <t>VRC-F GND</t>
         </is>
       </c>
       <c r="P85" s="29" t="inlineStr"/>
       <c r="Q85" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A7</t>
+          <t>ECU-A.A24</t>
         </is>
       </c>
       <c r="R85" s="31" t="inlineStr">
         <is>
-          <t>Screen A (ECU A7, SHIELD_A)</t>
+          <t>Sensor GND (ECU-A A24)</t>
         </is>
       </c>
       <c r="S85" s="32" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>sp_gndout</t>
         </is>
       </c>
       <c r="T85" s="32" t="inlineStr">
@@ -11108,16 +11102,18 @@
           <t>cab_fspur</t>
         </is>
       </c>
-      <c r="U85" s="33" t="inlineStr"/>
+      <c r="U85" s="33" t="n">
+        <v>20</v>
+      </c>
       <c r="V85" s="34" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="W85" s="34" t="inlineStr"/>
       <c r="X85" s="34" t="inlineStr">
         <is>
-          <t>White-Blue-Blue</t>
+          <t>Yellow-Yellow-Blue</t>
         </is>
       </c>
       <c r="Y85" s="34" t="inlineStr"/>
@@ -11132,7 +11128,7 @@
       <c r="AD85" s="38" t="inlineStr"/>
       <c r="AE85" s="38" t="inlineStr">
         <is>
-          <t>splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>splice sp_gndout: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF85" s="38" t="inlineStr">
@@ -11150,7 +11146,7 @@
       </c>
       <c r="B86" s="39" t="inlineStr">
         <is>
-          <t>cab_fspur_fr_sh_ac</t>
+          <t>cab_fspur_l</t>
         </is>
       </c>
       <c r="C86" s="39" t="inlineStr">
@@ -11161,72 +11157,76 @@
       <c r="D86" s="39" t="inlineStr"/>
       <c r="E86" s="40" t="inlineStr">
         <is>
-          <t>cable screen</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="F86" s="41" t="inlineStr">
         <is>
-          <t>cab_fspur_fr_ac</t>
+          <t>ix_ws_front_p</t>
         </is>
       </c>
       <c r="G86" s="42" t="inlineStr">
         <is>
-          <t>cable screen (one end only)</t>
-        </is>
-      </c>
-      <c r="H86" s="41" t="inlineStr"/>
+          <t>FRONT WS INLINE</t>
+        </is>
+      </c>
+      <c r="H86" s="41" t="n">
+        <v>3</v>
+      </c>
       <c r="I86" s="42" t="inlineStr">
         <is>
-          <t>FR wheel spd shield</t>
+          <t>FL conditioned out</t>
         </is>
       </c>
       <c r="J86" s="42" t="inlineStr"/>
       <c r="K86" s="43" t="inlineStr">
         <is>
-          <t>splice</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="L86" s="44" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>ecu_a</t>
         </is>
       </c>
       <c r="M86" s="45" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
-        </is>
-      </c>
-      <c r="N86" s="44" t="inlineStr"/>
+          <t>ECU-A</t>
+        </is>
+      </c>
+      <c r="N86" s="44" t="inlineStr">
+        <is>
+          <t>A23</t>
+        </is>
+      </c>
       <c r="O86" s="45" t="inlineStr">
         <is>
-          <t>FR wheel spd shield</t>
+          <t>FL conditioned out</t>
         </is>
       </c>
       <c r="P86" s="45" t="inlineStr"/>
       <c r="Q86" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A7</t>
+          <t>ECU-A.A23</t>
         </is>
       </c>
       <c r="R86" s="47" t="inlineStr">
         <is>
-          <t>Screen A (ECU A7, SHIELD_A)</t>
-        </is>
-      </c>
-      <c r="S86" s="48" t="inlineStr">
-        <is>
-          <t>sp_shield_a</t>
-        </is>
-      </c>
+          <t>FL conditioned out (ECU-A A23)</t>
+        </is>
+      </c>
+      <c r="S86" s="48" t="inlineStr"/>
       <c r="T86" s="48" t="inlineStr">
         <is>
-          <t>cab_fspur_fr_ac</t>
-        </is>
-      </c>
-      <c r="U86" s="49" t="inlineStr"/>
+          <t>cab_fspur</t>
+        </is>
+      </c>
+      <c r="U86" s="49" t="n">
+        <v>20</v>
+      </c>
       <c r="V86" s="50" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="W86" s="50" t="inlineStr"/>
@@ -11235,7 +11235,9 @@
           <t>White-Blue-Blue</t>
         </is>
       </c>
-      <c r="Y86" s="50" t="inlineStr"/>
+      <c r="Y86" s="50" t="n">
+        <v>330</v>
+      </c>
       <c r="Z86" s="51" t="inlineStr">
         <is>
           <t>dash branch (front WS inline)</t>
@@ -11247,7 +11249,7 @@
       <c r="AD86" s="54" t="inlineStr"/>
       <c r="AE86" s="54" t="inlineStr">
         <is>
-          <t>splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>channels.csv ecu_a A23 DI 3 (DI3_WSS_FL)</t>
         </is>
       </c>
       <c r="AF86" s="54" t="inlineStr">
@@ -11255,15 +11257,19 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG86" s="54" t="inlineStr">
-        <is>
-          <t>tied at the A end only; the far (B) end floats, dressed back at the ECU-B plug (no A-B shield bridge)</t>
-        </is>
-      </c>
+      <c r="AG86" s="54" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="23" t="inlineStr"/>
-      <c r="B87" s="23" t="inlineStr"/>
+      <c r="A87" s="23" t="inlineStr">
+        <is>
+          <t>WSSF</t>
+        </is>
+      </c>
+      <c r="B87" s="23" t="inlineStr">
+        <is>
+          <t>cab_fspur_sh</t>
+        </is>
+      </c>
       <c r="C87" s="23" t="inlineStr">
         <is>
           <t>A-cabin</t>
@@ -11277,54 +11283,90 @@
       </c>
       <c r="F87" s="25" t="inlineStr">
         <is>
-          <t>bh_a_fw</t>
+          <t>ix_ws_front_p</t>
         </is>
       </c>
       <c r="G87" s="26" t="inlineStr">
         <is>
-          <t>BULKHEAD</t>
+          <t>FRONT WS INLINE</t>
         </is>
       </c>
       <c r="H87" s="25" t="n">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="I87" s="26" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
+          <t>WS-F screen drain</t>
         </is>
       </c>
       <c r="J87" s="26" t="inlineStr"/>
-      <c r="K87" s="27" t="inlineStr"/>
-      <c r="L87" s="28" t="inlineStr"/>
-      <c r="M87" s="29" t="inlineStr"/>
+      <c r="K87" s="27" t="inlineStr">
+        <is>
+          <t>splice</t>
+        </is>
+      </c>
+      <c r="L87" s="28" t="inlineStr">
+        <is>
+          <t>sp_shield_a_wsf</t>
+        </is>
+      </c>
+      <c r="M87" s="29" t="inlineStr">
+        <is>
+          <t>splice sp_shield_a_wsf (SP-SHIELD-A-WSF)</t>
+        </is>
+      </c>
       <c r="N87" s="28" t="inlineStr"/>
-      <c r="O87" s="29" t="inlineStr"/>
+      <c r="O87" s="29" t="inlineStr">
+        <is>
+          <t>WS-F screen drain</t>
+        </is>
+      </c>
       <c r="P87" s="29" t="inlineStr"/>
       <c r="Q87" s="30" t="inlineStr">
         <is>
-          <t>DRB102.45</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R87" s="31" t="inlineStr">
         <is>
-          <t>spare (DRB102 45)</t>
-        </is>
-      </c>
-      <c r="S87" s="32" t="inlineStr"/>
-      <c r="T87" s="32" t="inlineStr"/>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="S87" s="32" t="inlineStr">
+        <is>
+          <t>sp_shield_a_wsf</t>
+        </is>
+      </c>
+      <c r="T87" s="32" t="inlineStr">
+        <is>
+          <t>cab_fspur</t>
+        </is>
+      </c>
       <c r="U87" s="33" t="inlineStr"/>
-      <c r="V87" s="34" t="inlineStr"/>
+      <c r="V87" s="34" t="inlineStr">
+        <is>
+          <t>Shield</t>
+        </is>
+      </c>
       <c r="W87" s="34" t="inlineStr"/>
-      <c r="X87" s="34" t="inlineStr"/>
+      <c r="X87" s="34" t="inlineStr">
+        <is>
+          <t>White-Blue-Blue</t>
+        </is>
+      </c>
       <c r="Y87" s="34" t="inlineStr"/>
-      <c r="Z87" s="35" t="inlineStr"/>
+      <c r="Z87" s="35" t="inlineStr">
+        <is>
+          <t>dash branch (front WS inline)</t>
+        </is>
+      </c>
       <c r="AA87" s="36" t="inlineStr"/>
       <c r="AB87" s="37" t="inlineStr"/>
       <c r="AC87" s="38" t="inlineStr"/>
       <c r="AD87" s="38" t="inlineStr"/>
       <c r="AE87" s="38" t="inlineStr">
         <is>
-          <t>DRB102 45 = 'spare (size 16) - was the A/C coolant switch signal, deleted (S35)'</t>
+          <t>splice sp_shield_a_wsf: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF87" s="38" t="inlineStr">
@@ -11335,8 +11377,16 @@
       <c r="AG87" s="38" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="39" t="inlineStr"/>
-      <c r="B88" s="39" t="inlineStr"/>
+      <c r="A88" s="39" t="inlineStr">
+        <is>
+          <t>WSSF</t>
+        </is>
+      </c>
+      <c r="B88" s="39" t="inlineStr">
+        <is>
+          <t>cab_fspur_fr_sh_ac</t>
+        </is>
+      </c>
       <c r="C88" s="39" t="inlineStr">
         <is>
           <t>A-cabin</t>
@@ -11345,59 +11395,93 @@
       <c r="D88" s="39" t="inlineStr"/>
       <c r="E88" s="40" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>cable screen</t>
         </is>
       </c>
       <c r="F88" s="41" t="inlineStr">
         <is>
-          <t>bh_a_fw</t>
+          <t>cab_fspur_fr_ac</t>
         </is>
       </c>
       <c r="G88" s="42" t="inlineStr">
         <is>
-          <t>BULKHEAD</t>
-        </is>
-      </c>
-      <c r="H88" s="41" t="n">
-        <v>46</v>
-      </c>
+          <t>cable screen (one end only)</t>
+        </is>
+      </c>
+      <c r="H88" s="41" t="inlineStr"/>
       <c r="I88" s="42" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
+          <t>FR wheel spd shield</t>
         </is>
       </c>
       <c r="J88" s="42" t="inlineStr"/>
-      <c r="K88" s="43" t="inlineStr"/>
-      <c r="L88" s="44" t="inlineStr"/>
-      <c r="M88" s="45" t="inlineStr"/>
+      <c r="K88" s="43" t="inlineStr">
+        <is>
+          <t>splice</t>
+        </is>
+      </c>
+      <c r="L88" s="44" t="inlineStr">
+        <is>
+          <t>sp_shield_a_wsf</t>
+        </is>
+      </c>
+      <c r="M88" s="45" t="inlineStr">
+        <is>
+          <t>splice sp_shield_a_wsf (SP-SHIELD-A-WSF)</t>
+        </is>
+      </c>
       <c r="N88" s="44" t="inlineStr"/>
-      <c r="O88" s="45" t="inlineStr"/>
+      <c r="O88" s="45" t="inlineStr">
+        <is>
+          <t>FR wheel spd shield</t>
+        </is>
+      </c>
       <c r="P88" s="45" t="inlineStr"/>
       <c r="Q88" s="46" t="inlineStr">
         <is>
-          <t>DRB102.46</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R88" s="47" t="inlineStr">
         <is>
-          <t>spare (DRB102 46)</t>
-        </is>
-      </c>
-      <c r="S88" s="48" t="inlineStr"/>
-      <c r="T88" s="48" t="inlineStr"/>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="S88" s="48" t="inlineStr">
+        <is>
+          <t>sp_shield_a_wsf</t>
+        </is>
+      </c>
+      <c r="T88" s="48" t="inlineStr">
+        <is>
+          <t>cab_fspur_fr_ac</t>
+        </is>
+      </c>
       <c r="U88" s="49" t="inlineStr"/>
-      <c r="V88" s="50" t="inlineStr"/>
+      <c r="V88" s="50" t="inlineStr">
+        <is>
+          <t>Shield</t>
+        </is>
+      </c>
       <c r="W88" s="50" t="inlineStr"/>
-      <c r="X88" s="50" t="inlineStr"/>
+      <c r="X88" s="50" t="inlineStr">
+        <is>
+          <t>White-Blue-Blue</t>
+        </is>
+      </c>
       <c r="Y88" s="50" t="inlineStr"/>
-      <c r="Z88" s="51" t="inlineStr"/>
+      <c r="Z88" s="51" t="inlineStr">
+        <is>
+          <t>dash branch (front WS inline)</t>
+        </is>
+      </c>
       <c r="AA88" s="52" t="inlineStr"/>
       <c r="AB88" s="53" t="inlineStr"/>
       <c r="AC88" s="54" t="inlineStr"/>
       <c r="AD88" s="54" t="inlineStr"/>
       <c r="AE88" s="54" t="inlineStr">
         <is>
-          <t>DRB102 46 = 'spare (size 16) - was the A/C coolant switch return, deleted (S35)'</t>
+          <t>splice sp_shield_a_wsf: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF88" s="54" t="inlineStr">
@@ -11405,7 +11489,11 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG88" s="54" t="inlineStr"/>
+      <c r="AG88" s="54" t="inlineStr">
+        <is>
+          <t>tied at the A end only; the far (B) end floats, dressed back at the ECU-B plug (no A-B shield bridge)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="23" t="inlineStr"/>
@@ -11432,7 +11520,7 @@
         </is>
       </c>
       <c r="H89" s="25" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="I89" s="26" t="inlineStr">
         <is>
@@ -11448,12 +11536,12 @@
       <c r="P89" s="29" t="inlineStr"/>
       <c r="Q89" s="30" t="inlineStr">
         <is>
-          <t>DRB102.52</t>
+          <t>DRB102.45</t>
         </is>
       </c>
       <c r="R89" s="31" t="inlineStr">
         <is>
-          <t>spare (DRB102 52)</t>
+          <t>spare (DRB102 45)</t>
         </is>
       </c>
       <c r="S89" s="32" t="inlineStr"/>
@@ -11470,7 +11558,7 @@
       <c r="AD89" s="38" t="inlineStr"/>
       <c r="AE89" s="38" t="inlineStr">
         <is>
-          <t>DRB102 52 = 'spare (size 16)'</t>
+          <t>DRB102 45 = 'spare (size 16) - was the A/C coolant switch signal, deleted (S35)'</t>
         </is>
       </c>
       <c r="AF89" s="38" t="inlineStr">
@@ -11505,7 +11593,7 @@
         </is>
       </c>
       <c r="H90" s="41" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="I90" s="42" t="inlineStr">
         <is>
@@ -11521,12 +11609,12 @@
       <c r="P90" s="45" t="inlineStr"/>
       <c r="Q90" s="46" t="inlineStr">
         <is>
-          <t>DRB102.53</t>
+          <t>DRB102.46</t>
         </is>
       </c>
       <c r="R90" s="47" t="inlineStr">
         <is>
-          <t>spare (DRB102 53)</t>
+          <t>spare (DRB102 46)</t>
         </is>
       </c>
       <c r="S90" s="48" t="inlineStr"/>
@@ -11543,7 +11631,7 @@
       <c r="AD90" s="54" t="inlineStr"/>
       <c r="AE90" s="54" t="inlineStr">
         <is>
-          <t>DRB102 53 = 'spare (size 16)'</t>
+          <t>DRB102 46 = 'spare (size 16) - was the A/C coolant switch return, deleted (S35)'</t>
         </is>
       </c>
       <c r="AF90" s="54" t="inlineStr">
@@ -11578,7 +11666,7 @@
         </is>
       </c>
       <c r="H91" s="25" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="I91" s="26" t="inlineStr">
         <is>
@@ -11594,12 +11682,12 @@
       <c r="P91" s="29" t="inlineStr"/>
       <c r="Q91" s="30" t="inlineStr">
         <is>
-          <t>DRB102.57</t>
+          <t>DRB102.52</t>
         </is>
       </c>
       <c r="R91" s="31" t="inlineStr">
         <is>
-          <t>spare (DRB102 57)</t>
+          <t>spare (DRB102 52)</t>
         </is>
       </c>
       <c r="S91" s="32" t="inlineStr"/>
@@ -11616,7 +11704,7 @@
       <c r="AD91" s="38" t="inlineStr"/>
       <c r="AE91" s="38" t="inlineStr">
         <is>
-          <t>DRB102 57 = 'spare (size 16)'</t>
+          <t>DRB102 52 = 'spare (size 16)'</t>
         </is>
       </c>
       <c r="AF91" s="38" t="inlineStr">
@@ -11651,7 +11739,7 @@
         </is>
       </c>
       <c r="H92" s="41" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I92" s="42" t="inlineStr">
         <is>
@@ -11667,12 +11755,12 @@
       <c r="P92" s="45" t="inlineStr"/>
       <c r="Q92" s="46" t="inlineStr">
         <is>
-          <t>DRB102.58</t>
+          <t>DRB102.53</t>
         </is>
       </c>
       <c r="R92" s="47" t="inlineStr">
         <is>
-          <t>spare (DRB102 58)</t>
+          <t>spare (DRB102 53)</t>
         </is>
       </c>
       <c r="S92" s="48" t="inlineStr"/>
@@ -11689,7 +11777,7 @@
       <c r="AD92" s="54" t="inlineStr"/>
       <c r="AE92" s="54" t="inlineStr">
         <is>
-          <t>DRB102 58 = 'spare (size 16)'</t>
+          <t>DRB102 53 = 'spare (size 16)'</t>
         </is>
       </c>
       <c r="AF92" s="54" t="inlineStr">
@@ -11724,7 +11812,7 @@
         </is>
       </c>
       <c r="H93" s="25" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I93" s="26" t="inlineStr">
         <is>
@@ -11740,12 +11828,12 @@
       <c r="P93" s="29" t="inlineStr"/>
       <c r="Q93" s="30" t="inlineStr">
         <is>
-          <t>DRB102.59</t>
+          <t>DRB102.57</t>
         </is>
       </c>
       <c r="R93" s="31" t="inlineStr">
         <is>
-          <t>spare (DRB102 59)</t>
+          <t>spare (DRB102 57)</t>
         </is>
       </c>
       <c r="S93" s="32" t="inlineStr"/>
@@ -11762,7 +11850,7 @@
       <c r="AD93" s="38" t="inlineStr"/>
       <c r="AE93" s="38" t="inlineStr">
         <is>
-          <t>DRB102 59 = 'spare (size 16)'</t>
+          <t>DRB102 57 = 'spare (size 16)'</t>
         </is>
       </c>
       <c r="AF93" s="38" t="inlineStr">
@@ -11797,7 +11885,7 @@
         </is>
       </c>
       <c r="H94" s="41" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I94" s="42" t="inlineStr">
         <is>
@@ -11813,12 +11901,12 @@
       <c r="P94" s="45" t="inlineStr"/>
       <c r="Q94" s="46" t="inlineStr">
         <is>
-          <t>DRB102.61</t>
+          <t>DRB102.58</t>
         </is>
       </c>
       <c r="R94" s="47" t="inlineStr">
         <is>
-          <t>spare (DRB102 61)</t>
+          <t>spare (DRB102 58)</t>
         </is>
       </c>
       <c r="S94" s="48" t="inlineStr"/>
@@ -11835,7 +11923,7 @@
       <c r="AD94" s="54" t="inlineStr"/>
       <c r="AE94" s="54" t="inlineStr">
         <is>
-          <t>DRB102 61 = 'spare (size 16)'</t>
+          <t>DRB102 58 = 'spare (size 16)'</t>
         </is>
       </c>
       <c r="AF94" s="54" t="inlineStr">
@@ -11861,16 +11949,16 @@
       </c>
       <c r="F95" s="25" t="inlineStr">
         <is>
-          <t>ix_ws_front_p</t>
+          <t>bh_a_fw</t>
         </is>
       </c>
       <c r="G95" s="26" t="inlineStr">
         <is>
-          <t>FRONT WS INLINE</t>
+          <t>BULKHEAD</t>
         </is>
       </c>
       <c r="H95" s="25" t="n">
-        <v>6</v>
+        <v>59</v>
       </c>
       <c r="I95" s="26" t="inlineStr">
         <is>
@@ -11886,12 +11974,12 @@
       <c r="P95" s="29" t="inlineStr"/>
       <c r="Q95" s="30" t="inlineStr">
         <is>
-          <t>ix_ws_front_p.6</t>
+          <t>DRB102.59</t>
         </is>
       </c>
       <c r="R95" s="31" t="inlineStr">
         <is>
-          <t>spare (ix_ws_front_p 6)</t>
+          <t>spare (DRB102 59)</t>
         </is>
       </c>
       <c r="S95" s="32" t="inlineStr"/>
@@ -11906,7 +11994,11 @@
       <c r="AB95" s="37" t="inlineStr"/>
       <c r="AC95" s="38" t="inlineStr"/>
       <c r="AD95" s="38" t="inlineStr"/>
-      <c r="AE95" s="38" t="inlineStr"/>
+      <c r="AE95" s="38" t="inlineStr">
+        <is>
+          <t>DRB102 59 = 'spare (size 16)'</t>
+        </is>
+      </c>
       <c r="AF95" s="38" t="inlineStr">
         <is>
           <t>OK</t>
@@ -11930,16 +12022,16 @@
       </c>
       <c r="F96" s="41" t="inlineStr">
         <is>
-          <t>bus_5v_bha_p</t>
+          <t>bh_a_fw</t>
         </is>
       </c>
       <c r="G96" s="42" t="inlineStr">
         <is>
-          <t>+5V BUS</t>
+          <t>BULKHEAD</t>
         </is>
       </c>
       <c r="H96" s="41" t="n">
-        <v>8</v>
+        <v>61</v>
       </c>
       <c r="I96" s="42" t="inlineStr">
         <is>
@@ -11955,12 +12047,12 @@
       <c r="P96" s="45" t="inlineStr"/>
       <c r="Q96" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A32</t>
+          <t>DRB102.61</t>
         </is>
       </c>
       <c r="R96" s="47" t="inlineStr">
         <is>
-          <t>+5V sensor (ECU-A A32)</t>
+          <t>spare (DRB102 61)</t>
         </is>
       </c>
       <c r="S96" s="48" t="inlineStr"/>
@@ -11975,7 +12067,11 @@
       <c r="AB96" s="53" t="inlineStr"/>
       <c r="AC96" s="54" t="inlineStr"/>
       <c r="AD96" s="54" t="inlineStr"/>
-      <c r="AE96" s="54" t="inlineStr"/>
+      <c r="AE96" s="54" t="inlineStr">
+        <is>
+          <t>DRB102 61 = 'spare (size 16)'</t>
+        </is>
+      </c>
       <c r="AF96" s="54" t="inlineStr">
         <is>
           <t>OK</t>
@@ -11999,16 +12095,16 @@
       </c>
       <c r="F97" s="25" t="inlineStr">
         <is>
-          <t>bus_gnd_bha_p</t>
+          <t>ix_ws_front_p</t>
         </is>
       </c>
       <c r="G97" s="26" t="inlineStr">
         <is>
-          <t>SENSOR GND BUS</t>
+          <t>FRONT WS INLINE</t>
         </is>
       </c>
       <c r="H97" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I97" s="26" t="inlineStr">
         <is>
@@ -12024,12 +12120,12 @@
       <c r="P97" s="29" t="inlineStr"/>
       <c r="Q97" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A24</t>
+          <t>ix_ws_front_p.6</t>
         </is>
       </c>
       <c r="R97" s="31" t="inlineStr">
         <is>
-          <t>Sensor GND (ECU-A A24)</t>
+          <t>spare (ix_ws_front_p 6)</t>
         </is>
       </c>
       <c r="S97" s="32" t="inlineStr"/>
@@ -12068,12 +12164,12 @@
       </c>
       <c r="F98" s="41" t="inlineStr">
         <is>
-          <t>bus_gnd_bha_p</t>
+          <t>bus_5v_bha_p</t>
         </is>
       </c>
       <c r="G98" s="42" t="inlineStr">
         <is>
-          <t>SENSOR GND BUS</t>
+          <t>+5V BUS</t>
         </is>
       </c>
       <c r="H98" s="41" t="n">
@@ -12093,12 +12189,12 @@
       <c r="P98" s="45" t="inlineStr"/>
       <c r="Q98" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A24</t>
+          <t>ECU-A.A32</t>
         </is>
       </c>
       <c r="R98" s="47" t="inlineStr">
         <is>
-          <t>Sensor GND (ECU-A A24)</t>
+          <t>+5V sensor (ECU-A A32)</t>
         </is>
       </c>
       <c r="S98" s="48" t="inlineStr"/>
@@ -12121,8 +12217,146 @@
       </c>
       <c r="AG98" s="54" t="inlineStr"/>
     </row>
+    <row r="99">
+      <c r="A99" s="23" t="inlineStr"/>
+      <c r="B99" s="23" t="inlineStr"/>
+      <c r="C99" s="23" t="inlineStr">
+        <is>
+          <t>A-cabin</t>
+        </is>
+      </c>
+      <c r="D99" s="23" t="inlineStr"/>
+      <c r="E99" s="24" t="inlineStr">
+        <is>
+          <t>connector</t>
+        </is>
+      </c>
+      <c r="F99" s="25" t="inlineStr">
+        <is>
+          <t>bus_gnd_bha_p</t>
+        </is>
+      </c>
+      <c r="G99" s="26" t="inlineStr">
+        <is>
+          <t>SENSOR GND BUS</t>
+        </is>
+      </c>
+      <c r="H99" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="I99" s="26" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="J99" s="26" t="inlineStr"/>
+      <c r="K99" s="27" t="inlineStr"/>
+      <c r="L99" s="28" t="inlineStr"/>
+      <c r="M99" s="29" t="inlineStr"/>
+      <c r="N99" s="28" t="inlineStr"/>
+      <c r="O99" s="29" t="inlineStr"/>
+      <c r="P99" s="29" t="inlineStr"/>
+      <c r="Q99" s="30" t="inlineStr">
+        <is>
+          <t>ECU-A.A24</t>
+        </is>
+      </c>
+      <c r="R99" s="31" t="inlineStr">
+        <is>
+          <t>Sensor GND (ECU-A A24)</t>
+        </is>
+      </c>
+      <c r="S99" s="32" t="inlineStr"/>
+      <c r="T99" s="32" t="inlineStr"/>
+      <c r="U99" s="33" t="inlineStr"/>
+      <c r="V99" s="34" t="inlineStr"/>
+      <c r="W99" s="34" t="inlineStr"/>
+      <c r="X99" s="34" t="inlineStr"/>
+      <c r="Y99" s="34" t="inlineStr"/>
+      <c r="Z99" s="35" t="inlineStr"/>
+      <c r="AA99" s="36" t="inlineStr"/>
+      <c r="AB99" s="37" t="inlineStr"/>
+      <c r="AC99" s="38" t="inlineStr"/>
+      <c r="AD99" s="38" t="inlineStr"/>
+      <c r="AE99" s="38" t="inlineStr"/>
+      <c r="AF99" s="38" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AG99" s="38" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="39" t="inlineStr"/>
+      <c r="B100" s="39" t="inlineStr"/>
+      <c r="C100" s="39" t="inlineStr">
+        <is>
+          <t>A-cabin</t>
+        </is>
+      </c>
+      <c r="D100" s="39" t="inlineStr"/>
+      <c r="E100" s="40" t="inlineStr">
+        <is>
+          <t>connector</t>
+        </is>
+      </c>
+      <c r="F100" s="41" t="inlineStr">
+        <is>
+          <t>bus_gnd_bha_p</t>
+        </is>
+      </c>
+      <c r="G100" s="42" t="inlineStr">
+        <is>
+          <t>SENSOR GND BUS</t>
+        </is>
+      </c>
+      <c r="H100" s="41" t="n">
+        <v>8</v>
+      </c>
+      <c r="I100" s="42" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="J100" s="42" t="inlineStr"/>
+      <c r="K100" s="43" t="inlineStr"/>
+      <c r="L100" s="44" t="inlineStr"/>
+      <c r="M100" s="45" t="inlineStr"/>
+      <c r="N100" s="44" t="inlineStr"/>
+      <c r="O100" s="45" t="inlineStr"/>
+      <c r="P100" s="45" t="inlineStr"/>
+      <c r="Q100" s="46" t="inlineStr">
+        <is>
+          <t>ECU-A.A24</t>
+        </is>
+      </c>
+      <c r="R100" s="47" t="inlineStr">
+        <is>
+          <t>Sensor GND (ECU-A A24)</t>
+        </is>
+      </c>
+      <c r="S100" s="48" t="inlineStr"/>
+      <c r="T100" s="48" t="inlineStr"/>
+      <c r="U100" s="49" t="inlineStr"/>
+      <c r="V100" s="50" t="inlineStr"/>
+      <c r="W100" s="50" t="inlineStr"/>
+      <c r="X100" s="50" t="inlineStr"/>
+      <c r="Y100" s="50" t="inlineStr"/>
+      <c r="Z100" s="51" t="inlineStr"/>
+      <c r="AA100" s="52" t="inlineStr"/>
+      <c r="AB100" s="53" t="inlineStr"/>
+      <c r="AC100" s="54" t="inlineStr"/>
+      <c r="AD100" s="54" t="inlineStr"/>
+      <c r="AE100" s="54" t="inlineStr"/>
+      <c r="AF100" s="54" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AG100" s="54" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AG98"/>
+  <autoFilter ref="A2:AG100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -12134,16 +12368,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
@@ -12414,18 +12648,18 @@
         </is>
       </c>
       <c r="F5" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="32" t="inlineStr">
+        <is>
+          <t>20+20+20+20+20+20+20+20</t>
+        </is>
+      </c>
+      <c r="H5" s="32" t="n">
+        <v>8176</v>
+      </c>
+      <c r="I5" s="32" t="n">
         <v>10</v>
-      </c>
-      <c r="G5" s="32" t="inlineStr">
-        <is>
-          <t>20+20+20+20+20+20 + shield</t>
-        </is>
-      </c>
-      <c r="H5" s="32" t="n">
-        <v>6132</v>
-      </c>
-      <c r="I5" s="32" t="n">
-        <v>12</v>
       </c>
       <c r="J5" s="56" t="inlineStr">
         <is>
@@ -12835,8 +13069,120 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>sp_shield_a_aps</t>
+        </is>
+      </c>
+      <c r="B13" s="55" t="inlineStr">
+        <is>
+          <t>At the pedal branch - SP-SHIELD-A-APS: pedal drains</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>A-cabin</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>ECU-A.A7</t>
+        </is>
+      </c>
+      <c r="E13" s="31" t="inlineStr">
+        <is>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="F13" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" s="32" t="inlineStr">
+        <is>
+          <t>20 + shield</t>
+        </is>
+      </c>
+      <c r="H13" s="32" t="n">
+        <v>1022</v>
+      </c>
+      <c r="I13" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="J13" s="56" t="inlineStr">
+        <is>
+          <t>SPLICE, SOLDERED, ADHESIVE HEATSHRINK OVER</t>
+        </is>
+      </c>
+      <c r="K13" s="36" t="inlineStr">
+        <is>
+          <t>At the pedal branch (layout node bp_960)</t>
+        </is>
+      </c>
+      <c r="L13" s="38" t="inlineStr">
+        <is>
+          <t>node of the wire list (SoT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="39" t="inlineStr">
+        <is>
+          <t>sp_shield_a_wsf</t>
+        </is>
+      </c>
+      <c r="B14" s="57" t="inlineStr">
+        <is>
+          <t>At the front WS inline - SP-SHIELD-A-WSF: front wheel-speed drains</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="inlineStr">
+        <is>
+          <t>A-cabin</t>
+        </is>
+      </c>
+      <c r="D14" s="46" t="inlineStr">
+        <is>
+          <t>ECU-A.A7</t>
+        </is>
+      </c>
+      <c r="E14" s="47" t="inlineStr">
+        <is>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="F14" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="48" t="inlineStr">
+        <is>
+          <t>20 + shield</t>
+        </is>
+      </c>
+      <c r="H14" s="48" t="n">
+        <v>1022</v>
+      </c>
+      <c r="I14" s="48" t="n">
+        <v>20</v>
+      </c>
+      <c r="J14" s="58" t="inlineStr">
+        <is>
+          <t>SPLICE, SOLDERED, ADHESIVE HEATSHRINK OVER</t>
+        </is>
+      </c>
+      <c r="K14" s="52" t="inlineStr">
+        <is>
+          <t>At the front WS inline (layout node bp_1020)</t>
+        </is>
+      </c>
+      <c r="L14" s="54" t="inlineStr">
+        <is>
+          <t>node of the wire list (SoT)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L12"/>
+  <autoFilter ref="A2:L14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Shield branch-point rule (R207 addendum): pedal and wheel-speed drains join at their own branch splice (#347)
sp_shield_a_aps, sp_shield_a_wsf, sp_shield_b_wsr; bulkhead devices keep own pins straight to the ECU splice; audit_shields S5.

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-wirelist.xlsx
+++ b/docs/harness/wirelist/A-cabin-wirelist.xlsx
@@ -13,9 +13,9 @@
     <sheet name="Mates" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wire list'!$A$2:$AG$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wire list'!$A$2:$AG$100</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Wire list'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Splices'!$A$2:$L$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Splices'!$A$2:$L$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Splices'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Connectors'!$A$2:$G$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Connectors'!$1:$2</definedName>
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AG98"/>
+  <dimension ref="A1:AG100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -759,14 +759,14 @@
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="36" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="36" customWidth="1" min="16" max="16"/>
     <col width="45" customWidth="1" min="17" max="17"/>
     <col width="32" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
     <col width="18" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="9" customWidth="1" min="22" max="22"/>
@@ -8014,12 +8014,12 @@
     <row r="61">
       <c r="A61" s="23" t="inlineStr">
         <is>
-          <t>CRANKC</t>
+          <t>SHLD</t>
         </is>
       </c>
       <c r="B61" s="23" t="inlineStr">
         <is>
-          <t>w_shc_crank</t>
+          <t>w_shd_a_aps</t>
         </is>
       </c>
       <c r="C61" s="23" t="inlineStr">
@@ -8030,25 +8030,23 @@
       <c r="D61" s="23" t="inlineStr"/>
       <c r="E61" s="24" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="F61" s="25" t="inlineStr">
         <is>
-          <t>bh_a_fw</t>
+          <t>sp_shield_a_aps</t>
         </is>
       </c>
       <c r="G61" s="26" t="inlineStr">
         <is>
-          <t>BULKHEAD</t>
-        </is>
-      </c>
-      <c r="H61" s="25" t="n">
-        <v>11</v>
-      </c>
+          <t>splice sp_shield_a_aps (SP-SHIELD-A-APS)</t>
+        </is>
+      </c>
+      <c r="H61" s="25" t="inlineStr"/>
       <c r="I61" s="26" t="inlineStr">
         <is>
-          <t>Crank sensor shield</t>
+          <t>Shield drain</t>
         </is>
       </c>
       <c r="J61" s="26" t="inlineStr"/>
@@ -8064,13 +8062,13 @@
       </c>
       <c r="M61" s="29" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>splice sp_shield_a (SP-SHIELD-A)</t>
         </is>
       </c>
       <c r="N61" s="28" t="inlineStr"/>
       <c r="O61" s="29" t="inlineStr">
         <is>
-          <t>Crank sensor shield</t>
+          <t>Shield drain</t>
         </is>
       </c>
       <c r="P61" s="29" t="inlineStr"/>
@@ -8105,22 +8103,18 @@
       </c>
       <c r="X61" s="34" t="inlineStr">
         <is>
-          <t>White-Blue-White</t>
+          <t>White-Yellow-Blue</t>
         </is>
       </c>
       <c r="Y61" s="34" t="inlineStr"/>
-      <c r="Z61" s="35" t="inlineStr">
-        <is>
-          <t>trunk ECU-A to bulkhead (RH firewall)</t>
-        </is>
-      </c>
+      <c r="Z61" s="35" t="inlineStr"/>
       <c r="AA61" s="36" t="inlineStr"/>
       <c r="AB61" s="37" t="inlineStr"/>
       <c r="AC61" s="38" t="inlineStr"/>
       <c r="AD61" s="38" t="inlineStr"/>
       <c r="AE61" s="38" t="inlineStr">
         <is>
-          <t>DRB102 11 = section A c33 'Crank VR screen'; splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>splice sp_shield_a_aps: node of the wire list (SoT); splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF61" s="38" t="inlineStr">
@@ -8130,19 +8124,19 @@
       </c>
       <c r="AG61" s="38" t="inlineStr">
         <is>
-          <t>build (R30): this drain is the one crimped into A7</t>
+          <t>branch-point join (R207): the device drain meets the loom shield trunk where its signal wires join the main loom, then runs to the ECU splice</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="39" t="inlineStr">
         <is>
-          <t>CAM</t>
+          <t>SHLD</t>
         </is>
       </c>
       <c r="B62" s="39" t="inlineStr">
         <is>
-          <t>w_shc_cam</t>
+          <t>w_shd_a_wsf</t>
         </is>
       </c>
       <c r="C62" s="39" t="inlineStr">
@@ -8153,25 +8147,23 @@
       <c r="D62" s="39" t="inlineStr"/>
       <c r="E62" s="40" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="F62" s="41" t="inlineStr">
         <is>
-          <t>bh_a_fw</t>
+          <t>sp_shield_a_wsf</t>
         </is>
       </c>
       <c r="G62" s="42" t="inlineStr">
         <is>
-          <t>BULKHEAD</t>
-        </is>
-      </c>
-      <c r="H62" s="41" t="n">
-        <v>15</v>
-      </c>
+          <t>splice sp_shield_a_wsf (SP-SHIELD-A-WSF)</t>
+        </is>
+      </c>
+      <c r="H62" s="41" t="inlineStr"/>
       <c r="I62" s="42" t="inlineStr">
         <is>
-          <t>Cam sensor shield</t>
+          <t>Shield drain</t>
         </is>
       </c>
       <c r="J62" s="42" t="inlineStr"/>
@@ -8187,13 +8179,13 @@
       </c>
       <c r="M62" s="45" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>splice sp_shield_a (SP-SHIELD-A)</t>
         </is>
       </c>
       <c r="N62" s="44" t="inlineStr"/>
       <c r="O62" s="45" t="inlineStr">
         <is>
-          <t>Cam sensor shield</t>
+          <t>Shield drain</t>
         </is>
       </c>
       <c r="P62" s="45" t="inlineStr"/>
@@ -8228,22 +8220,18 @@
       </c>
       <c r="X62" s="50" t="inlineStr">
         <is>
-          <t>Yellow-Yellow</t>
+          <t>White-Yellow-Blue</t>
         </is>
       </c>
       <c r="Y62" s="50" t="inlineStr"/>
-      <c r="Z62" s="51" t="inlineStr">
-        <is>
-          <t>trunk ECU-A to bulkhead (RH firewall)</t>
-        </is>
-      </c>
+      <c r="Z62" s="51" t="inlineStr"/>
       <c r="AA62" s="52" t="inlineStr"/>
       <c r="AB62" s="53" t="inlineStr"/>
       <c r="AC62" s="54" t="inlineStr"/>
       <c r="AD62" s="54" t="inlineStr"/>
       <c r="AE62" s="54" t="inlineStr">
         <is>
-          <t>DRB102 15 = section A c34 'Cam Hall screen'; splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>splice sp_shield_a_wsf: node of the wire list (SoT); splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF62" s="54" t="inlineStr">
@@ -8251,17 +8239,21 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG62" s="54" t="inlineStr"/>
+      <c r="AG62" s="54" t="inlineStr">
+        <is>
+          <t>branch-point join (R207): the device drain meets the loom shield trunk where its signal wires join the main loom, then runs to the ECU splice</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="23" t="inlineStr">
         <is>
-          <t>TURBO</t>
+          <t>CRANKC</t>
         </is>
       </c>
       <c r="B63" s="23" t="inlineStr">
         <is>
-          <t>w_shc_turbo</t>
+          <t>w_shc_crank</t>
         </is>
       </c>
       <c r="C63" s="23" t="inlineStr">
@@ -8286,11 +8278,11 @@
         </is>
       </c>
       <c r="H63" s="25" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="I63" s="26" t="inlineStr">
         <is>
-          <t>Turbo speed shield</t>
+          <t>Crank sensor shield</t>
         </is>
       </c>
       <c r="J63" s="26" t="inlineStr"/>
@@ -8312,7 +8304,7 @@
       <c r="N63" s="28" t="inlineStr"/>
       <c r="O63" s="29" t="inlineStr">
         <is>
-          <t>Turbo speed shield</t>
+          <t>Crank sensor shield</t>
         </is>
       </c>
       <c r="P63" s="29" t="inlineStr"/>
@@ -8347,7 +8339,7 @@
       </c>
       <c r="X63" s="34" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>White-Blue-White</t>
         </is>
       </c>
       <c r="Y63" s="34" t="inlineStr"/>
@@ -8362,7 +8354,7 @@
       <c r="AD63" s="38" t="inlineStr"/>
       <c r="AE63" s="38" t="inlineStr">
         <is>
-          <t>DRB102 19 = section A c6 'Turbo speed screen (to A7)'; splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>DRB102 11 = section A c33 'Crank VR screen'; splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF63" s="38" t="inlineStr">
@@ -8370,17 +8362,21 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG63" s="38" t="inlineStr"/>
+      <c r="AG63" s="38" t="inlineStr">
+        <is>
+          <t>build (R30): this drain is the one crimped into A7</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="39" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>CAM</t>
         </is>
       </c>
       <c r="B64" s="39" t="inlineStr">
         <is>
-          <t>w_shc_flex</t>
+          <t>w_shc_cam</t>
         </is>
       </c>
       <c r="C64" s="39" t="inlineStr">
@@ -8405,11 +8401,11 @@
         </is>
       </c>
       <c r="H64" s="41" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="I64" s="42" t="inlineStr">
         <is>
-          <t>Flex fuel shield</t>
+          <t>Cam sensor shield</t>
         </is>
       </c>
       <c r="J64" s="42" t="inlineStr"/>
@@ -8431,7 +8427,7 @@
       <c r="N64" s="44" t="inlineStr"/>
       <c r="O64" s="45" t="inlineStr">
         <is>
-          <t>Flex fuel shield</t>
+          <t>Cam sensor shield</t>
         </is>
       </c>
       <c r="P64" s="45" t="inlineStr"/>
@@ -8466,7 +8462,7 @@
       </c>
       <c r="X64" s="50" t="inlineStr">
         <is>
-          <t>White-Blue</t>
+          <t>Yellow-Yellow</t>
         </is>
       </c>
       <c r="Y64" s="50" t="inlineStr"/>
@@ -8481,7 +8477,7 @@
       <c r="AD64" s="54" t="inlineStr"/>
       <c r="AE64" s="54" t="inlineStr">
         <is>
-          <t>DRB102 22 = section A c10 'Flex fuel screen (to A7)'; splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>DRB102 15 = section A c34 'Cam Hall screen'; splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF64" s="54" t="inlineStr">
@@ -8494,12 +8490,12 @@
     <row r="65">
       <c r="A65" s="23" t="inlineStr">
         <is>
-          <t>ETBS</t>
+          <t>TURBO</t>
         </is>
       </c>
       <c r="B65" s="23" t="inlineStr">
         <is>
-          <t>w_shc_etbs</t>
+          <t>w_shc_turbo</t>
         </is>
       </c>
       <c r="C65" s="23" t="inlineStr">
@@ -8524,11 +8520,11 @@
         </is>
       </c>
       <c r="H65" s="25" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="I65" s="26" t="inlineStr">
         <is>
-          <t>Throttle shield</t>
+          <t>Turbo speed shield</t>
         </is>
       </c>
       <c r="J65" s="26" t="inlineStr"/>
@@ -8550,7 +8546,7 @@
       <c r="N65" s="28" t="inlineStr"/>
       <c r="O65" s="29" t="inlineStr">
         <is>
-          <t>Throttle shield</t>
+          <t>Turbo speed shield</t>
         </is>
       </c>
       <c r="P65" s="29" t="inlineStr"/>
@@ -8585,7 +8581,7 @@
       </c>
       <c r="X65" s="34" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>White</t>
         </is>
       </c>
       <c r="Y65" s="34" t="inlineStr"/>
@@ -8600,7 +8596,7 @@
       <c r="AD65" s="38" t="inlineStr"/>
       <c r="AE65" s="38" t="inlineStr">
         <is>
-          <t>DRB102 27 = section A c11 'ETB sensor group screen (to A7)'; splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>DRB102 19 = section A c6 'Turbo speed screen (to A7)'; splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF65" s="38" t="inlineStr">
@@ -8613,12 +8609,12 @@
     <row r="66">
       <c r="A66" s="39" t="inlineStr">
         <is>
-          <t>FP</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B66" s="39" t="inlineStr">
         <is>
-          <t>w_fp85</t>
+          <t>w_shc_flex</t>
         </is>
       </c>
       <c r="C66" s="39" t="inlineStr">
@@ -8626,11 +8622,7 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D66" s="39" t="inlineStr">
-        <is>
-          <t>HeavyDC</t>
-        </is>
-      </c>
+      <c r="D66" s="39" t="inlineStr"/>
       <c r="E66" s="40" t="inlineStr">
         <is>
           <t>connector</t>
@@ -8638,85 +8630,83 @@
       </c>
       <c r="F66" s="41" t="inlineStr">
         <is>
-          <t>k_fp</t>
+          <t>bh_a_fw</t>
         </is>
       </c>
       <c r="G66" s="42" t="inlineStr">
         <is>
-          <t>FP RELAY K1</t>
+          <t>BULKHEAD</t>
         </is>
       </c>
       <c r="H66" s="41" t="n">
-        <v>85</v>
+        <v>22</v>
       </c>
       <c r="I66" s="42" t="inlineStr">
         <is>
-          <t>Fuel pump relay (-)</t>
-        </is>
-      </c>
-      <c r="J66" s="42" t="inlineStr">
-        <is>
-          <t>Battery relay block (trunk) relay K1 fuel pump, pin 85</t>
-        </is>
-      </c>
+          <t>Flex fuel shield</t>
+        </is>
+      </c>
+      <c r="J66" s="42" t="inlineStr"/>
       <c r="K66" s="43" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="L66" s="44" t="inlineStr">
         <is>
-          <t>ecu_a</t>
+          <t>sp_shield_a</t>
         </is>
       </c>
       <c r="M66" s="45" t="inlineStr">
         <is>
-          <t>ECU-A</t>
-        </is>
-      </c>
-      <c r="N66" s="44" t="inlineStr">
-        <is>
-          <t>A19</t>
-        </is>
-      </c>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+        </is>
+      </c>
+      <c r="N66" s="44" t="inlineStr"/>
       <c r="O66" s="45" t="inlineStr">
         <is>
-          <t>Fuel pump relay (-)</t>
+          <t>Flex fuel shield</t>
         </is>
       </c>
       <c r="P66" s="45" t="inlineStr"/>
       <c r="Q66" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A19</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R66" s="47" t="inlineStr">
         <is>
-          <t>Fuel pump relay (-) (ECU-A A19)</t>
-        </is>
-      </c>
-      <c r="S66" s="48" t="inlineStr"/>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="S66" s="48" t="inlineStr">
+        <is>
+          <t>sp_shield_a</t>
+        </is>
+      </c>
       <c r="T66" s="48" t="inlineStr"/>
       <c r="U66" s="49" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="V66" s="50" t="inlineStr">
         <is>
-          <t>White</t>
-        </is>
-      </c>
-      <c r="W66" s="50" t="inlineStr"/>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="W66" s="50" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
       <c r="X66" s="50" t="inlineStr">
         <is>
-          <t>White-White-Blue</t>
-        </is>
-      </c>
-      <c r="Y66" s="50" t="n">
-        <v>390</v>
-      </c>
+          <t>White-Blue</t>
+        </is>
+      </c>
+      <c r="Y66" s="50" t="inlineStr"/>
       <c r="Z66" s="51" t="inlineStr">
         <is>
-          <t>glove-box branch (POWER / LOGIC boxes)</t>
+          <t>trunk ECU-A to bulkhead (RH firewall)</t>
         </is>
       </c>
       <c r="AA66" s="52" t="inlineStr"/>
@@ -8725,7 +8715,7 @@
       <c r="AD66" s="54" t="inlineStr"/>
       <c r="AE66" s="54" t="inlineStr">
         <is>
-          <t>fuse-box plan k_fp 85 (18 AWG); channels.csv ecu_a A19 Aux 3 (AUX3_FP_RLY)</t>
+          <t>DRB102 22 = section A c10 'Flex fuel screen (to A7)'; splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF66" s="54" t="inlineStr">
@@ -8733,21 +8723,17 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG66" s="54" t="inlineStr">
-        <is>
-          <t>owner proposed: longer half (drawn today as w_fp85 on A-cabin, 390 mm; w_fp85_h on HeavyDC, 150 mm)</t>
-        </is>
-      </c>
+      <c r="AG66" s="54" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="23" t="inlineStr">
         <is>
-          <t>STR</t>
+          <t>ETBS</t>
         </is>
       </c>
       <c r="B67" s="23" t="inlineStr">
         <is>
-          <t>w_str85</t>
+          <t>w_shc_etbs</t>
         </is>
       </c>
       <c r="C67" s="23" t="inlineStr">
@@ -8755,11 +8741,7 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D67" s="23" t="inlineStr">
-        <is>
-          <t>CabinPower</t>
-        </is>
-      </c>
+      <c r="D67" s="23" t="inlineStr"/>
       <c r="E67" s="24" t="inlineStr">
         <is>
           <t>connector</t>
@@ -8767,85 +8749,83 @@
       </c>
       <c r="F67" s="25" t="inlineStr">
         <is>
-          <t>k_str</t>
+          <t>bh_a_fw</t>
         </is>
       </c>
       <c r="G67" s="26" t="inlineStr">
         <is>
-          <t>POWER R3</t>
+          <t>BULKHEAD</t>
         </is>
       </c>
       <c r="H67" s="25" t="n">
-        <v>85</v>
+        <v>27</v>
       </c>
       <c r="I67" s="26" t="inlineStr">
         <is>
-          <t>Start relay coil (-)</t>
-        </is>
-      </c>
-      <c r="J67" s="26" t="inlineStr">
-        <is>
-          <t>POWER box (glove box) relay R3 start, pin 85</t>
-        </is>
-      </c>
+          <t>Throttle shield</t>
+        </is>
+      </c>
+      <c r="J67" s="26" t="inlineStr"/>
       <c r="K67" s="27" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="L67" s="28" t="inlineStr">
         <is>
-          <t>ecu_a</t>
+          <t>sp_shield_a</t>
         </is>
       </c>
       <c r="M67" s="29" t="inlineStr">
         <is>
-          <t>ECU-A</t>
-        </is>
-      </c>
-      <c r="N67" s="28" t="inlineStr">
-        <is>
-          <t>A26</t>
-        </is>
-      </c>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+        </is>
+      </c>
+      <c r="N67" s="28" t="inlineStr"/>
       <c r="O67" s="29" t="inlineStr">
         <is>
-          <t>Start relay coil (-)</t>
+          <t>Throttle shield</t>
         </is>
       </c>
       <c r="P67" s="29" t="inlineStr"/>
       <c r="Q67" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A26</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R67" s="31" t="inlineStr">
         <is>
-          <t>Start relay coil (-) (ECU-A A26)</t>
-        </is>
-      </c>
-      <c r="S67" s="32" t="inlineStr"/>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="S67" s="32" t="inlineStr">
+        <is>
+          <t>sp_shield_a</t>
+        </is>
+      </c>
       <c r="T67" s="32" t="inlineStr"/>
       <c r="U67" s="33" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="V67" s="34" t="inlineStr">
         <is>
-          <t>White</t>
-        </is>
-      </c>
-      <c r="W67" s="34" t="inlineStr"/>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="W67" s="34" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
       <c r="X67" s="34" t="inlineStr">
         <is>
-          <t>White-Yellow</t>
-        </is>
-      </c>
-      <c r="Y67" s="34" t="n">
-        <v>400</v>
-      </c>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="Y67" s="34" t="inlineStr"/>
       <c r="Z67" s="35" t="inlineStr">
         <is>
-          <t>glove-box branch (POWER / LOGIC boxes)</t>
+          <t>trunk ECU-A to bulkhead (RH firewall)</t>
         </is>
       </c>
       <c r="AA67" s="36" t="inlineStr"/>
@@ -8854,7 +8834,7 @@
       <c r="AD67" s="38" t="inlineStr"/>
       <c r="AE67" s="38" t="inlineStr">
         <is>
-          <t>fuse-box plan k_str 85 (18 AWG); channels.csv ecu_a A26 Aux 8 (AUX8_START_RLY)</t>
+          <t>DRB102 27 = section A c11 'ETB sensor group screen (to A7)'; splice sp_shield_a: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF67" s="38" t="inlineStr">
@@ -8862,21 +8842,17 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG67" s="38" t="inlineStr">
-        <is>
-          <t>owner proposed: longer half (drawn today as w_str85 on A-cabin, 400 mm; w_str85_cp on CabinPower, 400 mm)</t>
-        </is>
-      </c>
+      <c r="AG67" s="38" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="39" t="inlineStr">
         <is>
-          <t>FAN</t>
+          <t>FP</t>
         </is>
       </c>
       <c r="B68" s="39" t="inlineStr">
         <is>
-          <t>w_fan85</t>
+          <t>w_fp85</t>
         </is>
       </c>
       <c r="C68" s="39" t="inlineStr">
@@ -8886,7 +8862,7 @@
       </c>
       <c r="D68" s="39" t="inlineStr">
         <is>
-          <t>CabinPower</t>
+          <t>HeavyDC</t>
         </is>
       </c>
       <c r="E68" s="40" t="inlineStr">
@@ -8896,12 +8872,12 @@
       </c>
       <c r="F68" s="41" t="inlineStr">
         <is>
-          <t>k_fan</t>
+          <t>k_fp</t>
         </is>
       </c>
       <c r="G68" s="42" t="inlineStr">
         <is>
-          <t>POWER R4</t>
+          <t>FP RELAY K1</t>
         </is>
       </c>
       <c r="H68" s="41" t="n">
@@ -8909,12 +8885,12 @@
       </c>
       <c r="I68" s="42" t="inlineStr">
         <is>
-          <t>Rad fan relay (-)</t>
+          <t>Fuel pump relay (-)</t>
         </is>
       </c>
       <c r="J68" s="42" t="inlineStr">
         <is>
-          <t>POWER box (glove box) relay R4 radiator fan, pin 85</t>
+          <t>Battery relay block (trunk) relay K1 fuel pump, pin 85</t>
         </is>
       </c>
       <c r="K68" s="43" t="inlineStr">
@@ -8934,23 +8910,23 @@
       </c>
       <c r="N68" s="44" t="inlineStr">
         <is>
-          <t>A29</t>
+          <t>A19</t>
         </is>
       </c>
       <c r="O68" s="45" t="inlineStr">
         <is>
-          <t>Rad fan relay (-)</t>
+          <t>Fuel pump relay (-)</t>
         </is>
       </c>
       <c r="P68" s="45" t="inlineStr"/>
       <c r="Q68" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A29</t>
+          <t>ECU-A.A19</t>
         </is>
       </c>
       <c r="R68" s="47" t="inlineStr">
         <is>
-          <t>Rad fan relay (-) (ECU-A A29)</t>
+          <t>Fuel pump relay (-) (ECU-A A19)</t>
         </is>
       </c>
       <c r="S68" s="48" t="inlineStr"/>
@@ -8966,11 +8942,11 @@
       <c r="W68" s="50" t="inlineStr"/>
       <c r="X68" s="50" t="inlineStr">
         <is>
-          <t>Yellow-White</t>
+          <t>White-White-Blue</t>
         </is>
       </c>
       <c r="Y68" s="50" t="n">
-        <v>410</v>
+        <v>390</v>
       </c>
       <c r="Z68" s="51" t="inlineStr">
         <is>
@@ -8983,7 +8959,7 @@
       <c r="AD68" s="54" t="inlineStr"/>
       <c r="AE68" s="54" t="inlineStr">
         <is>
-          <t>fuse-box plan k_fan 85 (18 AWG); channels.csv ecu_a A29 Aux 5 (AUX5_RAD_FAN)</t>
+          <t>fuse-box plan k_fp 85 (18 AWG); channels.csv ecu_a A19 Aux 3 (AUX3_FP_RLY)</t>
         </is>
       </c>
       <c r="AF68" s="54" t="inlineStr">
@@ -8993,19 +8969,19 @@
       </c>
       <c r="AG68" s="54" t="inlineStr">
         <is>
-          <t>owner proposed: longer half (drawn today as w_fan85 on A-cabin, 410 mm; w_fan85_cp on CabinPower, 400 mm)</t>
+          <t>owner proposed: longer half (drawn today as w_fp85 on A-cabin, 390 mm; w_fp85_h on HeavyDC, 150 mm)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="23" t="inlineStr">
         <is>
-          <t>EPS</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="B69" s="23" t="inlineStr">
         <is>
-          <t>w_eps_rly</t>
+          <t>w_str85</t>
         </is>
       </c>
       <c r="C69" s="23" t="inlineStr">
@@ -9025,12 +9001,12 @@
       </c>
       <c r="F69" s="25" t="inlineStr">
         <is>
-          <t>k_eps</t>
+          <t>k_str</t>
         </is>
       </c>
       <c r="G69" s="26" t="inlineStr">
         <is>
-          <t>EHPS RELAY</t>
+          <t>POWER R3</t>
         </is>
       </c>
       <c r="H69" s="25" t="n">
@@ -9038,12 +9014,12 @@
       </c>
       <c r="I69" s="26" t="inlineStr">
         <is>
-          <t>EHPS relay coil (-)</t>
+          <t>Start relay coil (-)</t>
         </is>
       </c>
       <c r="J69" s="26" t="inlineStr">
         <is>
-          <t>EHPS pump relay (glove box), pin 85</t>
+          <t>POWER box (glove box) relay R3 start, pin 85</t>
         </is>
       </c>
       <c r="K69" s="27" t="inlineStr">
@@ -9053,31 +9029,33 @@
       </c>
       <c r="L69" s="28" t="inlineStr">
         <is>
-          <t>bh_a_fw</t>
+          <t>ecu_a</t>
         </is>
       </c>
       <c r="M69" s="29" t="inlineStr">
         <is>
-          <t>BULKHEAD</t>
-        </is>
-      </c>
-      <c r="N69" s="28" t="n">
-        <v>56</v>
+          <t>ECU-A</t>
+        </is>
+      </c>
+      <c r="N69" s="28" t="inlineStr">
+        <is>
+          <t>A26</t>
+        </is>
       </c>
       <c r="O69" s="29" t="inlineStr">
         <is>
-          <t>EHPS relay coil (-)</t>
+          <t>Start relay coil (-)</t>
         </is>
       </c>
       <c r="P69" s="29" t="inlineStr"/>
       <c r="Q69" s="30" t="inlineStr">
         <is>
-          <t>DRB102.56</t>
+          <t>ECU-A.A26</t>
         </is>
       </c>
       <c r="R69" s="31" t="inlineStr">
         <is>
-          <t>EHPS relay coil (-) (DRB102 56)</t>
+          <t>Start relay coil (-) (ECU-A A26)</t>
         </is>
       </c>
       <c r="S69" s="32" t="inlineStr"/>
@@ -9087,21 +9065,21 @@
       </c>
       <c r="V69" s="34" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W69" s="34" t="inlineStr"/>
       <c r="X69" s="34" t="inlineStr">
         <is>
-          <t>Blue-Blue-Blue</t>
+          <t>White-Yellow</t>
         </is>
       </c>
       <c r="Y69" s="34" t="n">
-        <v>530</v>
+        <v>400</v>
       </c>
       <c r="Z69" s="35" t="inlineStr">
         <is>
-          <t>glove-box branch (POWER / LOGIC boxes) / trunk ECU-A to bulkhead (RH firewall)</t>
+          <t>glove-box branch (POWER / LOGIC boxes)</t>
         </is>
       </c>
       <c r="AA69" s="36" t="inlineStr"/>
@@ -9110,7 +9088,7 @@
       <c r="AD69" s="38" t="inlineStr"/>
       <c r="AE69" s="38" t="inlineStr">
         <is>
-          <t>channels.csv k_eps c2 Coil 85 (MRS_RLY); DRB102 56 = section A c27 'EPS relay coil 85 (R22) - from the MR-S pump B5'</t>
+          <t>fuse-box plan k_str 85 (18 AWG); channels.csv ecu_a A26 Aux 8 (AUX8_START_RLY)</t>
         </is>
       </c>
       <c r="AF69" s="38" t="inlineStr">
@@ -9120,19 +9098,19 @@
       </c>
       <c r="AG69" s="38" t="inlineStr">
         <is>
-          <t>owner proposed: longer half (drawn today as w_eps_rly on A-cabin, 530 mm; w_eps_rly_cp on CabinPower, 400 mm)</t>
+          <t>owner proposed: longer half (drawn today as w_str85 on A-cabin, 400 mm; w_str85_cp on CabinPower, 400 mm)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="39" t="inlineStr">
         <is>
-          <t>ACKILL</t>
+          <t>FAN</t>
         </is>
       </c>
       <c r="B70" s="39" t="inlineStr">
         <is>
-          <t>w_ac_kill</t>
+          <t>w_fan85</t>
         </is>
       </c>
       <c r="C70" s="39" t="inlineStr">
@@ -9140,7 +9118,11 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D70" s="39" t="inlineStr"/>
+      <c r="D70" s="39" t="inlineStr">
+        <is>
+          <t>CabinPower</t>
+        </is>
+      </c>
       <c r="E70" s="40" t="inlineStr">
         <is>
           <t>connector</t>
@@ -9148,110 +9130,94 @@
       </c>
       <c r="F70" s="41" t="inlineStr">
         <is>
+          <t>k_fan</t>
+        </is>
+      </c>
+      <c r="G70" s="42" t="inlineStr">
+        <is>
+          <t>POWER R4</t>
+        </is>
+      </c>
+      <c r="H70" s="41" t="n">
+        <v>85</v>
+      </c>
+      <c r="I70" s="42" t="inlineStr">
+        <is>
+          <t>Rad fan relay (-)</t>
+        </is>
+      </c>
+      <c r="J70" s="42" t="inlineStr">
+        <is>
+          <t>POWER box (glove box) relay R4 radiator fan, pin 85</t>
+        </is>
+      </c>
+      <c r="K70" s="43" t="inlineStr">
+        <is>
+          <t>connector</t>
+        </is>
+      </c>
+      <c r="L70" s="44" t="inlineStr">
+        <is>
           <t>ecu_a</t>
         </is>
       </c>
-      <c r="G70" s="42" t="inlineStr">
+      <c r="M70" s="45" t="inlineStr">
         <is>
           <t>ECU-A</t>
         </is>
       </c>
-      <c r="H70" s="41" t="inlineStr">
-        <is>
-          <t>A18</t>
-        </is>
-      </c>
-      <c r="I70" s="42" t="inlineStr">
-        <is>
-          <t>A/C cancel (ACT)</t>
-        </is>
-      </c>
-      <c r="J70" s="42" t="inlineStr"/>
-      <c r="K70" s="43" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="L70" s="44" t="inlineStr">
-        <is>
-          <t>A18 (factory)</t>
-        </is>
-      </c>
-      <c r="M70" s="45" t="inlineStr">
-        <is>
-          <t>OEM A/C amplifier</t>
-        </is>
-      </c>
-      <c r="N70" s="44" t="n">
-        <v>11</v>
+      <c r="N70" s="44" t="inlineStr">
+        <is>
+          <t>A29</t>
+        </is>
       </c>
       <c r="O70" s="45" t="inlineStr">
         <is>
-          <t>A/C cancel (ACT)</t>
-        </is>
-      </c>
-      <c r="P70" s="45" t="inlineStr">
-        <is>
-          <t>A/C amp A18 pin 11 (1993: A15), behind the glove box. Solder splice onto the factory G-Y lead. EWD 1992 p.93 / p.218; locator 1990 p.17.</t>
-        </is>
-      </c>
+          <t>Rad fan relay (-)</t>
+        </is>
+      </c>
+      <c r="P70" s="45" t="inlineStr"/>
       <c r="Q70" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A18</t>
+          <t>ECU-A.A29</t>
         </is>
       </c>
       <c r="R70" s="47" t="inlineStr">
         <is>
-          <t>A/C cancel (ACT) (ECU-A A18)</t>
+          <t>Rad fan relay (-) (ECU-A A29)</t>
         </is>
       </c>
       <c r="S70" s="48" t="inlineStr"/>
       <c r="T70" s="48" t="inlineStr"/>
       <c r="U70" s="49" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="V70" s="50" t="inlineStr">
         <is>
-          <t>Gray</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W70" s="50" t="inlineStr"/>
       <c r="X70" s="50" t="inlineStr">
         <is>
-          <t>White-Yellow-Yellow</t>
+          <t>Yellow-White</t>
         </is>
       </c>
       <c r="Y70" s="50" t="n">
-        <v>600</v>
+        <v>410</v>
       </c>
       <c r="Z70" s="51" t="inlineStr">
         <is>
-          <t>A/C amp branch (behind dash)</t>
-        </is>
-      </c>
-      <c r="AA70" s="52" t="inlineStr">
-        <is>
-          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD</t>
-        </is>
-      </c>
-      <c r="AB70" s="53" t="inlineStr">
-        <is>
-          <t>G-Y</t>
-        </is>
-      </c>
-      <c r="AC70" s="54" t="inlineStr">
-        <is>
-          <t>1992 Celica EWD132U p.93 and p.218 (docs/electrical/ewd-snips/1992-celica-ewd132u-a17-act-p093.png, 1992-celica-ewd132u-a17-clutch-p218.png); 1990 ST185 book locator A18; 1992 EWD132U p.93 and p.218 (A17-11 = A18-11); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html)</t>
-        </is>
-      </c>
-      <c r="AD70" s="54" t="inlineStr">
-        <is>
-          <t>solder splice onto the factory G-Y ACT lead at the A/C amplifier</t>
-        </is>
-      </c>
+          <t>glove-box branch (POWER / LOGIC boxes)</t>
+        </is>
+      </c>
+      <c r="AA70" s="52" t="inlineStr"/>
+      <c r="AB70" s="53" t="inlineStr"/>
+      <c r="AC70" s="54" t="inlineStr"/>
+      <c r="AD70" s="54" t="inlineStr"/>
       <c r="AE70" s="54" t="inlineStr">
         <is>
-          <t>channels.csv ecu_a A18 Aux 4 (AUX4_AC_KILL); flying lead FL_ACAMP_ACT: EWD A18 pin 11 G-Y</t>
+          <t>fuse-box plan k_fan 85 (18 AWG); channels.csv ecu_a A29 Aux 5 (AUX5_RAD_FAN)</t>
         </is>
       </c>
       <c r="AF70" s="54" t="inlineStr">
@@ -9259,17 +9225,21 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG70" s="54" t="inlineStr"/>
+      <c r="AG70" s="54" t="inlineStr">
+        <is>
+          <t>owner proposed: longer half (drawn today as w_fan85 on A-cabin, 410 mm; w_fan85_cp on CabinPower, 400 mm)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="23" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>EPS</t>
         </is>
       </c>
       <c r="B71" s="23" t="inlineStr">
         <is>
-          <t>w_ac_psw_in</t>
+          <t>w_eps_rly</t>
         </is>
       </c>
       <c r="C71" s="23" t="inlineStr">
@@ -9279,122 +9249,102 @@
       </c>
       <c r="D71" s="23" t="inlineStr">
         <is>
-          <t>EngineRoom-C</t>
+          <t>CabinPower</t>
         </is>
       </c>
       <c r="E71" s="24" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="F71" s="25" t="inlineStr">
         <is>
-          <t>A5 (factory)</t>
+          <t>k_eps</t>
         </is>
       </c>
       <c r="G71" s="26" t="inlineStr">
         <is>
-          <t>OEM A5, factory Y-R lead</t>
+          <t>EHPS RELAY</t>
         </is>
       </c>
       <c r="H71" s="25" t="n">
-        <v>4</v>
+        <v>85</v>
       </c>
       <c r="I71" s="26" t="inlineStr">
         <is>
-          <t>A/C pressure sw out</t>
+          <t>EHPS relay coil (-)</t>
         </is>
       </c>
       <c r="J71" s="26" t="inlineStr">
         <is>
-          <t>Runs on in ST185-EngineRoom-C to A/C pressure switch A5 pin 4 (engine bay): new wire to the switch's own mating plug, plug part TBD. EWD 1990 p.152.</t>
+          <t>EHPS pump relay (glove box), pin 85</t>
         </is>
       </c>
       <c r="K71" s="27" t="inlineStr">
         <is>
-          <t>splice</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="L71" s="28" t="inlineStr">
         <is>
-          <t>sp_ac_psw</t>
+          <t>bh_a_fw</t>
         </is>
       </c>
       <c r="M71" s="29" t="inlineStr">
         <is>
-          <t>splice sp_ac_psw (SP-AC-PSW: A/C pressure switch output)</t>
-        </is>
-      </c>
-      <c r="N71" s="28" t="inlineStr"/>
+          <t>BULKHEAD</t>
+        </is>
+      </c>
+      <c r="N71" s="28" t="n">
+        <v>56</v>
+      </c>
       <c r="O71" s="29" t="inlineStr">
         <is>
-          <t>A/C pressure sw out</t>
+          <t>EHPS relay coil (-)</t>
         </is>
       </c>
       <c r="P71" s="29" t="inlineStr"/>
       <c r="Q71" s="30" t="inlineStr">
         <is>
-          <t>A5.4</t>
+          <t>DRB102.56</t>
         </is>
       </c>
       <c r="R71" s="31" t="inlineStr">
         <is>
-          <t>A/C pressure-switched relay coil +</t>
-        </is>
-      </c>
-      <c r="S71" s="32" t="inlineStr">
-        <is>
-          <t>sp_ac_psw</t>
-        </is>
-      </c>
+          <t>EHPS relay coil (-) (DRB102 56)</t>
+        </is>
+      </c>
+      <c r="S71" s="32" t="inlineStr"/>
       <c r="T71" s="32" t="inlineStr"/>
       <c r="U71" s="33" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="V71" s="34" t="inlineStr">
         <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="W71" s="34" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
+          <t>Violet</t>
+        </is>
+      </c>
+      <c r="W71" s="34" t="inlineStr"/>
       <c r="X71" s="34" t="inlineStr">
         <is>
-          <t>Yellow-Blue</t>
-        </is>
-      </c>
-      <c r="Y71" s="34" t="inlineStr"/>
+          <t>Blue-Blue-Blue</t>
+        </is>
+      </c>
+      <c r="Y71" s="34" t="n">
+        <v>530</v>
+      </c>
       <c r="Z71" s="35" t="inlineStr">
         <is>
-          <t>A/C amp branch (behind dash)</t>
-        </is>
-      </c>
-      <c r="AA71" s="36" t="inlineStr">
-        <is>
-          <t>A/C pressure switch A5, engine bay; exact spot TBD (no locator figure in the repo)</t>
-        </is>
-      </c>
-      <c r="AB71" s="37" t="inlineStr">
-        <is>
-          <t>Y-R (factory wiring; new wire here)</t>
-        </is>
-      </c>
-      <c r="AC71" s="38" t="inlineStr">
-        <is>
-          <t>1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1990 ST185 EWD p.152 (A5 pin 4 Y-R)</t>
-        </is>
-      </c>
-      <c r="AD71" s="38" t="inlineStr">
-        <is>
-          <t>new-wire run terminated at the switch's own mating plug (no factory engine-bay wire reused, Section 39, 2026-10-04); plug part number not yet chosen</t>
-        </is>
-      </c>
+          <t>glove-box branch (POWER / LOGIC boxes) / trunk ECU-A to bulkhead (RH firewall)</t>
+        </is>
+      </c>
+      <c r="AA71" s="36" t="inlineStr"/>
+      <c r="AB71" s="37" t="inlineStr"/>
+      <c r="AC71" s="38" t="inlineStr"/>
+      <c r="AD71" s="38" t="inlineStr"/>
       <c r="AE71" s="38" t="inlineStr">
         <is>
-          <t>flying lead FL_A5_4: EWD A5 pin 4 Y-R (factory wiring; new wire here); splice sp_ac_psw: node of the wire list (SoT)</t>
+          <t>channels.csv k_eps c2 Coil 85 (MRS_RLY); DRB102 56 = section A c27 'EPS relay coil 85 (R22) - from the MR-S pump B5'</t>
         </is>
       </c>
       <c r="AF71" s="38" t="inlineStr">
@@ -9404,19 +9354,19 @@
       </c>
       <c r="AG71" s="38" t="inlineStr">
         <is>
-          <t>owner TBD: a half has no length estimate (drawn today as w_ac_psw_in on A-cabin, ? mm; w_ac_psw on EngineRoom-C, 100 mm)</t>
+          <t>owner proposed: longer half (drawn today as w_eps_rly on A-cabin, 530 mm; w_eps_rly_cp on CabinPower, 400 mm)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="39" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>ACKILL</t>
         </is>
       </c>
       <c r="B72" s="39" t="inlineStr">
         <is>
-          <t>w_ac_psw_sw</t>
+          <t>w_ac_kill</t>
         </is>
       </c>
       <c r="C72" s="39" t="inlineStr">
@@ -9427,89 +9377,87 @@
       <c r="D72" s="39" t="inlineStr"/>
       <c r="E72" s="40" t="inlineStr">
         <is>
+          <t>connector</t>
+        </is>
+      </c>
+      <c r="F72" s="41" t="inlineStr">
+        <is>
+          <t>ecu_a</t>
+        </is>
+      </c>
+      <c r="G72" s="42" t="inlineStr">
+        <is>
+          <t>ECU-A</t>
+        </is>
+      </c>
+      <c r="H72" s="41" t="inlineStr">
+        <is>
+          <t>A18</t>
+        </is>
+      </c>
+      <c r="I72" s="42" t="inlineStr">
+        <is>
+          <t>A/C cancel (ACT)</t>
+        </is>
+      </c>
+      <c r="J72" s="42" t="inlineStr"/>
+      <c r="K72" s="43" t="inlineStr">
+        <is>
           <t>OEM</t>
         </is>
       </c>
-      <c r="F72" s="41" t="inlineStr">
+      <c r="L72" s="44" t="inlineStr">
         <is>
           <t>A18 (factory)</t>
         </is>
       </c>
-      <c r="G72" s="42" t="inlineStr">
+      <c r="M72" s="45" t="inlineStr">
         <is>
           <t>OEM A/C amplifier</t>
         </is>
       </c>
-      <c r="H72" s="41" t="n">
-        <v>13</v>
-      </c>
-      <c r="I72" s="42" t="inlineStr">
-        <is>
-          <t>A/C pressure sw out</t>
-        </is>
-      </c>
-      <c r="J72" s="42" t="inlineStr">
-        <is>
-          <t>A/C amp A18 pin 13 (1993: A15), behind the glove box. Solder splice onto the factory Y-R lead. EWD 1990 p.152; locator 1990 p.17.</t>
-        </is>
-      </c>
-      <c r="K72" s="43" t="inlineStr">
-        <is>
-          <t>splice</t>
-        </is>
-      </c>
-      <c r="L72" s="44" t="inlineStr">
-        <is>
-          <t>sp_ac_psw</t>
-        </is>
-      </c>
-      <c r="M72" s="45" t="inlineStr">
-        <is>
-          <t>splice sp_ac_psw (SP-AC-PSW: A/C pressure switch output)</t>
-        </is>
-      </c>
-      <c r="N72" s="44" t="inlineStr"/>
+      <c r="N72" s="44" t="n">
+        <v>11</v>
+      </c>
       <c r="O72" s="45" t="inlineStr">
         <is>
-          <t>A/C pressure sw out</t>
-        </is>
-      </c>
-      <c r="P72" s="45" t="inlineStr"/>
+          <t>A/C cancel (ACT)</t>
+        </is>
+      </c>
+      <c r="P72" s="45" t="inlineStr">
+        <is>
+          <t>A/C amp A18 pin 11 (1993: A15), behind the glove box. Solder splice onto the factory G-Y lead. EWD 1992 p.93 / p.218; locator 1990 p.17.</t>
+        </is>
+      </c>
       <c r="Q72" s="46" t="inlineStr">
         <is>
-          <t>A5.4</t>
+          <t>ECU-A.A18</t>
         </is>
       </c>
       <c r="R72" s="47" t="inlineStr">
         <is>
-          <t>A/C pressure-switched relay coil +</t>
-        </is>
-      </c>
-      <c r="S72" s="48" t="inlineStr">
-        <is>
-          <t>sp_ac_psw</t>
-        </is>
-      </c>
+          <t>A/C cancel (ACT) (ECU-A A18)</t>
+        </is>
+      </c>
+      <c r="S72" s="48" t="inlineStr"/>
       <c r="T72" s="48" t="inlineStr"/>
       <c r="U72" s="49" t="n">
         <v>20</v>
       </c>
       <c r="V72" s="50" t="inlineStr">
         <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="W72" s="50" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
+          <t>Gray</t>
+        </is>
+      </c>
+      <c r="W72" s="50" t="inlineStr"/>
       <c r="X72" s="50" t="inlineStr">
         <is>
-          <t>Yellow-Blue</t>
-        </is>
-      </c>
-      <c r="Y72" s="50" t="inlineStr"/>
+          <t>White-Yellow-Yellow</t>
+        </is>
+      </c>
+      <c r="Y72" s="50" t="n">
+        <v>600</v>
+      </c>
       <c r="Z72" s="51" t="inlineStr">
         <is>
           <t>A/C amp branch (behind dash)</t>
@@ -9522,22 +9470,22 @@
       </c>
       <c r="AB72" s="53" t="inlineStr">
         <is>
-          <t>Y-R</t>
+          <t>G-Y</t>
         </is>
       </c>
       <c r="AC72" s="54" t="inlineStr">
         <is>
-          <t>1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1992 EWD132U p.219 A17-13 (ewd-snips/1992-celica-ewd132u-a17-pressure-p219.png); 1990 ST185 EWD p.152; 1992 EWD132U p.219 (A17-13); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html)</t>
+          <t>1992 Celica EWD132U p.93 and p.218 (docs/electrical/ewd-snips/1992-celica-ewd132u-a17-act-p093.png, 1992-celica-ewd132u-a17-clutch-p218.png); 1990 ST185 book locator A18; 1992 EWD132U p.93 and p.218 (A17-11 = A18-11); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html)</t>
         </is>
       </c>
       <c r="AD72" s="54" t="inlineStr">
         <is>
-          <t>solder splice onto the factory Y-R lead at the A/C amplifier</t>
+          <t>solder splice onto the factory G-Y ACT lead at the A/C amplifier</t>
         </is>
       </c>
       <c r="AE72" s="54" t="inlineStr">
         <is>
-          <t>flying lead FL_ACAMP_PSW: EWD A18 pin 13 Y-R; splice sp_ac_psw: node of the wire list (SoT)</t>
+          <t>channels.csv ecu_a A18 Aux 4 (AUX4_AC_KILL); flying lead FL_ACAMP_ACT: EWD A18 pin 11 G-Y</t>
         </is>
       </c>
       <c r="AF72" s="54" t="inlineStr">
@@ -9555,7 +9503,7 @@
       </c>
       <c r="B73" s="23" t="inlineStr">
         <is>
-          <t>w_acc86</t>
+          <t>w_ac_psw_in</t>
         </is>
       </c>
       <c r="C73" s="23" t="inlineStr">
@@ -9565,59 +9513,59 @@
       </c>
       <c r="D73" s="23" t="inlineStr">
         <is>
-          <t>CabinPower</t>
+          <t>EngineRoom-C</t>
         </is>
       </c>
       <c r="E73" s="24" t="inlineStr">
         <is>
+          <t>OEM</t>
+        </is>
+      </c>
+      <c r="F73" s="25" t="inlineStr">
+        <is>
+          <t>A5 (factory)</t>
+        </is>
+      </c>
+      <c r="G73" s="26" t="inlineStr">
+        <is>
+          <t>OEM A5, factory Y-R lead</t>
+        </is>
+      </c>
+      <c r="H73" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="I73" s="26" t="inlineStr">
+        <is>
+          <t>A/C pressure sw out</t>
+        </is>
+      </c>
+      <c r="J73" s="26" t="inlineStr">
+        <is>
+          <t>Runs on in ST185-EngineRoom-C to A/C pressure switch A5 pin 4 (engine bay): new wire to the switch's own mating plug, plug part TBD. EWD 1990 p.152.</t>
+        </is>
+      </c>
+      <c r="K73" s="27" t="inlineStr">
+        <is>
           <t>splice</t>
         </is>
       </c>
-      <c r="F73" s="25" t="inlineStr">
+      <c r="L73" s="28" t="inlineStr">
         <is>
           <t>sp_ac_psw</t>
         </is>
       </c>
-      <c r="G73" s="26" t="inlineStr">
+      <c r="M73" s="29" t="inlineStr">
         <is>
           <t>splice sp_ac_psw (SP-AC-PSW: A/C pressure switch output)</t>
         </is>
       </c>
-      <c r="H73" s="25" t="inlineStr"/>
-      <c r="I73" s="26" t="inlineStr">
-        <is>
-          <t>A/C clutch relay (+)</t>
-        </is>
-      </c>
-      <c r="J73" s="26" t="inlineStr"/>
-      <c r="K73" s="27" t="inlineStr">
-        <is>
-          <t>connector</t>
-        </is>
-      </c>
-      <c r="L73" s="28" t="inlineStr">
-        <is>
-          <t>k_acc</t>
-        </is>
-      </c>
-      <c r="M73" s="29" t="inlineStr">
-        <is>
-          <t>LOGIC M5</t>
-        </is>
-      </c>
-      <c r="N73" s="28" t="n">
-        <v>86</v>
-      </c>
+      <c r="N73" s="28" t="inlineStr"/>
       <c r="O73" s="29" t="inlineStr">
         <is>
-          <t>A/C clutch relay (+)</t>
-        </is>
-      </c>
-      <c r="P73" s="29" t="inlineStr">
-        <is>
-          <t>LOGIC box (glove box) relay M15 A/C clutch, pin 86</t>
-        </is>
-      </c>
+          <t>A/C pressure sw out</t>
+        </is>
+      </c>
+      <c r="P73" s="29" t="inlineStr"/>
       <c r="Q73" s="30" t="inlineStr">
         <is>
           <t>A5.4</t>
@@ -9635,7 +9583,7 @@
       </c>
       <c r="T73" s="32" t="inlineStr"/>
       <c r="U73" s="33" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="V73" s="34" t="inlineStr">
         <is>
@@ -9658,13 +9606,29 @@
           <t>A/C amp branch (behind dash)</t>
         </is>
       </c>
-      <c r="AA73" s="36" t="inlineStr"/>
-      <c r="AB73" s="37" t="inlineStr"/>
-      <c r="AC73" s="38" t="inlineStr"/>
-      <c r="AD73" s="38" t="inlineStr"/>
+      <c r="AA73" s="36" t="inlineStr">
+        <is>
+          <t>A/C pressure switch A5, engine bay; exact spot TBD (no locator figure in the repo)</t>
+        </is>
+      </c>
+      <c r="AB73" s="37" t="inlineStr">
+        <is>
+          <t>Y-R (factory wiring; new wire here)</t>
+        </is>
+      </c>
+      <c r="AC73" s="38" t="inlineStr">
+        <is>
+          <t>1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1990 ST185 EWD p.152 (A5 pin 4 Y-R)</t>
+        </is>
+      </c>
+      <c r="AD73" s="38" t="inlineStr">
+        <is>
+          <t>new-wire run terminated at the switch's own mating plug (no factory engine-bay wire reused, Section 39, 2026-10-04); plug part number not yet chosen</t>
+        </is>
+      </c>
       <c r="AE73" s="38" t="inlineStr">
         <is>
-          <t>splice sp_ac_psw: node of the wire list (SoT); fuse-box plan k_acc 86 (18 AWG)</t>
+          <t>flying lead FL_A5_4: EWD A5 pin 4 Y-R (factory wiring; new wire here); splice sp_ac_psw: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF73" s="38" t="inlineStr">
@@ -9674,19 +9638,19 @@
       </c>
       <c r="AG73" s="38" t="inlineStr">
         <is>
-          <t>owner TBD: a half has no length estimate (drawn today as w_acc86 on A-cabin, ? mm; w_acc86_cp on CabinPower, 400 mm)</t>
+          <t>owner TBD: a half has no length estimate (drawn today as w_ac_psw_in on A-cabin, ? mm; w_ac_psw on EngineRoom-C, 100 mm)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="39" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="B74" s="39" t="inlineStr">
         <is>
-          <t>w_aps_vc1</t>
+          <t>w_ac_psw_sw</t>
         </is>
       </c>
       <c r="C74" s="39" t="inlineStr">
@@ -9697,28 +9661,32 @@
       <c r="D74" s="39" t="inlineStr"/>
       <c r="E74" s="40" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F74" s="41" t="inlineStr">
         <is>
-          <t>aps</t>
+          <t>A18 (factory)</t>
         </is>
       </c>
       <c r="G74" s="42" t="inlineStr">
         <is>
-          <t>PEDAL</t>
+          <t>OEM A/C amplifier</t>
         </is>
       </c>
       <c r="H74" s="41" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="I74" s="42" t="inlineStr">
         <is>
-          <t>+5 V pedal sensor 1</t>
-        </is>
-      </c>
-      <c r="J74" s="42" t="inlineStr"/>
+          <t>A/C pressure sw out</t>
+        </is>
+      </c>
+      <c r="J74" s="42" t="inlineStr">
+        <is>
+          <t>A/C amp A18 pin 13 (1993: A15), behind the glove box. Solder splice onto the factory Y-R lead. EWD 1990 p.152; locator 1990 p.17.</t>
+        </is>
+      </c>
       <c r="K74" s="43" t="inlineStr">
         <is>
           <t>splice</t>
@@ -9726,68 +9694,84 @@
       </c>
       <c r="L74" s="44" t="inlineStr">
         <is>
-          <t>sp_5v_2</t>
+          <t>sp_ac_psw</t>
         </is>
       </c>
       <c r="M74" s="45" t="inlineStr">
         <is>
-          <t>splice sp_5v_2 (SP-5V-PEDAL: +5 V to pedal + cruise)</t>
+          <t>splice sp_ac_psw (SP-AC-PSW: A/C pressure switch output)</t>
         </is>
       </c>
       <c r="N74" s="44" t="inlineStr"/>
       <c r="O74" s="45" t="inlineStr">
         <is>
-          <t>+5 V pedal sensor 1</t>
+          <t>A/C pressure sw out</t>
         </is>
       </c>
       <c r="P74" s="45" t="inlineStr"/>
       <c r="Q74" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A32</t>
+          <t>A5.4</t>
         </is>
       </c>
       <c r="R74" s="47" t="inlineStr">
         <is>
-          <t>+5V sensor (ECU-A A32)</t>
+          <t>A/C pressure-switched relay coil +</t>
         </is>
       </c>
       <c r="S74" s="48" t="inlineStr">
         <is>
-          <t>sp_5v_2</t>
-        </is>
-      </c>
-      <c r="T74" s="48" t="inlineStr">
-        <is>
-          <t>cab_aps1</t>
-        </is>
-      </c>
+          <t>sp_ac_psw</t>
+        </is>
+      </c>
+      <c r="T74" s="48" t="inlineStr"/>
       <c r="U74" s="49" t="n">
         <v>20</v>
       </c>
       <c r="V74" s="50" t="inlineStr">
         <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="W74" s="50" t="inlineStr">
+        <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="W74" s="50" t="inlineStr"/>
       <c r="X74" s="50" t="inlineStr">
         <is>
-          <t>Blue-Blue</t>
+          <t>Yellow-Blue</t>
         </is>
       </c>
       <c r="Y74" s="50" t="inlineStr"/>
       <c r="Z74" s="51" t="inlineStr">
         <is>
-          <t>pedal branch (driver footwell)</t>
-        </is>
-      </c>
-      <c r="AA74" s="52" t="inlineStr"/>
-      <c r="AB74" s="53" t="inlineStr"/>
-      <c r="AC74" s="54" t="inlineStr"/>
-      <c r="AD74" s="54" t="inlineStr"/>
+          <t>A/C amp branch (behind dash)</t>
+        </is>
+      </c>
+      <c r="AA74" s="52" t="inlineStr">
+        <is>
+          <t>A/C amplifier A18 (1993 book: A15), passenger side behind the glove box, on the bottom of the evaporator housing; tap point on the lead at the amplifier, distance TBD</t>
+        </is>
+      </c>
+      <c r="AB74" s="53" t="inlineStr">
+        <is>
+          <t>Y-R</t>
+        </is>
+      </c>
+      <c r="AC74" s="54" t="inlineStr">
+        <is>
+          <t>1990 ST185 EWD p.152 (docs/electrical/ewd-snips/1990-st185-autoac-pressure-clutch-p152.png); 1992 EWD132U p.219 A17-13 (ewd-snips/1992-celica-ewd132u-a17-pressure-p219.png); 1990 ST185 EWD p.152; 1992 EWD132U p.219 (A17-13); locator 1990 ST185 EWD p.17 Instrument Panel (ewd-snips/1990-st185-locations-dash.png); Mitchell locations (docs/research/AUTO-AC-AMP-OPTIONS.html)</t>
+        </is>
+      </c>
+      <c r="AD74" s="54" t="inlineStr">
+        <is>
+          <t>solder splice onto the factory Y-R lead at the A/C amplifier</t>
+        </is>
+      </c>
       <c r="AE74" s="54" t="inlineStr">
         <is>
-          <t>splice sp_5v_2: node of the wire list (SoT)</t>
+          <t>flying lead FL_ACAMP_PSW: EWD A18 pin 13 Y-R; splice sp_ac_psw: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF74" s="54" t="inlineStr">
@@ -9795,21 +9779,17 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG74" s="54" t="inlineStr">
-        <is>
-          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
-        </is>
-      </c>
+      <c r="AG74" s="54" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="23" t="inlineStr">
         <is>
-          <t>SGND</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="B75" s="23" t="inlineStr">
         <is>
-          <t>w40</t>
+          <t>w_acc86</t>
         </is>
       </c>
       <c r="C75" s="23" t="inlineStr">
@@ -9817,91 +9797,99 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D75" s="23" t="inlineStr"/>
+      <c r="D75" s="23" t="inlineStr">
+        <is>
+          <t>CabinPower</t>
+        </is>
+      </c>
       <c r="E75" s="24" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="F75" s="25" t="inlineStr">
         <is>
-          <t>aps</t>
+          <t>sp_ac_psw</t>
         </is>
       </c>
       <c r="G75" s="26" t="inlineStr">
         <is>
-          <t>PEDAL</t>
-        </is>
-      </c>
-      <c r="H75" s="25" t="n">
-        <v>5</v>
-      </c>
+          <t>splice sp_ac_psw (SP-AC-PSW: A/C pressure switch output)</t>
+        </is>
+      </c>
+      <c r="H75" s="25" t="inlineStr"/>
       <c r="I75" s="26" t="inlineStr">
         <is>
-          <t>Pedal 1 ground</t>
+          <t>A/C clutch relay (+)</t>
         </is>
       </c>
       <c r="J75" s="26" t="inlineStr"/>
       <c r="K75" s="27" t="inlineStr">
         <is>
-          <t>splice</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="L75" s="28" t="inlineStr">
         <is>
-          <t>sp_gndout</t>
+          <t>k_acc</t>
         </is>
       </c>
       <c r="M75" s="29" t="inlineStr">
         <is>
-          <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
-        </is>
-      </c>
-      <c r="N75" s="28" t="inlineStr"/>
+          <t>LOGIC M5</t>
+        </is>
+      </c>
+      <c r="N75" s="28" t="n">
+        <v>86</v>
+      </c>
       <c r="O75" s="29" t="inlineStr">
         <is>
-          <t>Pedal 1 ground</t>
-        </is>
-      </c>
-      <c r="P75" s="29" t="inlineStr"/>
+          <t>A/C clutch relay (+)</t>
+        </is>
+      </c>
+      <c r="P75" s="29" t="inlineStr">
+        <is>
+          <t>LOGIC box (glove box) relay M15 A/C clutch, pin 86</t>
+        </is>
+      </c>
       <c r="Q75" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A24</t>
+          <t>A5.4</t>
         </is>
       </c>
       <c r="R75" s="31" t="inlineStr">
         <is>
-          <t>Sensor GND (ECU-A A24)</t>
+          <t>A/C pressure-switched relay coil +</t>
         </is>
       </c>
       <c r="S75" s="32" t="inlineStr">
         <is>
-          <t>sp_gndout</t>
-        </is>
-      </c>
-      <c r="T75" s="32" t="inlineStr">
-        <is>
-          <t>cab_aps1</t>
-        </is>
-      </c>
+          <t>sp_ac_psw</t>
+        </is>
+      </c>
+      <c r="T75" s="32" t="inlineStr"/>
       <c r="U75" s="33" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="V75" s="34" t="inlineStr">
         <is>
           <t>Yellow</t>
         </is>
       </c>
-      <c r="W75" s="34" t="inlineStr"/>
+      <c r="W75" s="34" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
       <c r="X75" s="34" t="inlineStr">
         <is>
-          <t>Yellow-Yellow-Blue</t>
+          <t>Yellow-Blue</t>
         </is>
       </c>
       <c r="Y75" s="34" t="inlineStr"/>
       <c r="Z75" s="35" t="inlineStr">
         <is>
-          <t>pedal branch (driver footwell)</t>
+          <t>A/C amp branch (behind dash)</t>
         </is>
       </c>
       <c r="AA75" s="36" t="inlineStr"/>
@@ -9910,7 +9898,7 @@
       <c r="AD75" s="38" t="inlineStr"/>
       <c r="AE75" s="38" t="inlineStr">
         <is>
-          <t>splice sp_gndout: node of the wire list (SoT)</t>
+          <t>splice sp_ac_psw: node of the wire list (SoT); fuse-box plan k_acc 86 (18 AWG)</t>
         </is>
       </c>
       <c r="AF75" s="38" t="inlineStr">
@@ -9920,19 +9908,19 @@
       </c>
       <c r="AG75" s="38" t="inlineStr">
         <is>
-          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
+          <t>owner TBD: a half has no length estimate (drawn today as w_acc86 on A-cabin, ? mm; w_acc86_cp on CabinPower, 400 mm)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="39" t="inlineStr">
         <is>
-          <t>APS</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="B76" s="39" t="inlineStr">
         <is>
-          <t>w38</t>
+          <t>w_aps_vc1</t>
         </is>
       </c>
       <c r="C76" s="39" t="inlineStr">
@@ -9957,51 +9945,51 @@
         </is>
       </c>
       <c r="H76" s="41" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I76" s="42" t="inlineStr">
         <is>
-          <t>Pedal 1 signal main</t>
+          <t>+5 V pedal sensor 1</t>
         </is>
       </c>
       <c r="J76" s="42" t="inlineStr"/>
       <c r="K76" s="43" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="L76" s="44" t="inlineStr">
         <is>
-          <t>ecu_a</t>
+          <t>sp_5v_2</t>
         </is>
       </c>
       <c r="M76" s="45" t="inlineStr">
         <is>
-          <t>ECU-A</t>
-        </is>
-      </c>
-      <c r="N76" s="44" t="inlineStr">
-        <is>
-          <t>A14</t>
-        </is>
-      </c>
+          <t>splice sp_5v_2 (SP-5V-PEDAL: +5 V to pedal + cruise)</t>
+        </is>
+      </c>
+      <c r="N76" s="44" t="inlineStr"/>
       <c r="O76" s="45" t="inlineStr">
         <is>
-          <t>Pedal 1 signal main</t>
+          <t>+5 V pedal sensor 1</t>
         </is>
       </c>
       <c r="P76" s="45" t="inlineStr"/>
       <c r="Q76" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A14</t>
+          <t>ECU-A.A32</t>
         </is>
       </c>
       <c r="R76" s="47" t="inlineStr">
         <is>
-          <t>Pedal 1 signal main (ECU-A A14)</t>
-        </is>
-      </c>
-      <c r="S76" s="48" t="inlineStr"/>
+          <t>+5V sensor (ECU-A A32)</t>
+        </is>
+      </c>
+      <c r="S76" s="48" t="inlineStr">
+        <is>
+          <t>sp_5v_2</t>
+        </is>
+      </c>
       <c r="T76" s="48" t="inlineStr">
         <is>
           <t>cab_aps1</t>
@@ -10012,18 +10000,16 @@
       </c>
       <c r="V76" s="50" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="W76" s="50" t="inlineStr"/>
       <c r="X76" s="50" t="inlineStr">
         <is>
-          <t>White-Blue-Yellow</t>
-        </is>
-      </c>
-      <c r="Y76" s="50" t="n">
-        <v>1050</v>
-      </c>
+          <t>Blue-Blue</t>
+        </is>
+      </c>
+      <c r="Y76" s="50" t="inlineStr"/>
       <c r="Z76" s="51" t="inlineStr">
         <is>
           <t>pedal branch (driver footwell)</t>
@@ -10035,7 +10021,7 @@
       <c r="AD76" s="54" t="inlineStr"/>
       <c r="AE76" s="54" t="inlineStr">
         <is>
-          <t>channels.csv ecu_a A14 An Volt 4 (AV4_APS_MAIN)</t>
+          <t>splice sp_5v_2: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF76" s="54" t="inlineStr">
@@ -10052,12 +10038,12 @@
     <row r="77">
       <c r="A77" s="23" t="inlineStr">
         <is>
-          <t>APS</t>
+          <t>SGND</t>
         </is>
       </c>
       <c r="B77" s="23" t="inlineStr">
         <is>
-          <t>cab_aps1_sh</t>
+          <t>w40</t>
         </is>
       </c>
       <c r="C77" s="23" t="inlineStr">
@@ -10068,23 +10054,25 @@
       <c r="D77" s="23" t="inlineStr"/>
       <c r="E77" s="24" t="inlineStr">
         <is>
-          <t>cable screen</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="F77" s="25" t="inlineStr">
         <is>
-          <t>cab_aps1</t>
+          <t>aps</t>
         </is>
       </c>
       <c r="G77" s="26" t="inlineStr">
         <is>
-          <t>cable screen (one end only)</t>
-        </is>
-      </c>
-      <c r="H77" s="25" t="inlineStr"/>
+          <t>PEDAL</t>
+        </is>
+      </c>
+      <c r="H77" s="25" t="n">
+        <v>5</v>
+      </c>
       <c r="I77" s="26" t="inlineStr">
         <is>
-          <t>Pedal 1 cable shield</t>
+          <t>Pedal 1 ground</t>
         </is>
       </c>
       <c r="J77" s="26" t="inlineStr"/>
@@ -10095,34 +10083,34 @@
       </c>
       <c r="L77" s="28" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>sp_gndout</t>
         </is>
       </c>
       <c r="M77" s="29" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
       <c r="N77" s="28" t="inlineStr"/>
       <c r="O77" s="29" t="inlineStr">
         <is>
-          <t>Pedal 1 cable shield</t>
+          <t>Pedal 1 ground</t>
         </is>
       </c>
       <c r="P77" s="29" t="inlineStr"/>
       <c r="Q77" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A7</t>
+          <t>ECU-A.A24</t>
         </is>
       </c>
       <c r="R77" s="31" t="inlineStr">
         <is>
-          <t>Screen A (ECU A7, SHIELD_A)</t>
+          <t>Sensor GND (ECU-A A24)</t>
         </is>
       </c>
       <c r="S77" s="32" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>sp_gndout</t>
         </is>
       </c>
       <c r="T77" s="32" t="inlineStr">
@@ -10130,22 +10118,24 @@
           <t>cab_aps1</t>
         </is>
       </c>
-      <c r="U77" s="33" t="inlineStr"/>
+      <c r="U77" s="33" t="n">
+        <v>20</v>
+      </c>
       <c r="V77" s="34" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="W77" s="34" t="inlineStr"/>
       <c r="X77" s="34" t="inlineStr">
         <is>
-          <t>White-Blue-Yellow</t>
+          <t>Yellow-Yellow-Blue</t>
         </is>
       </c>
       <c r="Y77" s="34" t="inlineStr"/>
       <c r="Z77" s="35" t="inlineStr">
         <is>
-          <t>at ECU-A plug</t>
+          <t>pedal branch (driver footwell)</t>
         </is>
       </c>
       <c r="AA77" s="36" t="inlineStr"/>
@@ -10154,7 +10144,7 @@
       <c r="AD77" s="38" t="inlineStr"/>
       <c r="AE77" s="38" t="inlineStr">
         <is>
-          <t>splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>splice sp_gndout: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF77" s="38" t="inlineStr">
@@ -10164,19 +10154,19 @@
       </c>
       <c r="AG77" s="38" t="inlineStr">
         <is>
-          <t>screen floats at the far end; pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
+          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="39" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>APS</t>
         </is>
       </c>
       <c r="B78" s="39" t="inlineStr">
         <is>
-          <t>w210</t>
+          <t>w38</t>
         </is>
       </c>
       <c r="C78" s="39" t="inlineStr">
@@ -10201,54 +10191,54 @@
         </is>
       </c>
       <c r="H78" s="41" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I78" s="42" t="inlineStr">
         <is>
-          <t>+5 V pedal sensor 2</t>
+          <t>Pedal 1 signal main</t>
         </is>
       </c>
       <c r="J78" s="42" t="inlineStr"/>
       <c r="K78" s="43" t="inlineStr">
         <is>
-          <t>splice</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="L78" s="44" t="inlineStr">
         <is>
-          <t>sp_5v_2</t>
+          <t>ecu_a</t>
         </is>
       </c>
       <c r="M78" s="45" t="inlineStr">
         <is>
-          <t>splice sp_5v_2 (SP-5V-PEDAL: +5 V to pedal + cruise)</t>
-        </is>
-      </c>
-      <c r="N78" s="44" t="inlineStr"/>
+          <t>ECU-A</t>
+        </is>
+      </c>
+      <c r="N78" s="44" t="inlineStr">
+        <is>
+          <t>A14</t>
+        </is>
+      </c>
       <c r="O78" s="45" t="inlineStr">
         <is>
-          <t>+5 V pedal sensor 2</t>
+          <t>Pedal 1 signal main</t>
         </is>
       </c>
       <c r="P78" s="45" t="inlineStr"/>
       <c r="Q78" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A32</t>
+          <t>ECU-A.A14</t>
         </is>
       </c>
       <c r="R78" s="47" t="inlineStr">
         <is>
-          <t>+5V sensor (ECU-A A32)</t>
-        </is>
-      </c>
-      <c r="S78" s="48" t="inlineStr">
-        <is>
-          <t>sp_5v_2</t>
-        </is>
-      </c>
+          <t>Pedal 1 signal main (ECU-A A14)</t>
+        </is>
+      </c>
+      <c r="S78" s="48" t="inlineStr"/>
       <c r="T78" s="48" t="inlineStr">
         <is>
-          <t>cab_aps2</t>
+          <t>cab_aps1</t>
         </is>
       </c>
       <c r="U78" s="49" t="n">
@@ -10256,16 +10246,18 @@
       </c>
       <c r="V78" s="50" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="W78" s="50" t="inlineStr"/>
       <c r="X78" s="50" t="inlineStr">
         <is>
-          <t>Blue-Blue</t>
-        </is>
-      </c>
-      <c r="Y78" s="50" t="inlineStr"/>
+          <t>White-Blue-Yellow</t>
+        </is>
+      </c>
+      <c r="Y78" s="50" t="n">
+        <v>1050</v>
+      </c>
       <c r="Z78" s="51" t="inlineStr">
         <is>
           <t>pedal branch (driver footwell)</t>
@@ -10277,7 +10269,7 @@
       <c r="AD78" s="54" t="inlineStr"/>
       <c r="AE78" s="54" t="inlineStr">
         <is>
-          <t>splice sp_5v_2: node of the wire list (SoT)</t>
+          <t>channels.csv ecu_a A14 An Volt 4 (AV4_APS_MAIN)</t>
         </is>
       </c>
       <c r="AF78" s="54" t="inlineStr">
@@ -10294,12 +10286,12 @@
     <row r="79">
       <c r="A79" s="23" t="inlineStr">
         <is>
-          <t>SGND</t>
+          <t>APS</t>
         </is>
       </c>
       <c r="B79" s="23" t="inlineStr">
         <is>
-          <t>w_aps_gnd2</t>
+          <t>cab_aps1_sh</t>
         </is>
       </c>
       <c r="C79" s="23" t="inlineStr">
@@ -10310,25 +10302,23 @@
       <c r="D79" s="23" t="inlineStr"/>
       <c r="E79" s="24" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>cable screen</t>
         </is>
       </c>
       <c r="F79" s="25" t="inlineStr">
         <is>
-          <t>aps</t>
+          <t>cab_aps1</t>
         </is>
       </c>
       <c r="G79" s="26" t="inlineStr">
         <is>
-          <t>PEDAL</t>
-        </is>
-      </c>
-      <c r="H79" s="25" t="n">
-        <v>2</v>
-      </c>
+          <t>cable screen (one end only)</t>
+        </is>
+      </c>
+      <c r="H79" s="25" t="inlineStr"/>
       <c r="I79" s="26" t="inlineStr">
         <is>
-          <t>Pedal 2 ground</t>
+          <t>Pedal 1 cable shield</t>
         </is>
       </c>
       <c r="J79" s="26" t="inlineStr"/>
@@ -10339,59 +10329,57 @@
       </c>
       <c r="L79" s="28" t="inlineStr">
         <is>
-          <t>sp_gndout</t>
+          <t>sp_shield_a_aps</t>
         </is>
       </c>
       <c r="M79" s="29" t="inlineStr">
         <is>
-          <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
+          <t>splice sp_shield_a_aps (SP-SHIELD-A-APS)</t>
         </is>
       </c>
       <c r="N79" s="28" t="inlineStr"/>
       <c r="O79" s="29" t="inlineStr">
         <is>
-          <t>Pedal 2 ground</t>
+          <t>Pedal 1 cable shield</t>
         </is>
       </c>
       <c r="P79" s="29" t="inlineStr"/>
       <c r="Q79" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A24</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R79" s="31" t="inlineStr">
         <is>
-          <t>Sensor GND (ECU-A A24)</t>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
         </is>
       </c>
       <c r="S79" s="32" t="inlineStr">
         <is>
-          <t>sp_gndout</t>
+          <t>sp_shield_a_aps</t>
         </is>
       </c>
       <c r="T79" s="32" t="inlineStr">
         <is>
-          <t>cab_aps2</t>
-        </is>
-      </c>
-      <c r="U79" s="33" t="n">
-        <v>20</v>
-      </c>
+          <t>cab_aps1</t>
+        </is>
+      </c>
+      <c r="U79" s="33" t="inlineStr"/>
       <c r="V79" s="34" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="W79" s="34" t="inlineStr"/>
       <c r="X79" s="34" t="inlineStr">
         <is>
-          <t>Yellow-Yellow-Blue</t>
+          <t>White-Blue-Yellow</t>
         </is>
       </c>
       <c r="Y79" s="34" t="inlineStr"/>
       <c r="Z79" s="35" t="inlineStr">
         <is>
-          <t>pedal branch (driver footwell)</t>
+          <t>at ECU-A plug</t>
         </is>
       </c>
       <c r="AA79" s="36" t="inlineStr"/>
@@ -10400,7 +10388,7 @@
       <c r="AD79" s="38" t="inlineStr"/>
       <c r="AE79" s="38" t="inlineStr">
         <is>
-          <t>splice sp_gndout: node of the wire list (SoT)</t>
+          <t>splice sp_shield_a_aps: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF79" s="38" t="inlineStr">
@@ -10410,19 +10398,19 @@
       </c>
       <c r="AG79" s="38" t="inlineStr">
         <is>
-          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
+          <t>screen floats at the far end; pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="39" t="inlineStr">
         <is>
-          <t>APS</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="B80" s="39" t="inlineStr">
         <is>
-          <t>w_aps_vpa2</t>
+          <t>w210</t>
         </is>
       </c>
       <c r="C80" s="39" t="inlineStr">
@@ -10430,11 +10418,7 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D80" s="39" t="inlineStr">
-        <is>
-          <t>B-cabin</t>
-        </is>
-      </c>
+      <c r="D80" s="39" t="inlineStr"/>
       <c r="E80" s="40" t="inlineStr">
         <is>
           <t>connector</t>
@@ -10451,55 +10435,51 @@
         </is>
       </c>
       <c r="H80" s="41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I80" s="42" t="inlineStr">
         <is>
-          <t>Pedal 2 signal sub</t>
+          <t>+5 V pedal sensor 2</t>
         </is>
       </c>
       <c r="J80" s="42" t="inlineStr"/>
       <c r="K80" s="43" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="L80" s="44" t="inlineStr">
         <is>
-          <t>ecu_b</t>
+          <t>sp_5v_2</t>
         </is>
       </c>
       <c r="M80" s="45" t="inlineStr">
         <is>
-          <t>ECU-B (Link G4X plug B, centre dash)</t>
-        </is>
-      </c>
-      <c r="N80" s="44" t="inlineStr">
-        <is>
-          <t>B33</t>
-        </is>
-      </c>
+          <t>splice sp_5v_2 (SP-5V-PEDAL: +5 V to pedal + cruise)</t>
+        </is>
+      </c>
+      <c r="N80" s="44" t="inlineStr"/>
       <c r="O80" s="45" t="inlineStr">
         <is>
-          <t>Pedal 2 signal sub</t>
-        </is>
-      </c>
-      <c r="P80" s="45" t="inlineStr">
-        <is>
-          <t>ECU-B plug pin B33 (Link G4X, centre dash); VPA2</t>
-        </is>
-      </c>
+          <t>+5 V pedal sensor 2</t>
+        </is>
+      </c>
+      <c r="P80" s="45" t="inlineStr"/>
       <c r="Q80" s="46" t="inlineStr">
         <is>
-          <t>ECU-B.B33</t>
+          <t>ECU-A.A32</t>
         </is>
       </c>
       <c r="R80" s="47" t="inlineStr">
         <is>
-          <t>Pedal 2 signal sub (ECU-B B33)</t>
-        </is>
-      </c>
-      <c r="S80" s="48" t="inlineStr"/>
+          <t>+5V sensor (ECU-A A32)</t>
+        </is>
+      </c>
+      <c r="S80" s="48" t="inlineStr">
+        <is>
+          <t>sp_5v_2</t>
+        </is>
+      </c>
       <c r="T80" s="48" t="inlineStr">
         <is>
           <t>cab_aps2</t>
@@ -10510,21 +10490,19 @@
       </c>
       <c r="V80" s="50" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="W80" s="50" t="inlineStr"/>
       <c r="X80" s="50" t="inlineStr">
         <is>
-          <t>White-Blue-Yellow</t>
-        </is>
-      </c>
-      <c r="Y80" s="50" t="n">
-        <v>1720</v>
-      </c>
+          <t>Blue-Blue</t>
+        </is>
+      </c>
+      <c r="Y80" s="50" t="inlineStr"/>
       <c r="Z80" s="51" t="inlineStr">
         <is>
-          <t>pedal branch (driver footwell) / to ECU-B plug (beside ECU-A)</t>
+          <t>pedal branch (driver footwell)</t>
         </is>
       </c>
       <c r="AA80" s="52" t="inlineStr"/>
@@ -10533,7 +10511,7 @@
       <c r="AD80" s="54" t="inlineStr"/>
       <c r="AE80" s="54" t="inlineStr">
         <is>
-          <t>channels.csv ecu_b B33 An Volt 5 (AV5_APS_SUB)</t>
+          <t>splice sp_5v_2: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF80" s="54" t="inlineStr">
@@ -10543,19 +10521,19 @@
       </c>
       <c r="AG80" s="54" t="inlineStr">
         <is>
-          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143); owner proposed: longer half (drawn today as w_aps_vpa2 on A-cabin, 1720 mm; w39 on B-cabin, 1250 mm)</t>
+          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="23" t="inlineStr">
         <is>
-          <t>APS</t>
+          <t>SGND</t>
         </is>
       </c>
       <c r="B81" s="23" t="inlineStr">
         <is>
-          <t>cab_aps_sh</t>
+          <t>w_aps_gnd2</t>
         </is>
       </c>
       <c r="C81" s="23" t="inlineStr">
@@ -10566,23 +10544,25 @@
       <c r="D81" s="23" t="inlineStr"/>
       <c r="E81" s="24" t="inlineStr">
         <is>
-          <t>cable screen</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="F81" s="25" t="inlineStr">
         <is>
-          <t>cab_aps2</t>
+          <t>aps</t>
         </is>
       </c>
       <c r="G81" s="26" t="inlineStr">
         <is>
-          <t>cable screen (one end only)</t>
-        </is>
-      </c>
-      <c r="H81" s="25" t="inlineStr"/>
+          <t>PEDAL</t>
+        </is>
+      </c>
+      <c r="H81" s="25" t="n">
+        <v>2</v>
+      </c>
       <c r="I81" s="26" t="inlineStr">
         <is>
-          <t>Pedal 2 cable shield</t>
+          <t>Pedal 2 ground</t>
         </is>
       </c>
       <c r="J81" s="26" t="inlineStr"/>
@@ -10593,34 +10573,34 @@
       </c>
       <c r="L81" s="28" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>sp_gndout</t>
         </is>
       </c>
       <c r="M81" s="29" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
       <c r="N81" s="28" t="inlineStr"/>
       <c r="O81" s="29" t="inlineStr">
         <is>
-          <t>Pedal 2 cable shield</t>
+          <t>Pedal 2 ground</t>
         </is>
       </c>
       <c r="P81" s="29" t="inlineStr"/>
       <c r="Q81" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A7</t>
+          <t>ECU-A.A24</t>
         </is>
       </c>
       <c r="R81" s="31" t="inlineStr">
         <is>
-          <t>Screen A (ECU A7, SHIELD_A)</t>
+          <t>Sensor GND (ECU-A A24)</t>
         </is>
       </c>
       <c r="S81" s="32" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>sp_gndout</t>
         </is>
       </c>
       <c r="T81" s="32" t="inlineStr">
@@ -10628,22 +10608,24 @@
           <t>cab_aps2</t>
         </is>
       </c>
-      <c r="U81" s="33" t="inlineStr"/>
+      <c r="U81" s="33" t="n">
+        <v>20</v>
+      </c>
       <c r="V81" s="34" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="W81" s="34" t="inlineStr"/>
       <c r="X81" s="34" t="inlineStr">
         <is>
-          <t>White-Blue-Yellow</t>
+          <t>Yellow-Yellow-Blue</t>
         </is>
       </c>
       <c r="Y81" s="34" t="inlineStr"/>
       <c r="Z81" s="35" t="inlineStr">
         <is>
-          <t>at ECU-A plug</t>
+          <t>pedal branch (driver footwell)</t>
         </is>
       </c>
       <c r="AA81" s="36" t="inlineStr"/>
@@ -10652,7 +10634,7 @@
       <c r="AD81" s="38" t="inlineStr"/>
       <c r="AE81" s="38" t="inlineStr">
         <is>
-          <t>splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>splice sp_gndout: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF81" s="38" t="inlineStr">
@@ -10662,19 +10644,19 @@
       </c>
       <c r="AG81" s="38" t="inlineStr">
         <is>
-          <t>screen floats at the far end; pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
+          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="39" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>APS</t>
         </is>
       </c>
       <c r="B82" s="39" t="inlineStr">
         <is>
-          <t>cab_fspur_5v</t>
+          <t>w_aps_vpa2</t>
         </is>
       </c>
       <c r="C82" s="39" t="inlineStr">
@@ -10682,7 +10664,11 @@
           <t>A-cabin</t>
         </is>
       </c>
-      <c r="D82" s="39" t="inlineStr"/>
+      <c r="D82" s="39" t="inlineStr">
+        <is>
+          <t>B-cabin</t>
+        </is>
+      </c>
       <c r="E82" s="40" t="inlineStr">
         <is>
           <t>connector</t>
@@ -10690,63 +10676,67 @@
       </c>
       <c r="F82" s="41" t="inlineStr">
         <is>
-          <t>ix_ws_front_p</t>
+          <t>aps</t>
         </is>
       </c>
       <c r="G82" s="42" t="inlineStr">
         <is>
-          <t>FRONT WS INLINE</t>
+          <t>PEDAL</t>
         </is>
       </c>
       <c r="H82" s="41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I82" s="42" t="inlineStr">
         <is>
-          <t>VRC-F +5V</t>
+          <t>Pedal 2 signal sub</t>
         </is>
       </c>
       <c r="J82" s="42" t="inlineStr"/>
       <c r="K82" s="43" t="inlineStr">
         <is>
-          <t>splice</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="L82" s="44" t="inlineStr">
         <is>
-          <t>sp_5v</t>
+          <t>ecu_b</t>
         </is>
       </c>
       <c r="M82" s="45" t="inlineStr">
         <is>
-          <t>splice sp_5v (SP-5V-A: +5 V sensor supply)</t>
-        </is>
-      </c>
-      <c r="N82" s="44" t="inlineStr"/>
+          <t>ECU-B (Link G4X plug B, centre dash)</t>
+        </is>
+      </c>
+      <c r="N82" s="44" t="inlineStr">
+        <is>
+          <t>B33</t>
+        </is>
+      </c>
       <c r="O82" s="45" t="inlineStr">
         <is>
-          <t>VRC-F +5V</t>
-        </is>
-      </c>
-      <c r="P82" s="45" t="inlineStr"/>
+          <t>Pedal 2 signal sub</t>
+        </is>
+      </c>
+      <c r="P82" s="45" t="inlineStr">
+        <is>
+          <t>ECU-B plug pin B33 (Link G4X, centre dash); VPA2</t>
+        </is>
+      </c>
       <c r="Q82" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A32</t>
+          <t>ECU-B.B33</t>
         </is>
       </c>
       <c r="R82" s="47" t="inlineStr">
         <is>
-          <t>+5V sensor (ECU-A A32)</t>
-        </is>
-      </c>
-      <c r="S82" s="48" t="inlineStr">
-        <is>
-          <t>sp_5v</t>
-        </is>
-      </c>
+          <t>Pedal 2 signal sub (ECU-B B33)</t>
+        </is>
+      </c>
+      <c r="S82" s="48" t="inlineStr"/>
       <c r="T82" s="48" t="inlineStr">
         <is>
-          <t>cab_fspur</t>
+          <t>cab_aps2</t>
         </is>
       </c>
       <c r="U82" s="49" t="n">
@@ -10754,19 +10744,21 @@
       </c>
       <c r="V82" s="50" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="W82" s="50" t="inlineStr"/>
       <c r="X82" s="50" t="inlineStr">
         <is>
-          <t>Blue-Blue</t>
-        </is>
-      </c>
-      <c r="Y82" s="50" t="inlineStr"/>
+          <t>White-Blue-Yellow</t>
+        </is>
+      </c>
+      <c r="Y82" s="50" t="n">
+        <v>1720</v>
+      </c>
       <c r="Z82" s="51" t="inlineStr">
         <is>
-          <t>dash branch (front WS inline)</t>
+          <t>pedal branch (driver footwell) / to ECU-B plug (beside ECU-A)</t>
         </is>
       </c>
       <c r="AA82" s="52" t="inlineStr"/>
@@ -10775,7 +10767,7 @@
       <c r="AD82" s="54" t="inlineStr"/>
       <c r="AE82" s="54" t="inlineStr">
         <is>
-          <t>splice sp_5v: node of the wire list (SoT)</t>
+          <t>channels.csv ecu_b B33 An Volt 5 (AV5_APS_SUB)</t>
         </is>
       </c>
       <c r="AF82" s="54" t="inlineStr">
@@ -10783,17 +10775,21 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG82" s="54" t="inlineStr"/>
+      <c r="AG82" s="54" t="inlineStr">
+        <is>
+          <t>pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143); owner proposed: longer half (drawn today as w_aps_vpa2 on A-cabin, 1720 mm; w39 on B-cabin, 1250 mm)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="23" t="inlineStr">
         <is>
-          <t>SGND</t>
+          <t>APS</t>
         </is>
       </c>
       <c r="B83" s="23" t="inlineStr">
         <is>
-          <t>cab_fspur_gnd</t>
+          <t>cab_aps_sh</t>
         </is>
       </c>
       <c r="C83" s="23" t="inlineStr">
@@ -10804,25 +10800,23 @@
       <c r="D83" s="23" t="inlineStr"/>
       <c r="E83" s="24" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>cable screen</t>
         </is>
       </c>
       <c r="F83" s="25" t="inlineStr">
         <is>
-          <t>ix_ws_front_p</t>
+          <t>cab_aps2</t>
         </is>
       </c>
       <c r="G83" s="26" t="inlineStr">
         <is>
-          <t>FRONT WS INLINE</t>
-        </is>
-      </c>
-      <c r="H83" s="25" t="n">
-        <v>2</v>
-      </c>
+          <t>cable screen (one end only)</t>
+        </is>
+      </c>
+      <c r="H83" s="25" t="inlineStr"/>
       <c r="I83" s="26" t="inlineStr">
         <is>
-          <t>VRC-F GND</t>
+          <t>Pedal 2 cable shield</t>
         </is>
       </c>
       <c r="J83" s="26" t="inlineStr"/>
@@ -10833,59 +10827,57 @@
       </c>
       <c r="L83" s="28" t="inlineStr">
         <is>
-          <t>sp_gndout</t>
+          <t>sp_shield_a_aps</t>
         </is>
       </c>
       <c r="M83" s="29" t="inlineStr">
         <is>
-          <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
+          <t>splice sp_shield_a_aps (SP-SHIELD-A-APS)</t>
         </is>
       </c>
       <c r="N83" s="28" t="inlineStr"/>
       <c r="O83" s="29" t="inlineStr">
         <is>
-          <t>VRC-F GND</t>
+          <t>Pedal 2 cable shield</t>
         </is>
       </c>
       <c r="P83" s="29" t="inlineStr"/>
       <c r="Q83" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A24</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R83" s="31" t="inlineStr">
         <is>
-          <t>Sensor GND (ECU-A A24)</t>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
         </is>
       </c>
       <c r="S83" s="32" t="inlineStr">
         <is>
-          <t>sp_gndout</t>
+          <t>sp_shield_a_aps</t>
         </is>
       </c>
       <c r="T83" s="32" t="inlineStr">
         <is>
-          <t>cab_fspur</t>
-        </is>
-      </c>
-      <c r="U83" s="33" t="n">
-        <v>20</v>
-      </c>
+          <t>cab_aps2</t>
+        </is>
+      </c>
+      <c r="U83" s="33" t="inlineStr"/>
       <c r="V83" s="34" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="W83" s="34" t="inlineStr"/>
       <c r="X83" s="34" t="inlineStr">
         <is>
-          <t>Yellow-Yellow-Blue</t>
+          <t>White-Blue-Yellow</t>
         </is>
       </c>
       <c r="Y83" s="34" t="inlineStr"/>
       <c r="Z83" s="35" t="inlineStr">
         <is>
-          <t>dash branch (front WS inline)</t>
+          <t>at ECU-A plug</t>
         </is>
       </c>
       <c r="AA83" s="36" t="inlineStr"/>
@@ -10894,7 +10886,7 @@
       <c r="AD83" s="38" t="inlineStr"/>
       <c r="AE83" s="38" t="inlineStr">
         <is>
-          <t>splice sp_gndout: node of the wire list (SoT)</t>
+          <t>splice sp_shield_a_aps: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF83" s="38" t="inlineStr">
@@ -10902,17 +10894,21 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG83" s="38" t="inlineStr"/>
+      <c r="AG83" s="38" t="inlineStr">
+        <is>
+          <t>screen floats at the far end; pedal branch length is a placeholder: measure at the car (OPEN-ITEMS row 143)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="39" t="inlineStr">
         <is>
-          <t>WSSF</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="B84" s="39" t="inlineStr">
         <is>
-          <t>cab_fspur_l</t>
+          <t>cab_fspur_5v</t>
         </is>
       </c>
       <c r="C84" s="39" t="inlineStr">
@@ -10937,51 +10933,51 @@
         </is>
       </c>
       <c r="H84" s="41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I84" s="42" t="inlineStr">
         <is>
-          <t>FL conditioned out</t>
+          <t>VRC-F +5V</t>
         </is>
       </c>
       <c r="J84" s="42" t="inlineStr"/>
       <c r="K84" s="43" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="L84" s="44" t="inlineStr">
         <is>
-          <t>ecu_a</t>
+          <t>sp_5v</t>
         </is>
       </c>
       <c r="M84" s="45" t="inlineStr">
         <is>
-          <t>ECU-A</t>
-        </is>
-      </c>
-      <c r="N84" s="44" t="inlineStr">
-        <is>
-          <t>A23</t>
-        </is>
-      </c>
+          <t>splice sp_5v (SP-5V-A: +5 V sensor supply)</t>
+        </is>
+      </c>
+      <c r="N84" s="44" t="inlineStr"/>
       <c r="O84" s="45" t="inlineStr">
         <is>
-          <t>FL conditioned out</t>
+          <t>VRC-F +5V</t>
         </is>
       </c>
       <c r="P84" s="45" t="inlineStr"/>
       <c r="Q84" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A23</t>
+          <t>ECU-A.A32</t>
         </is>
       </c>
       <c r="R84" s="47" t="inlineStr">
         <is>
-          <t>FL conditioned out (ECU-A A23)</t>
-        </is>
-      </c>
-      <c r="S84" s="48" t="inlineStr"/>
+          <t>+5V sensor (ECU-A A32)</t>
+        </is>
+      </c>
+      <c r="S84" s="48" t="inlineStr">
+        <is>
+          <t>sp_5v</t>
+        </is>
+      </c>
       <c r="T84" s="48" t="inlineStr">
         <is>
           <t>cab_fspur</t>
@@ -10992,18 +10988,16 @@
       </c>
       <c r="V84" s="50" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="W84" s="50" t="inlineStr"/>
       <c r="X84" s="50" t="inlineStr">
         <is>
-          <t>White-Blue-Blue</t>
-        </is>
-      </c>
-      <c r="Y84" s="50" t="n">
-        <v>330</v>
-      </c>
+          <t>Blue-Blue</t>
+        </is>
+      </c>
+      <c r="Y84" s="50" t="inlineStr"/>
       <c r="Z84" s="51" t="inlineStr">
         <is>
           <t>dash branch (front WS inline)</t>
@@ -11015,7 +11009,7 @@
       <c r="AD84" s="54" t="inlineStr"/>
       <c r="AE84" s="54" t="inlineStr">
         <is>
-          <t>channels.csv ecu_a A23 DI 3 (DI3_WSS_FL)</t>
+          <t>splice sp_5v: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF84" s="54" t="inlineStr">
@@ -11028,12 +11022,12 @@
     <row r="85">
       <c r="A85" s="23" t="inlineStr">
         <is>
-          <t>WSSF</t>
+          <t>SGND</t>
         </is>
       </c>
       <c r="B85" s="23" t="inlineStr">
         <is>
-          <t>cab_fspur_sh</t>
+          <t>cab_fspur_gnd</t>
         </is>
       </c>
       <c r="C85" s="23" t="inlineStr">
@@ -11058,11 +11052,11 @@
         </is>
       </c>
       <c r="H85" s="25" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I85" s="26" t="inlineStr">
         <is>
-          <t>WS-F screen drain</t>
+          <t>VRC-F GND</t>
         </is>
       </c>
       <c r="J85" s="26" t="inlineStr"/>
@@ -11073,34 +11067,34 @@
       </c>
       <c r="L85" s="28" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>sp_gndout</t>
         </is>
       </c>
       <c r="M85" s="29" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
       <c r="N85" s="28" t="inlineStr"/>
       <c r="O85" s="29" t="inlineStr">
         <is>
-          <t>WS-F screen drain</t>
+          <t>VRC-F GND</t>
         </is>
       </c>
       <c r="P85" s="29" t="inlineStr"/>
       <c r="Q85" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A7</t>
+          <t>ECU-A.A24</t>
         </is>
       </c>
       <c r="R85" s="31" t="inlineStr">
         <is>
-          <t>Screen A (ECU A7, SHIELD_A)</t>
+          <t>Sensor GND (ECU-A A24)</t>
         </is>
       </c>
       <c r="S85" s="32" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>sp_gndout</t>
         </is>
       </c>
       <c r="T85" s="32" t="inlineStr">
@@ -11108,16 +11102,18 @@
           <t>cab_fspur</t>
         </is>
       </c>
-      <c r="U85" s="33" t="inlineStr"/>
+      <c r="U85" s="33" t="n">
+        <v>20</v>
+      </c>
       <c r="V85" s="34" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="W85" s="34" t="inlineStr"/>
       <c r="X85" s="34" t="inlineStr">
         <is>
-          <t>White-Blue-Blue</t>
+          <t>Yellow-Yellow-Blue</t>
         </is>
       </c>
       <c r="Y85" s="34" t="inlineStr"/>
@@ -11132,7 +11128,7 @@
       <c r="AD85" s="38" t="inlineStr"/>
       <c r="AE85" s="38" t="inlineStr">
         <is>
-          <t>splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>splice sp_gndout: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF85" s="38" t="inlineStr">
@@ -11150,7 +11146,7 @@
       </c>
       <c r="B86" s="39" t="inlineStr">
         <is>
-          <t>cab_fspur_fr_sh_ac</t>
+          <t>cab_fspur_l</t>
         </is>
       </c>
       <c r="C86" s="39" t="inlineStr">
@@ -11161,72 +11157,76 @@
       <c r="D86" s="39" t="inlineStr"/>
       <c r="E86" s="40" t="inlineStr">
         <is>
-          <t>cable screen</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="F86" s="41" t="inlineStr">
         <is>
-          <t>cab_fspur_fr_ac</t>
+          <t>ix_ws_front_p</t>
         </is>
       </c>
       <c r="G86" s="42" t="inlineStr">
         <is>
-          <t>cable screen (one end only)</t>
-        </is>
-      </c>
-      <c r="H86" s="41" t="inlineStr"/>
+          <t>FRONT WS INLINE</t>
+        </is>
+      </c>
+      <c r="H86" s="41" t="n">
+        <v>3</v>
+      </c>
       <c r="I86" s="42" t="inlineStr">
         <is>
-          <t>FR wheel spd shield</t>
+          <t>FL conditioned out</t>
         </is>
       </c>
       <c r="J86" s="42" t="inlineStr"/>
       <c r="K86" s="43" t="inlineStr">
         <is>
-          <t>splice</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="L86" s="44" t="inlineStr">
         <is>
-          <t>sp_shield_a</t>
+          <t>ecu_a</t>
         </is>
       </c>
       <c r="M86" s="45" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
-        </is>
-      </c>
-      <c r="N86" s="44" t="inlineStr"/>
+          <t>ECU-A</t>
+        </is>
+      </c>
+      <c r="N86" s="44" t="inlineStr">
+        <is>
+          <t>A23</t>
+        </is>
+      </c>
       <c r="O86" s="45" t="inlineStr">
         <is>
-          <t>FR wheel spd shield</t>
+          <t>FL conditioned out</t>
         </is>
       </c>
       <c r="P86" s="45" t="inlineStr"/>
       <c r="Q86" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A7</t>
+          <t>ECU-A.A23</t>
         </is>
       </c>
       <c r="R86" s="47" t="inlineStr">
         <is>
-          <t>Screen A (ECU A7, SHIELD_A)</t>
-        </is>
-      </c>
-      <c r="S86" s="48" t="inlineStr">
-        <is>
-          <t>sp_shield_a</t>
-        </is>
-      </c>
+          <t>FL conditioned out (ECU-A A23)</t>
+        </is>
+      </c>
+      <c r="S86" s="48" t="inlineStr"/>
       <c r="T86" s="48" t="inlineStr">
         <is>
-          <t>cab_fspur_fr_ac</t>
-        </is>
-      </c>
-      <c r="U86" s="49" t="inlineStr"/>
+          <t>cab_fspur</t>
+        </is>
+      </c>
+      <c r="U86" s="49" t="n">
+        <v>20</v>
+      </c>
       <c r="V86" s="50" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="W86" s="50" t="inlineStr"/>
@@ -11235,7 +11235,9 @@
           <t>White-Blue-Blue</t>
         </is>
       </c>
-      <c r="Y86" s="50" t="inlineStr"/>
+      <c r="Y86" s="50" t="n">
+        <v>330</v>
+      </c>
       <c r="Z86" s="51" t="inlineStr">
         <is>
           <t>dash branch (front WS inline)</t>
@@ -11247,7 +11249,7 @@
       <c r="AD86" s="54" t="inlineStr"/>
       <c r="AE86" s="54" t="inlineStr">
         <is>
-          <t>splice sp_shield_a: node of the wire list (SoT)</t>
+          <t>channels.csv ecu_a A23 DI 3 (DI3_WSS_FL)</t>
         </is>
       </c>
       <c r="AF86" s="54" t="inlineStr">
@@ -11255,15 +11257,19 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG86" s="54" t="inlineStr">
-        <is>
-          <t>tied at the A end only; the far (B) end floats, dressed back at the ECU-B plug (no A-B shield bridge)</t>
-        </is>
-      </c>
+      <c r="AG86" s="54" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="23" t="inlineStr"/>
-      <c r="B87" s="23" t="inlineStr"/>
+      <c r="A87" s="23" t="inlineStr">
+        <is>
+          <t>WSSF</t>
+        </is>
+      </c>
+      <c r="B87" s="23" t="inlineStr">
+        <is>
+          <t>cab_fspur_sh</t>
+        </is>
+      </c>
       <c r="C87" s="23" t="inlineStr">
         <is>
           <t>A-cabin</t>
@@ -11277,54 +11283,90 @@
       </c>
       <c r="F87" s="25" t="inlineStr">
         <is>
-          <t>bh_a_fw</t>
+          <t>ix_ws_front_p</t>
         </is>
       </c>
       <c r="G87" s="26" t="inlineStr">
         <is>
-          <t>BULKHEAD</t>
+          <t>FRONT WS INLINE</t>
         </is>
       </c>
       <c r="H87" s="25" t="n">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="I87" s="26" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
+          <t>WS-F screen drain</t>
         </is>
       </c>
       <c r="J87" s="26" t="inlineStr"/>
-      <c r="K87" s="27" t="inlineStr"/>
-      <c r="L87" s="28" t="inlineStr"/>
-      <c r="M87" s="29" t="inlineStr"/>
+      <c r="K87" s="27" t="inlineStr">
+        <is>
+          <t>splice</t>
+        </is>
+      </c>
+      <c r="L87" s="28" t="inlineStr">
+        <is>
+          <t>sp_shield_a_wsf</t>
+        </is>
+      </c>
+      <c r="M87" s="29" t="inlineStr">
+        <is>
+          <t>splice sp_shield_a_wsf (SP-SHIELD-A-WSF)</t>
+        </is>
+      </c>
       <c r="N87" s="28" t="inlineStr"/>
-      <c r="O87" s="29" t="inlineStr"/>
+      <c r="O87" s="29" t="inlineStr">
+        <is>
+          <t>WS-F screen drain</t>
+        </is>
+      </c>
       <c r="P87" s="29" t="inlineStr"/>
       <c r="Q87" s="30" t="inlineStr">
         <is>
-          <t>DRB102.45</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R87" s="31" t="inlineStr">
         <is>
-          <t>spare (DRB102 45)</t>
-        </is>
-      </c>
-      <c r="S87" s="32" t="inlineStr"/>
-      <c r="T87" s="32" t="inlineStr"/>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="S87" s="32" t="inlineStr">
+        <is>
+          <t>sp_shield_a_wsf</t>
+        </is>
+      </c>
+      <c r="T87" s="32" t="inlineStr">
+        <is>
+          <t>cab_fspur</t>
+        </is>
+      </c>
       <c r="U87" s="33" t="inlineStr"/>
-      <c r="V87" s="34" t="inlineStr"/>
+      <c r="V87" s="34" t="inlineStr">
+        <is>
+          <t>Shield</t>
+        </is>
+      </c>
       <c r="W87" s="34" t="inlineStr"/>
-      <c r="X87" s="34" t="inlineStr"/>
+      <c r="X87" s="34" t="inlineStr">
+        <is>
+          <t>White-Blue-Blue</t>
+        </is>
+      </c>
       <c r="Y87" s="34" t="inlineStr"/>
-      <c r="Z87" s="35" t="inlineStr"/>
+      <c r="Z87" s="35" t="inlineStr">
+        <is>
+          <t>dash branch (front WS inline)</t>
+        </is>
+      </c>
       <c r="AA87" s="36" t="inlineStr"/>
       <c r="AB87" s="37" t="inlineStr"/>
       <c r="AC87" s="38" t="inlineStr"/>
       <c r="AD87" s="38" t="inlineStr"/>
       <c r="AE87" s="38" t="inlineStr">
         <is>
-          <t>DRB102 45 = 'spare (size 16) - was the A/C coolant switch signal, deleted (S35)'</t>
+          <t>splice sp_shield_a_wsf: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF87" s="38" t="inlineStr">
@@ -11335,8 +11377,16 @@
       <c r="AG87" s="38" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="39" t="inlineStr"/>
-      <c r="B88" s="39" t="inlineStr"/>
+      <c r="A88" s="39" t="inlineStr">
+        <is>
+          <t>WSSF</t>
+        </is>
+      </c>
+      <c r="B88" s="39" t="inlineStr">
+        <is>
+          <t>cab_fspur_fr_sh_ac</t>
+        </is>
+      </c>
       <c r="C88" s="39" t="inlineStr">
         <is>
           <t>A-cabin</t>
@@ -11345,59 +11395,93 @@
       <c r="D88" s="39" t="inlineStr"/>
       <c r="E88" s="40" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>cable screen</t>
         </is>
       </c>
       <c r="F88" s="41" t="inlineStr">
         <is>
-          <t>bh_a_fw</t>
+          <t>cab_fspur_fr_ac</t>
         </is>
       </c>
       <c r="G88" s="42" t="inlineStr">
         <is>
-          <t>BULKHEAD</t>
-        </is>
-      </c>
-      <c r="H88" s="41" t="n">
-        <v>46</v>
-      </c>
+          <t>cable screen (one end only)</t>
+        </is>
+      </c>
+      <c r="H88" s="41" t="inlineStr"/>
       <c r="I88" s="42" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
+          <t>FR wheel spd shield</t>
         </is>
       </c>
       <c r="J88" s="42" t="inlineStr"/>
-      <c r="K88" s="43" t="inlineStr"/>
-      <c r="L88" s="44" t="inlineStr"/>
-      <c r="M88" s="45" t="inlineStr"/>
+      <c r="K88" s="43" t="inlineStr">
+        <is>
+          <t>splice</t>
+        </is>
+      </c>
+      <c r="L88" s="44" t="inlineStr">
+        <is>
+          <t>sp_shield_a_wsf</t>
+        </is>
+      </c>
+      <c r="M88" s="45" t="inlineStr">
+        <is>
+          <t>splice sp_shield_a_wsf (SP-SHIELD-A-WSF)</t>
+        </is>
+      </c>
       <c r="N88" s="44" t="inlineStr"/>
-      <c r="O88" s="45" t="inlineStr"/>
+      <c r="O88" s="45" t="inlineStr">
+        <is>
+          <t>FR wheel spd shield</t>
+        </is>
+      </c>
       <c r="P88" s="45" t="inlineStr"/>
       <c r="Q88" s="46" t="inlineStr">
         <is>
-          <t>DRB102.46</t>
+          <t>ECU-A.A7</t>
         </is>
       </c>
       <c r="R88" s="47" t="inlineStr">
         <is>
-          <t>spare (DRB102 46)</t>
-        </is>
-      </c>
-      <c r="S88" s="48" t="inlineStr"/>
-      <c r="T88" s="48" t="inlineStr"/>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="S88" s="48" t="inlineStr">
+        <is>
+          <t>sp_shield_a_wsf</t>
+        </is>
+      </c>
+      <c r="T88" s="48" t="inlineStr">
+        <is>
+          <t>cab_fspur_fr_ac</t>
+        </is>
+      </c>
       <c r="U88" s="49" t="inlineStr"/>
-      <c r="V88" s="50" t="inlineStr"/>
+      <c r="V88" s="50" t="inlineStr">
+        <is>
+          <t>Shield</t>
+        </is>
+      </c>
       <c r="W88" s="50" t="inlineStr"/>
-      <c r="X88" s="50" t="inlineStr"/>
+      <c r="X88" s="50" t="inlineStr">
+        <is>
+          <t>White-Blue-Blue</t>
+        </is>
+      </c>
       <c r="Y88" s="50" t="inlineStr"/>
-      <c r="Z88" s="51" t="inlineStr"/>
+      <c r="Z88" s="51" t="inlineStr">
+        <is>
+          <t>dash branch (front WS inline)</t>
+        </is>
+      </c>
       <c r="AA88" s="52" t="inlineStr"/>
       <c r="AB88" s="53" t="inlineStr"/>
       <c r="AC88" s="54" t="inlineStr"/>
       <c r="AD88" s="54" t="inlineStr"/>
       <c r="AE88" s="54" t="inlineStr">
         <is>
-          <t>DRB102 46 = 'spare (size 16) - was the A/C coolant switch return, deleted (S35)'</t>
+          <t>splice sp_shield_a_wsf: node of the wire list (SoT)</t>
         </is>
       </c>
       <c r="AF88" s="54" t="inlineStr">
@@ -11405,7 +11489,11 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG88" s="54" t="inlineStr"/>
+      <c r="AG88" s="54" t="inlineStr">
+        <is>
+          <t>tied at the A end only; the far (B) end floats, dressed back at the ECU-B plug (no A-B shield bridge)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="23" t="inlineStr"/>
@@ -11432,7 +11520,7 @@
         </is>
       </c>
       <c r="H89" s="25" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="I89" s="26" t="inlineStr">
         <is>
@@ -11448,12 +11536,12 @@
       <c r="P89" s="29" t="inlineStr"/>
       <c r="Q89" s="30" t="inlineStr">
         <is>
-          <t>DRB102.52</t>
+          <t>DRB102.45</t>
         </is>
       </c>
       <c r="R89" s="31" t="inlineStr">
         <is>
-          <t>spare (DRB102 52)</t>
+          <t>spare (DRB102 45)</t>
         </is>
       </c>
       <c r="S89" s="32" t="inlineStr"/>
@@ -11470,7 +11558,7 @@
       <c r="AD89" s="38" t="inlineStr"/>
       <c r="AE89" s="38" t="inlineStr">
         <is>
-          <t>DRB102 52 = 'spare (size 16)'</t>
+          <t>DRB102 45 = 'spare (size 16) - was the A/C coolant switch signal, deleted (S35)'</t>
         </is>
       </c>
       <c r="AF89" s="38" t="inlineStr">
@@ -11505,7 +11593,7 @@
         </is>
       </c>
       <c r="H90" s="41" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="I90" s="42" t="inlineStr">
         <is>
@@ -11521,12 +11609,12 @@
       <c r="P90" s="45" t="inlineStr"/>
       <c r="Q90" s="46" t="inlineStr">
         <is>
-          <t>DRB102.53</t>
+          <t>DRB102.46</t>
         </is>
       </c>
       <c r="R90" s="47" t="inlineStr">
         <is>
-          <t>spare (DRB102 53)</t>
+          <t>spare (DRB102 46)</t>
         </is>
       </c>
       <c r="S90" s="48" t="inlineStr"/>
@@ -11543,7 +11631,7 @@
       <c r="AD90" s="54" t="inlineStr"/>
       <c r="AE90" s="54" t="inlineStr">
         <is>
-          <t>DRB102 53 = 'spare (size 16)'</t>
+          <t>DRB102 46 = 'spare (size 16) - was the A/C coolant switch return, deleted (S35)'</t>
         </is>
       </c>
       <c r="AF90" s="54" t="inlineStr">
@@ -11578,7 +11666,7 @@
         </is>
       </c>
       <c r="H91" s="25" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="I91" s="26" t="inlineStr">
         <is>
@@ -11594,12 +11682,12 @@
       <c r="P91" s="29" t="inlineStr"/>
       <c r="Q91" s="30" t="inlineStr">
         <is>
-          <t>DRB102.57</t>
+          <t>DRB102.52</t>
         </is>
       </c>
       <c r="R91" s="31" t="inlineStr">
         <is>
-          <t>spare (DRB102 57)</t>
+          <t>spare (DRB102 52)</t>
         </is>
       </c>
       <c r="S91" s="32" t="inlineStr"/>
@@ -11616,7 +11704,7 @@
       <c r="AD91" s="38" t="inlineStr"/>
       <c r="AE91" s="38" t="inlineStr">
         <is>
-          <t>DRB102 57 = 'spare (size 16)'</t>
+          <t>DRB102 52 = 'spare (size 16)'</t>
         </is>
       </c>
       <c r="AF91" s="38" t="inlineStr">
@@ -11651,7 +11739,7 @@
         </is>
       </c>
       <c r="H92" s="41" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I92" s="42" t="inlineStr">
         <is>
@@ -11667,12 +11755,12 @@
       <c r="P92" s="45" t="inlineStr"/>
       <c r="Q92" s="46" t="inlineStr">
         <is>
-          <t>DRB102.58</t>
+          <t>DRB102.53</t>
         </is>
       </c>
       <c r="R92" s="47" t="inlineStr">
         <is>
-          <t>spare (DRB102 58)</t>
+          <t>spare (DRB102 53)</t>
         </is>
       </c>
       <c r="S92" s="48" t="inlineStr"/>
@@ -11689,7 +11777,7 @@
       <c r="AD92" s="54" t="inlineStr"/>
       <c r="AE92" s="54" t="inlineStr">
         <is>
-          <t>DRB102 58 = 'spare (size 16)'</t>
+          <t>DRB102 53 = 'spare (size 16)'</t>
         </is>
       </c>
       <c r="AF92" s="54" t="inlineStr">
@@ -11724,7 +11812,7 @@
         </is>
       </c>
       <c r="H93" s="25" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I93" s="26" t="inlineStr">
         <is>
@@ -11740,12 +11828,12 @@
       <c r="P93" s="29" t="inlineStr"/>
       <c r="Q93" s="30" t="inlineStr">
         <is>
-          <t>DRB102.59</t>
+          <t>DRB102.57</t>
         </is>
       </c>
       <c r="R93" s="31" t="inlineStr">
         <is>
-          <t>spare (DRB102 59)</t>
+          <t>spare (DRB102 57)</t>
         </is>
       </c>
       <c r="S93" s="32" t="inlineStr"/>
@@ -11762,7 +11850,7 @@
       <c r="AD93" s="38" t="inlineStr"/>
       <c r="AE93" s="38" t="inlineStr">
         <is>
-          <t>DRB102 59 = 'spare (size 16)'</t>
+          <t>DRB102 57 = 'spare (size 16)'</t>
         </is>
       </c>
       <c r="AF93" s="38" t="inlineStr">
@@ -11797,7 +11885,7 @@
         </is>
       </c>
       <c r="H94" s="41" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I94" s="42" t="inlineStr">
         <is>
@@ -11813,12 +11901,12 @@
       <c r="P94" s="45" t="inlineStr"/>
       <c r="Q94" s="46" t="inlineStr">
         <is>
-          <t>DRB102.61</t>
+          <t>DRB102.58</t>
         </is>
       </c>
       <c r="R94" s="47" t="inlineStr">
         <is>
-          <t>spare (DRB102 61)</t>
+          <t>spare (DRB102 58)</t>
         </is>
       </c>
       <c r="S94" s="48" t="inlineStr"/>
@@ -11835,7 +11923,7 @@
       <c r="AD94" s="54" t="inlineStr"/>
       <c r="AE94" s="54" t="inlineStr">
         <is>
-          <t>DRB102 61 = 'spare (size 16)'</t>
+          <t>DRB102 58 = 'spare (size 16)'</t>
         </is>
       </c>
       <c r="AF94" s="54" t="inlineStr">
@@ -11861,16 +11949,16 @@
       </c>
       <c r="F95" s="25" t="inlineStr">
         <is>
-          <t>ix_ws_front_p</t>
+          <t>bh_a_fw</t>
         </is>
       </c>
       <c r="G95" s="26" t="inlineStr">
         <is>
-          <t>FRONT WS INLINE</t>
+          <t>BULKHEAD</t>
         </is>
       </c>
       <c r="H95" s="25" t="n">
-        <v>6</v>
+        <v>59</v>
       </c>
       <c r="I95" s="26" t="inlineStr">
         <is>
@@ -11886,12 +11974,12 @@
       <c r="P95" s="29" t="inlineStr"/>
       <c r="Q95" s="30" t="inlineStr">
         <is>
-          <t>ix_ws_front_p.6</t>
+          <t>DRB102.59</t>
         </is>
       </c>
       <c r="R95" s="31" t="inlineStr">
         <is>
-          <t>spare (ix_ws_front_p 6)</t>
+          <t>spare (DRB102 59)</t>
         </is>
       </c>
       <c r="S95" s="32" t="inlineStr"/>
@@ -11906,7 +11994,11 @@
       <c r="AB95" s="37" t="inlineStr"/>
       <c r="AC95" s="38" t="inlineStr"/>
       <c r="AD95" s="38" t="inlineStr"/>
-      <c r="AE95" s="38" t="inlineStr"/>
+      <c r="AE95" s="38" t="inlineStr">
+        <is>
+          <t>DRB102 59 = 'spare (size 16)'</t>
+        </is>
+      </c>
       <c r="AF95" s="38" t="inlineStr">
         <is>
           <t>OK</t>
@@ -11930,16 +12022,16 @@
       </c>
       <c r="F96" s="41" t="inlineStr">
         <is>
-          <t>bus_5v_bha_p</t>
+          <t>bh_a_fw</t>
         </is>
       </c>
       <c r="G96" s="42" t="inlineStr">
         <is>
-          <t>+5V BUS</t>
+          <t>BULKHEAD</t>
         </is>
       </c>
       <c r="H96" s="41" t="n">
-        <v>8</v>
+        <v>61</v>
       </c>
       <c r="I96" s="42" t="inlineStr">
         <is>
@@ -11955,12 +12047,12 @@
       <c r="P96" s="45" t="inlineStr"/>
       <c r="Q96" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A32</t>
+          <t>DRB102.61</t>
         </is>
       </c>
       <c r="R96" s="47" t="inlineStr">
         <is>
-          <t>+5V sensor (ECU-A A32)</t>
+          <t>spare (DRB102 61)</t>
         </is>
       </c>
       <c r="S96" s="48" t="inlineStr"/>
@@ -11975,7 +12067,11 @@
       <c r="AB96" s="53" t="inlineStr"/>
       <c r="AC96" s="54" t="inlineStr"/>
       <c r="AD96" s="54" t="inlineStr"/>
-      <c r="AE96" s="54" t="inlineStr"/>
+      <c r="AE96" s="54" t="inlineStr">
+        <is>
+          <t>DRB102 61 = 'spare (size 16)'</t>
+        </is>
+      </c>
       <c r="AF96" s="54" t="inlineStr">
         <is>
           <t>OK</t>
@@ -11999,16 +12095,16 @@
       </c>
       <c r="F97" s="25" t="inlineStr">
         <is>
-          <t>bus_gnd_bha_p</t>
+          <t>ix_ws_front_p</t>
         </is>
       </c>
       <c r="G97" s="26" t="inlineStr">
         <is>
-          <t>SENSOR GND BUS</t>
+          <t>FRONT WS INLINE</t>
         </is>
       </c>
       <c r="H97" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I97" s="26" t="inlineStr">
         <is>
@@ -12024,12 +12120,12 @@
       <c r="P97" s="29" t="inlineStr"/>
       <c r="Q97" s="30" t="inlineStr">
         <is>
-          <t>ECU-A.A24</t>
+          <t>ix_ws_front_p.6</t>
         </is>
       </c>
       <c r="R97" s="31" t="inlineStr">
         <is>
-          <t>Sensor GND (ECU-A A24)</t>
+          <t>spare (ix_ws_front_p 6)</t>
         </is>
       </c>
       <c r="S97" s="32" t="inlineStr"/>
@@ -12068,12 +12164,12 @@
       </c>
       <c r="F98" s="41" t="inlineStr">
         <is>
-          <t>bus_gnd_bha_p</t>
+          <t>bus_5v_bha_p</t>
         </is>
       </c>
       <c r="G98" s="42" t="inlineStr">
         <is>
-          <t>SENSOR GND BUS</t>
+          <t>+5V BUS</t>
         </is>
       </c>
       <c r="H98" s="41" t="n">
@@ -12093,12 +12189,12 @@
       <c r="P98" s="45" t="inlineStr"/>
       <c r="Q98" s="46" t="inlineStr">
         <is>
-          <t>ECU-A.A24</t>
+          <t>ECU-A.A32</t>
         </is>
       </c>
       <c r="R98" s="47" t="inlineStr">
         <is>
-          <t>Sensor GND (ECU-A A24)</t>
+          <t>+5V sensor (ECU-A A32)</t>
         </is>
       </c>
       <c r="S98" s="48" t="inlineStr"/>
@@ -12121,8 +12217,146 @@
       </c>
       <c r="AG98" s="54" t="inlineStr"/>
     </row>
+    <row r="99">
+      <c r="A99" s="23" t="inlineStr"/>
+      <c r="B99" s="23" t="inlineStr"/>
+      <c r="C99" s="23" t="inlineStr">
+        <is>
+          <t>A-cabin</t>
+        </is>
+      </c>
+      <c r="D99" s="23" t="inlineStr"/>
+      <c r="E99" s="24" t="inlineStr">
+        <is>
+          <t>connector</t>
+        </is>
+      </c>
+      <c r="F99" s="25" t="inlineStr">
+        <is>
+          <t>bus_gnd_bha_p</t>
+        </is>
+      </c>
+      <c r="G99" s="26" t="inlineStr">
+        <is>
+          <t>SENSOR GND BUS</t>
+        </is>
+      </c>
+      <c r="H99" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="I99" s="26" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="J99" s="26" t="inlineStr"/>
+      <c r="K99" s="27" t="inlineStr"/>
+      <c r="L99" s="28" t="inlineStr"/>
+      <c r="M99" s="29" t="inlineStr"/>
+      <c r="N99" s="28" t="inlineStr"/>
+      <c r="O99" s="29" t="inlineStr"/>
+      <c r="P99" s="29" t="inlineStr"/>
+      <c r="Q99" s="30" t="inlineStr">
+        <is>
+          <t>ECU-A.A24</t>
+        </is>
+      </c>
+      <c r="R99" s="31" t="inlineStr">
+        <is>
+          <t>Sensor GND (ECU-A A24)</t>
+        </is>
+      </c>
+      <c r="S99" s="32" t="inlineStr"/>
+      <c r="T99" s="32" t="inlineStr"/>
+      <c r="U99" s="33" t="inlineStr"/>
+      <c r="V99" s="34" t="inlineStr"/>
+      <c r="W99" s="34" t="inlineStr"/>
+      <c r="X99" s="34" t="inlineStr"/>
+      <c r="Y99" s="34" t="inlineStr"/>
+      <c r="Z99" s="35" t="inlineStr"/>
+      <c r="AA99" s="36" t="inlineStr"/>
+      <c r="AB99" s="37" t="inlineStr"/>
+      <c r="AC99" s="38" t="inlineStr"/>
+      <c r="AD99" s="38" t="inlineStr"/>
+      <c r="AE99" s="38" t="inlineStr"/>
+      <c r="AF99" s="38" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AG99" s="38" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="39" t="inlineStr"/>
+      <c r="B100" s="39" t="inlineStr"/>
+      <c r="C100" s="39" t="inlineStr">
+        <is>
+          <t>A-cabin</t>
+        </is>
+      </c>
+      <c r="D100" s="39" t="inlineStr"/>
+      <c r="E100" s="40" t="inlineStr">
+        <is>
+          <t>connector</t>
+        </is>
+      </c>
+      <c r="F100" s="41" t="inlineStr">
+        <is>
+          <t>bus_gnd_bha_p</t>
+        </is>
+      </c>
+      <c r="G100" s="42" t="inlineStr">
+        <is>
+          <t>SENSOR GND BUS</t>
+        </is>
+      </c>
+      <c r="H100" s="41" t="n">
+        <v>8</v>
+      </c>
+      <c r="I100" s="42" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="J100" s="42" t="inlineStr"/>
+      <c r="K100" s="43" t="inlineStr"/>
+      <c r="L100" s="44" t="inlineStr"/>
+      <c r="M100" s="45" t="inlineStr"/>
+      <c r="N100" s="44" t="inlineStr"/>
+      <c r="O100" s="45" t="inlineStr"/>
+      <c r="P100" s="45" t="inlineStr"/>
+      <c r="Q100" s="46" t="inlineStr">
+        <is>
+          <t>ECU-A.A24</t>
+        </is>
+      </c>
+      <c r="R100" s="47" t="inlineStr">
+        <is>
+          <t>Sensor GND (ECU-A A24)</t>
+        </is>
+      </c>
+      <c r="S100" s="48" t="inlineStr"/>
+      <c r="T100" s="48" t="inlineStr"/>
+      <c r="U100" s="49" t="inlineStr"/>
+      <c r="V100" s="50" t="inlineStr"/>
+      <c r="W100" s="50" t="inlineStr"/>
+      <c r="X100" s="50" t="inlineStr"/>
+      <c r="Y100" s="50" t="inlineStr"/>
+      <c r="Z100" s="51" t="inlineStr"/>
+      <c r="AA100" s="52" t="inlineStr"/>
+      <c r="AB100" s="53" t="inlineStr"/>
+      <c r="AC100" s="54" t="inlineStr"/>
+      <c r="AD100" s="54" t="inlineStr"/>
+      <c r="AE100" s="54" t="inlineStr"/>
+      <c r="AF100" s="54" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AG100" s="54" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AG98"/>
+  <autoFilter ref="A2:AG100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -12134,16 +12368,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
@@ -12414,18 +12648,18 @@
         </is>
       </c>
       <c r="F5" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="32" t="inlineStr">
+        <is>
+          <t>20+20+20+20+20+20+20+20</t>
+        </is>
+      </c>
+      <c r="H5" s="32" t="n">
+        <v>8176</v>
+      </c>
+      <c r="I5" s="32" t="n">
         <v>10</v>
-      </c>
-      <c r="G5" s="32" t="inlineStr">
-        <is>
-          <t>20+20+20+20+20+20 + shield</t>
-        </is>
-      </c>
-      <c r="H5" s="32" t="n">
-        <v>6132</v>
-      </c>
-      <c r="I5" s="32" t="n">
-        <v>12</v>
       </c>
       <c r="J5" s="56" t="inlineStr">
         <is>
@@ -12835,8 +13069,120 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>sp_shield_a_aps</t>
+        </is>
+      </c>
+      <c r="B13" s="55" t="inlineStr">
+        <is>
+          <t>At the pedal branch - SP-SHIELD-A-APS: pedal drains</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>A-cabin</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>ECU-A.A7</t>
+        </is>
+      </c>
+      <c r="E13" s="31" t="inlineStr">
+        <is>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="F13" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" s="32" t="inlineStr">
+        <is>
+          <t>20 + shield</t>
+        </is>
+      </c>
+      <c r="H13" s="32" t="n">
+        <v>1022</v>
+      </c>
+      <c r="I13" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="J13" s="56" t="inlineStr">
+        <is>
+          <t>SPLICE, SOLDERED, ADHESIVE HEATSHRINK OVER</t>
+        </is>
+      </c>
+      <c r="K13" s="36" t="inlineStr">
+        <is>
+          <t>At the pedal branch (layout node bp_960)</t>
+        </is>
+      </c>
+      <c r="L13" s="38" t="inlineStr">
+        <is>
+          <t>node of the wire list (SoT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="39" t="inlineStr">
+        <is>
+          <t>sp_shield_a_wsf</t>
+        </is>
+      </c>
+      <c r="B14" s="57" t="inlineStr">
+        <is>
+          <t>At the front WS inline - SP-SHIELD-A-WSF: front wheel-speed drains</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="inlineStr">
+        <is>
+          <t>A-cabin</t>
+        </is>
+      </c>
+      <c r="D14" s="46" t="inlineStr">
+        <is>
+          <t>ECU-A.A7</t>
+        </is>
+      </c>
+      <c r="E14" s="47" t="inlineStr">
+        <is>
+          <t>Screen A (ECU A7, SHIELD_A)</t>
+        </is>
+      </c>
+      <c r="F14" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="48" t="inlineStr">
+        <is>
+          <t>20 + shield</t>
+        </is>
+      </c>
+      <c r="H14" s="48" t="n">
+        <v>1022</v>
+      </c>
+      <c r="I14" s="48" t="n">
+        <v>20</v>
+      </c>
+      <c r="J14" s="58" t="inlineStr">
+        <is>
+          <t>SPLICE, SOLDERED, ADHESIVE HEATSHRINK OVER</t>
+        </is>
+      </c>
+      <c r="K14" s="52" t="inlineStr">
+        <is>
+          <t>At the front WS inline (layout node bp_1020)</t>
+        </is>
+      </c>
+      <c r="L14" s="54" t="inlineStr">
+        <is>
+          <t>node of the wire list (SoT)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L12"/>
+  <autoFilter ref="A2:L14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Wire colours: 7 solid colours by function (R209, Dan N52)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-wirelist.xlsx
+++ b/docs/harness/wirelist/A-cabin-wirelist.xlsx
@@ -1201,7 +1201,7 @@
       </c>
       <c r="V3" s="34" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W3" s="34" t="inlineStr"/>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="V4" s="50" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W4" s="50" t="inlineStr"/>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="V5" s="34" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W5" s="34" t="inlineStr"/>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="V6" s="50" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W6" s="50" t="inlineStr"/>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="V7" s="34" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W7" s="34" t="inlineStr"/>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="V8" s="50" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W8" s="50" t="inlineStr"/>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="V9" s="34" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W9" s="34" t="inlineStr"/>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="V10" s="50" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W10" s="50" t="inlineStr"/>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="V11" s="34" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W11" s="34" t="inlineStr"/>
@@ -2254,7 +2254,7 @@
       </c>
       <c r="V12" s="50" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W12" s="50" t="inlineStr"/>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="V13" s="34" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W13" s="34" t="inlineStr"/>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="V17" s="34" t="inlineStr">
         <is>
-          <t>Gray</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W17" s="34" t="inlineStr"/>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="V18" s="50" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W18" s="50" t="inlineStr"/>
@@ -3073,7 +3073,7 @@
       </c>
       <c r="V19" s="34" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W19" s="34" t="inlineStr"/>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="V20" s="50" t="inlineStr">
         <is>
-          <t>Gray</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W20" s="50" t="inlineStr"/>
@@ -3309,7 +3309,7 @@
       </c>
       <c r="V21" s="34" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W21" s="34" t="inlineStr"/>
@@ -3424,7 +3424,7 @@
       </c>
       <c r="V22" s="50" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W22" s="50" t="inlineStr"/>
@@ -3539,7 +3539,7 @@
       </c>
       <c r="V23" s="34" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W23" s="34" t="inlineStr"/>
@@ -3657,11 +3657,7 @@
           <t>Orange</t>
         </is>
       </c>
-      <c r="W24" s="50" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+      <c r="W24" s="50" t="inlineStr"/>
       <c r="X24" s="50" t="inlineStr">
         <is>
           <t>Yellow-Yellow</t>
@@ -3778,11 +3774,7 @@
           <t>Orange</t>
         </is>
       </c>
-      <c r="W25" s="34" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+      <c r="W25" s="34" t="inlineStr"/>
       <c r="X25" s="34" t="inlineStr">
         <is>
           <t>Yellow-Blue-Yellow</t>
@@ -3897,11 +3889,7 @@
           <t>Orange</t>
         </is>
       </c>
-      <c r="W26" s="50" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+      <c r="W26" s="50" t="inlineStr"/>
       <c r="X26" s="50" t="inlineStr">
         <is>
           <t>Yellow-Blue-Yellow</t>
@@ -5302,14 +5290,10 @@
       </c>
       <c r="V38" s="50" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W38" s="50" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W38" s="50" t="inlineStr"/>
       <c r="X38" s="50" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -5421,14 +5405,10 @@
       </c>
       <c r="V39" s="34" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W39" s="34" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W39" s="34" t="inlineStr"/>
       <c r="X39" s="34" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -5538,14 +5518,10 @@
       </c>
       <c r="V40" s="50" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W40" s="50" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W40" s="50" t="inlineStr"/>
       <c r="X40" s="50" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -5657,14 +5633,10 @@
       </c>
       <c r="V41" s="34" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W41" s="34" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W41" s="34" t="inlineStr"/>
       <c r="X41" s="34" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -5776,14 +5748,10 @@
       </c>
       <c r="V42" s="50" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W42" s="50" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W42" s="50" t="inlineStr"/>
       <c r="X42" s="50" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -5895,14 +5863,10 @@
       </c>
       <c r="V43" s="34" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W43" s="34" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W43" s="34" t="inlineStr"/>
       <c r="X43" s="34" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -6014,14 +5978,10 @@
       </c>
       <c r="V44" s="50" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W44" s="50" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W44" s="50" t="inlineStr"/>
       <c r="X44" s="50" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -6373,7 +6333,7 @@
       </c>
       <c r="V47" s="34" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="W47" s="34" t="inlineStr"/>
@@ -7975,11 +7935,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W60" s="50" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W60" s="50" t="inlineStr"/>
       <c r="X60" s="50" t="inlineStr">
         <is>
           <t>White-Yellow-Blue</t>
@@ -8096,11 +8052,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W61" s="34" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W61" s="34" t="inlineStr"/>
       <c r="X61" s="34" t="inlineStr">
         <is>
           <t>White-Yellow-Blue</t>
@@ -8213,11 +8165,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W62" s="50" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W62" s="50" t="inlineStr"/>
       <c r="X62" s="50" t="inlineStr">
         <is>
           <t>White-Yellow-Blue</t>
@@ -8332,11 +8280,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W63" s="34" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W63" s="34" t="inlineStr"/>
       <c r="X63" s="34" t="inlineStr">
         <is>
           <t>White-Blue-White</t>
@@ -8455,11 +8399,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W64" s="50" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W64" s="50" t="inlineStr"/>
       <c r="X64" s="50" t="inlineStr">
         <is>
           <t>Yellow-Yellow</t>
@@ -8574,11 +8514,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W65" s="34" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W65" s="34" t="inlineStr"/>
       <c r="X65" s="34" t="inlineStr">
         <is>
           <t>White</t>
@@ -8693,11 +8629,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W66" s="50" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W66" s="50" t="inlineStr"/>
       <c r="X66" s="50" t="inlineStr">
         <is>
           <t>White-Blue</t>
@@ -8812,11 +8744,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W67" s="34" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W67" s="34" t="inlineStr"/>
       <c r="X67" s="34" t="inlineStr">
         <is>
           <t>Yellow</t>
@@ -9321,7 +9249,7 @@
       </c>
       <c r="V71" s="34" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W71" s="34" t="inlineStr"/>
@@ -9446,7 +9374,7 @@
       </c>
       <c r="V72" s="50" t="inlineStr">
         <is>
-          <t>Gray</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W72" s="50" t="inlineStr"/>
@@ -9590,11 +9518,7 @@
           <t>Yellow</t>
         </is>
       </c>
-      <c r="W73" s="34" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
+      <c r="W73" s="34" t="inlineStr"/>
       <c r="X73" s="34" t="inlineStr">
         <is>
           <t>Yellow-Blue</t>
@@ -9733,11 +9657,7 @@
           <t>Yellow</t>
         </is>
       </c>
-      <c r="W74" s="50" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
+      <c r="W74" s="50" t="inlineStr"/>
       <c r="X74" s="50" t="inlineStr">
         <is>
           <t>Yellow-Blue</t>
@@ -9873,14 +9793,10 @@
       </c>
       <c r="V75" s="34" t="inlineStr">
         <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="W75" s="34" t="inlineStr">
-        <is>
           <t>Red</t>
         </is>
       </c>
+      <c r="W75" s="34" t="inlineStr"/>
       <c r="X75" s="34" t="inlineStr">
         <is>
           <t>Yellow-Blue</t>

</xml_diff>

<commit_message>
Wire colours: 7 solid colours by function (R209, Dan N52) (#354)
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-wirelist.xlsx
+++ b/docs/harness/wirelist/A-cabin-wirelist.xlsx
@@ -1201,7 +1201,7 @@
       </c>
       <c r="V3" s="34" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W3" s="34" t="inlineStr"/>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="V4" s="50" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W4" s="50" t="inlineStr"/>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="V5" s="34" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W5" s="34" t="inlineStr"/>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="V6" s="50" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W6" s="50" t="inlineStr"/>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="V7" s="34" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W7" s="34" t="inlineStr"/>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="V8" s="50" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W8" s="50" t="inlineStr"/>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="V9" s="34" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W9" s="34" t="inlineStr"/>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="V10" s="50" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W10" s="50" t="inlineStr"/>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="V11" s="34" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W11" s="34" t="inlineStr"/>
@@ -2254,7 +2254,7 @@
       </c>
       <c r="V12" s="50" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W12" s="50" t="inlineStr"/>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="V13" s="34" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W13" s="34" t="inlineStr"/>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="V17" s="34" t="inlineStr">
         <is>
-          <t>Gray</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W17" s="34" t="inlineStr"/>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="V18" s="50" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W18" s="50" t="inlineStr"/>
@@ -3073,7 +3073,7 @@
       </c>
       <c r="V19" s="34" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W19" s="34" t="inlineStr"/>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="V20" s="50" t="inlineStr">
         <is>
-          <t>Gray</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W20" s="50" t="inlineStr"/>
@@ -3309,7 +3309,7 @@
       </c>
       <c r="V21" s="34" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W21" s="34" t="inlineStr"/>
@@ -3424,7 +3424,7 @@
       </c>
       <c r="V22" s="50" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W22" s="50" t="inlineStr"/>
@@ -3539,7 +3539,7 @@
       </c>
       <c r="V23" s="34" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W23" s="34" t="inlineStr"/>
@@ -3657,11 +3657,7 @@
           <t>Orange</t>
         </is>
       </c>
-      <c r="W24" s="50" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+      <c r="W24" s="50" t="inlineStr"/>
       <c r="X24" s="50" t="inlineStr">
         <is>
           <t>Yellow-Yellow</t>
@@ -3778,11 +3774,7 @@
           <t>Orange</t>
         </is>
       </c>
-      <c r="W25" s="34" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+      <c r="W25" s="34" t="inlineStr"/>
       <c r="X25" s="34" t="inlineStr">
         <is>
           <t>Yellow-Blue-Yellow</t>
@@ -3897,11 +3889,7 @@
           <t>Orange</t>
         </is>
       </c>
-      <c r="W26" s="50" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+      <c r="W26" s="50" t="inlineStr"/>
       <c r="X26" s="50" t="inlineStr">
         <is>
           <t>Yellow-Blue-Yellow</t>
@@ -5302,14 +5290,10 @@
       </c>
       <c r="V38" s="50" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W38" s="50" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W38" s="50" t="inlineStr"/>
       <c r="X38" s="50" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -5421,14 +5405,10 @@
       </c>
       <c r="V39" s="34" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W39" s="34" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W39" s="34" t="inlineStr"/>
       <c r="X39" s="34" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -5538,14 +5518,10 @@
       </c>
       <c r="V40" s="50" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W40" s="50" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W40" s="50" t="inlineStr"/>
       <c r="X40" s="50" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -5657,14 +5633,10 @@
       </c>
       <c r="V41" s="34" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W41" s="34" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W41" s="34" t="inlineStr"/>
       <c r="X41" s="34" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -5776,14 +5748,10 @@
       </c>
       <c r="V42" s="50" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W42" s="50" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W42" s="50" t="inlineStr"/>
       <c r="X42" s="50" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -5895,14 +5863,10 @@
       </c>
       <c r="V43" s="34" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W43" s="34" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W43" s="34" t="inlineStr"/>
       <c r="X43" s="34" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -6014,14 +5978,10 @@
       </c>
       <c r="V44" s="50" t="inlineStr">
         <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="W44" s="50" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="W44" s="50" t="inlineStr"/>
       <c r="X44" s="50" t="inlineStr">
         <is>
           <t>Yellow-Yellow-Blue</t>
@@ -6373,7 +6333,7 @@
       </c>
       <c r="V47" s="34" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="W47" s="34" t="inlineStr"/>
@@ -7975,11 +7935,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W60" s="50" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W60" s="50" t="inlineStr"/>
       <c r="X60" s="50" t="inlineStr">
         <is>
           <t>White-Yellow-Blue</t>
@@ -8096,11 +8052,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W61" s="34" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W61" s="34" t="inlineStr"/>
       <c r="X61" s="34" t="inlineStr">
         <is>
           <t>White-Yellow-Blue</t>
@@ -8213,11 +8165,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W62" s="50" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W62" s="50" t="inlineStr"/>
       <c r="X62" s="50" t="inlineStr">
         <is>
           <t>White-Yellow-Blue</t>
@@ -8332,11 +8280,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W63" s="34" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W63" s="34" t="inlineStr"/>
       <c r="X63" s="34" t="inlineStr">
         <is>
           <t>White-Blue-White</t>
@@ -8455,11 +8399,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W64" s="50" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W64" s="50" t="inlineStr"/>
       <c r="X64" s="50" t="inlineStr">
         <is>
           <t>Yellow-Yellow</t>
@@ -8574,11 +8514,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W65" s="34" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W65" s="34" t="inlineStr"/>
       <c r="X65" s="34" t="inlineStr">
         <is>
           <t>White</t>
@@ -8693,11 +8629,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W66" s="50" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W66" s="50" t="inlineStr"/>
       <c r="X66" s="50" t="inlineStr">
         <is>
           <t>White-Blue</t>
@@ -8812,11 +8744,7 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="W67" s="34" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
+      <c r="W67" s="34" t="inlineStr"/>
       <c r="X67" s="34" t="inlineStr">
         <is>
           <t>Yellow</t>
@@ -9321,7 +9249,7 @@
       </c>
       <c r="V71" s="34" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W71" s="34" t="inlineStr"/>
@@ -9446,7 +9374,7 @@
       </c>
       <c r="V72" s="50" t="inlineStr">
         <is>
-          <t>Gray</t>
+          <t>White</t>
         </is>
       </c>
       <c r="W72" s="50" t="inlineStr"/>
@@ -9590,11 +9518,7 @@
           <t>Yellow</t>
         </is>
       </c>
-      <c r="W73" s="34" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
+      <c r="W73" s="34" t="inlineStr"/>
       <c r="X73" s="34" t="inlineStr">
         <is>
           <t>Yellow-Blue</t>
@@ -9733,11 +9657,7 @@
           <t>Yellow</t>
         </is>
       </c>
-      <c r="W74" s="50" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
+      <c r="W74" s="50" t="inlineStr"/>
       <c r="X74" s="50" t="inlineStr">
         <is>
           <t>Yellow-Blue</t>
@@ -9873,14 +9793,10 @@
       </c>
       <c r="V75" s="34" t="inlineStr">
         <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="W75" s="34" t="inlineStr">
-        <is>
           <t>Red</t>
         </is>
       </c>
+      <c r="W75" s="34" t="inlineStr"/>
       <c r="X75" s="34" t="inlineStr">
         <is>
           <t>Yellow-Blue</t>

</xml_diff>